<commit_message>
Add missing core-radial cell size to Mesh Levels sheet
Circumferential and axial divisions already had a physical cell-size
row; core-radial divisions didn't, because it needed an extra
assumption (O-grid centre-block size) that circumferential/axial
don't. Adds an editable core-block fraction input and the resulting
wedge-span/cell-size formulas, flagged as a planning estimate since
ANSYS's MultiZone method decides the actual core-block geometry itself.
</commit_message>
<xml_diff>
--- a/thesis/mesh-validation/Mesh_and_Validation_Workbook.xlsx
+++ b/thesis/mesh-validation/Mesh_and_Validation_Workbook.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="192">
   <si>
     <t xml:space="preserve">PTSC-HTSP Thesis — Meshing &amp; Validation Workbook</t>
   </si>
@@ -362,6 +362,27 @@
   </si>
   <si>
     <t xml:space="preserve">Approx. axial cell length (mm) = L / N_axial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Core-radial cell size -- needs one assumption circumferential/axial didn't: how big is the O-grid centre square?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Core block half-width, as a fraction of tube radius (editable -- common O-grid practice is 0.35-0.45, not a strict rule)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tube radius (mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Core block half-width (mm) = fraction × radius</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Radial (wedge) span (mm) = radius - core half-width</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approx. core-radial cell size (mm) = wedge span / N_core</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This is a planning estimate, not a guarantee of what ANSYS's automatic MultiZone O-grid will build -- MultiZone decides the actual core-block position and the size transition itself. Its purpose here is bookkeeping: it feeds the cell-count and representative-size formulas below so your GCI refinement ratio stays consistent across levels. If ANSYS reports poor skewness/orthogonal quality in the wedge blocks after meshing, that's the real signal to adjust the core fraction or Core radial divisions -- not this number on its own.</t>
   </si>
   <si>
     <t xml:space="preserve">Inflation (boundary layer) settings — CONSTANT across all three levels, do NOT change these between runs</t>
@@ -814,7 +835,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -927,6 +948,14 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="169" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -976,10 +1005,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="175" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2151,7 +2176,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:E23"/>
+  <dimension ref="B2:E31"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -2277,112 +2302,182 @@
         <v>17.7777777777778</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="22" t="s">
+    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="28" t="s">
         <v>110</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="7" t="s">
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+    </row>
+    <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C16" s="29" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="C17" s="21" t="n">
+        <f aca="false">Inputs!$C$6*1000/2</f>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C18" s="21" t="n">
+        <f aca="false">C16*C17</f>
+        <v>13.2</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="C19" s="21" t="n">
+        <f aca="false">C17-C18</f>
+        <v>19.8</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="C20" s="18" t="n">
+        <f aca="false">$C$19/C9</f>
+        <v>1.98</v>
+      </c>
+      <c r="D20" s="18" t="n">
+        <f aca="false">$C$19/D9</f>
+        <v>1.32</v>
+      </c>
+      <c r="E20" s="18" t="n">
+        <f aca="false">$C$19/E9</f>
+        <v>0.860869565217391</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="22" t="s">
+        <v>117</v>
+      </c>
+      <c r="C23" s="22"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="22"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="C16" s="28" t="n">
+      <c r="C24" s="30" t="n">
         <f aca="false">'YPlus Inflation'!$C$20</f>
         <v>0.0139171040876707</v>
       </c>
-      <c r="D16" s="28" t="n">
+      <c r="D24" s="30" t="n">
         <f aca="false">'YPlus Inflation'!$C$20</f>
         <v>0.0139171040876707</v>
       </c>
-      <c r="E16" s="28" t="n">
+      <c r="E24" s="30" t="n">
         <f aca="false">'YPlus Inflation'!$C$20</f>
         <v>0.0139171040876707</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="C17" s="29" t="n">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="C25" s="31" t="n">
         <f aca="false">'YPlus Inflation'!$C$22</f>
         <v>1.2</v>
       </c>
-      <c r="D17" s="29" t="n">
+      <c r="D25" s="31" t="n">
         <f aca="false">'YPlus Inflation'!$C$22</f>
         <v>1.2</v>
       </c>
-      <c r="E17" s="29" t="n">
+      <c r="E25" s="31" t="n">
         <f aca="false">'YPlus Inflation'!$C$22</f>
         <v>1.2</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="7" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="C18" s="30" t="n">
+      <c r="C26" s="32" t="n">
         <f aca="false">'YPlus Inflation'!$C$23</f>
         <v>20</v>
       </c>
-      <c r="D18" s="30" t="n">
+      <c r="D26" s="32" t="n">
         <f aca="false">'YPlus Inflation'!$C$23</f>
         <v>20</v>
       </c>
-      <c r="E18" s="30" t="n">
+      <c r="E26" s="32" t="n">
         <f aca="false">'YPlus Inflation'!$C$23</f>
         <v>20</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="C20" s="31" t="n">
-        <f aca="false">C8*C10*(C9+C18)</f>
+    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B28" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C28" s="33" t="n">
+        <f aca="false">C8*C10*(C9+C26)</f>
         <v>45000</v>
       </c>
-      <c r="D20" s="31" t="n">
-        <f aca="false">D8*D10*(D9+D18)</f>
+      <c r="D28" s="33" t="n">
+        <f aca="false">D8*D10*(D9+D26)</f>
         <v>120750</v>
       </c>
-      <c r="E20" s="31" t="n">
-        <f aca="false">E8*E10*(E9+E18)</f>
+      <c r="E28" s="33" t="n">
+        <f aca="false">E8*E10*(E9+E26)</f>
         <v>338625</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="C21" s="18" t="n">
-        <f aca="false">(PI()/4*(Inputs!$C$6*1000)^2*(Inputs!$C$7*1000)/C20)^(1/3)</f>
+    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B29" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C29" s="18" t="n">
+        <f aca="false">(PI()/4*(Inputs!$C$6*1000)^2*(Inputs!$C$7*1000)/C28)^(1/3)</f>
         <v>6.72473347933769</v>
       </c>
-      <c r="D21" s="18" t="n">
-        <f aca="false">(PI()/4*(Inputs!$C$6*1000)^2*(Inputs!$C$7*1000)/D20)^(1/3)</f>
+      <c r="D29" s="18" t="n">
+        <f aca="false">(PI()/4*(Inputs!$C$6*1000)^2*(Inputs!$C$7*1000)/D28)^(1/3)</f>
         <v>4.8393110188735</v>
       </c>
-      <c r="E21" s="18" t="n">
-        <f aca="false">(PI()/4*(Inputs!$C$6*1000)^2*(Inputs!$C$7*1000)/E20)^(1/3)</f>
+      <c r="E29" s="18" t="n">
+        <f aca="false">(PI()/4*(Inputs!$C$6*1000)^2*(Inputs!$C$7*1000)/E28)^(1/3)</f>
         <v>3.43167571948627</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12"/>
+    <row r="31" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B31" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="C31" s="12"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="12"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B21:E21"/>
     <mergeCell ref="B23:E23"/>
+    <mergeCell ref="B31:E31"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2414,12 +2509,12 @@
   <sheetData>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="12" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -2434,29 +2529,29 @@
         <v>79</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="32" t="n">
+      <c r="B6" s="34" t="n">
         <v>5000</v>
       </c>
       <c r="C6" s="18" t="n">
@@ -2471,19 +2566,19 @@
         <f aca="false">0.023*B6^0.8*'Fluid Properties'!$C$24^0.4</f>
         <v>50.2911752463619</v>
       </c>
-      <c r="F6" s="33"/>
-      <c r="G6" s="34" t="str">
+      <c r="F6" s="35"/>
+      <c r="G6" s="36" t="str">
         <f aca="false">IF(F6="","",ABS(F6-D6)/D6)</f>
         <v/>
       </c>
-      <c r="H6" s="33"/>
-      <c r="I6" s="34" t="str">
+      <c r="H6" s="35"/>
+      <c r="I6" s="36" t="str">
         <f aca="false">IF(H6="","",ABS(H6-C6)/C6)</f>
         <v/>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="32" t="n">
+      <c r="B7" s="34" t="n">
         <v>7500</v>
       </c>
       <c r="C7" s="18" t="n">
@@ -2498,19 +2593,19 @@
         <f aca="false">0.023*B7^0.8*'Fluid Properties'!$C$24^0.4</f>
         <v>69.5608358585765</v>
       </c>
-      <c r="F7" s="33"/>
-      <c r="G7" s="34" t="str">
+      <c r="F7" s="35"/>
+      <c r="G7" s="36" t="str">
         <f aca="false">IF(F7="","",ABS(F7-D7)/D7)</f>
         <v/>
       </c>
-      <c r="H7" s="33"/>
-      <c r="I7" s="34" t="str">
+      <c r="H7" s="35"/>
+      <c r="I7" s="36" t="str">
         <f aca="false">IF(H7="","",ABS(H7-C7)/C7)</f>
         <v/>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="32" t="n">
+      <c r="B8" s="34" t="n">
         <v>10000</v>
       </c>
       <c r="C8" s="18" t="n">
@@ -2525,19 +2620,19 @@
         <f aca="false">0.023*B8^0.8*'Fluid Properties'!$C$24^0.4</f>
         <v>87.5620218790889</v>
       </c>
-      <c r="F8" s="33"/>
-      <c r="G8" s="34" t="str">
+      <c r="F8" s="35"/>
+      <c r="G8" s="36" t="str">
         <f aca="false">IF(F8="","",ABS(F8-D8)/D8)</f>
         <v/>
       </c>
-      <c r="H8" s="33"/>
-      <c r="I8" s="34" t="str">
+      <c r="H8" s="35"/>
+      <c r="I8" s="36" t="str">
         <f aca="false">IF(H8="","",ABS(H8-C8)/C8)</f>
         <v/>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="32" t="n">
+      <c r="B9" s="34" t="n">
         <v>20000</v>
       </c>
       <c r="C9" s="18" t="n">
@@ -2552,19 +2647,19 @@
         <f aca="false">0.023*B9^0.8*'Fluid Properties'!$C$24^0.4</f>
         <v>152.454334940377</v>
       </c>
-      <c r="F9" s="33"/>
-      <c r="G9" s="34" t="str">
+      <c r="F9" s="35"/>
+      <c r="G9" s="36" t="str">
         <f aca="false">IF(F9="","",ABS(F9-D9)/D9)</f>
         <v/>
       </c>
-      <c r="H9" s="33"/>
-      <c r="I9" s="34" t="str">
+      <c r="H9" s="35"/>
+      <c r="I9" s="36" t="str">
         <f aca="false">IF(H9="","",ABS(H9-C9)/C9)</f>
         <v/>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="32" t="n">
+      <c r="B10" s="34" t="n">
         <v>30000</v>
       </c>
       <c r="C10" s="18" t="n">
@@ -2579,19 +2674,19 @@
         <f aca="false">0.023*B10^0.8*'Fluid Properties'!$C$24^0.4</f>
         <v>210.86902258231</v>
       </c>
-      <c r="F10" s="33"/>
-      <c r="G10" s="34" t="str">
+      <c r="F10" s="35"/>
+      <c r="G10" s="36" t="str">
         <f aca="false">IF(F10="","",ABS(F10-D10)/D10)</f>
         <v/>
       </c>
-      <c r="H10" s="33"/>
-      <c r="I10" s="34" t="str">
+      <c r="H10" s="35"/>
+      <c r="I10" s="36" t="str">
         <f aca="false">IF(H10="","",ABS(H10-C10)/C10)</f>
         <v/>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="32" t="n">
+      <c r="B11" s="34" t="n">
         <v>50000</v>
       </c>
       <c r="C11" s="18" t="n">
@@ -2606,19 +2701,19 @@
         <f aca="false">0.023*B11^0.8*'Fluid Properties'!$C$24^0.4</f>
         <v>317.315863842325</v>
       </c>
-      <c r="F11" s="33"/>
-      <c r="G11" s="34" t="str">
+      <c r="F11" s="35"/>
+      <c r="G11" s="36" t="str">
         <f aca="false">IF(F11="","",ABS(F11-D11)/D11)</f>
         <v/>
       </c>
-      <c r="H11" s="33"/>
-      <c r="I11" s="34" t="str">
+      <c r="H11" s="35"/>
+      <c r="I11" s="36" t="str">
         <f aca="false">IF(H11="","",ABS(H11-C11)/C11)</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="32" t="n">
+      <c r="B12" s="34" t="n">
         <v>70000</v>
       </c>
       <c r="C12" s="18" t="n">
@@ -2633,19 +2728,19 @@
         <f aca="false">0.023*B12^0.8*'Fluid Properties'!$C$24^0.4</f>
         <v>415.330871372776</v>
       </c>
-      <c r="F12" s="33"/>
-      <c r="G12" s="34" t="str">
+      <c r="F12" s="35"/>
+      <c r="G12" s="36" t="str">
         <f aca="false">IF(F12="","",ABS(F12-D12)/D12)</f>
         <v/>
       </c>
-      <c r="H12" s="33"/>
-      <c r="I12" s="34" t="str">
+      <c r="H12" s="35"/>
+      <c r="I12" s="36" t="str">
         <f aca="false">IF(H12="","",ABS(H12-C12)/C12)</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="32" t="n">
+      <c r="B13" s="34" t="n">
         <v>100000</v>
       </c>
       <c r="C13" s="18" t="n">
@@ -2660,20 +2755,20 @@
         <f aca="false">0.023*B13^0.8*'Fluid Properties'!$C$24^0.4</f>
         <v>552.479008021465</v>
       </c>
-      <c r="F13" s="33"/>
-      <c r="G13" s="34" t="str">
+      <c r="F13" s="35"/>
+      <c r="G13" s="36" t="str">
         <f aca="false">IF(F13="","",ABS(F13-D13)/D13)</f>
         <v/>
       </c>
-      <c r="H13" s="33"/>
-      <c r="I13" s="34" t="str">
+      <c r="H13" s="35"/>
+      <c r="I13" s="36" t="str">
         <f aca="false">IF(H13="","",ABS(H13-C13)/C13)</f>
         <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="12" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="12"/>
@@ -2730,12 +2825,12 @@
   <sheetData>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="12" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -2743,62 +2838,62 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="C5" s="32" t="n">
+        <v>134</v>
+      </c>
+      <c r="C5" s="34" t="n">
         <v>100000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="35" t="s">
-        <v>128</v>
-      </c>
-      <c r="C7" s="35"/>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35"/>
+      <c r="B7" s="37" t="s">
+        <v>135</v>
+      </c>
+      <c r="C7" s="37"/>
+      <c r="D7" s="37"/>
+      <c r="E7" s="37"/>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="C9" s="36" t="n">
-        <f aca="false">'Mesh Levels'!$E$21</f>
+        <v>139</v>
+      </c>
+      <c r="C9" s="38" t="n">
+        <f aca="false">'Mesh Levels'!$E$29</f>
         <v>3.43167571948627</v>
       </c>
-      <c r="D9" s="36" t="n">
-        <f aca="false">'Mesh Levels'!$D$21</f>
+      <c r="D9" s="38" t="n">
+        <f aca="false">'Mesh Levels'!$D$29</f>
         <v>4.8393110188735</v>
       </c>
-      <c r="E9" s="36" t="n">
-        <f aca="false">'Mesh Levels'!$C$21</f>
+      <c r="E9" s="38" t="n">
+        <f aca="false">'Mesh Levels'!$C$29</f>
         <v>6.72473347933769</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="C10" s="33"/>
-      <c r="D10" s="33"/>
-      <c r="E10" s="33"/>
+        <v>140</v>
+      </c>
+      <c r="C10" s="35"/>
+      <c r="D10" s="35"/>
+      <c r="E10" s="35"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="7" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C12" s="26" t="n">
         <f aca="false">D9/C9</f>
@@ -2807,7 +2902,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="7" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="C13" s="26" t="n">
         <f aca="false">E9/D9</f>
@@ -2816,7 +2911,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="7" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="C14" s="18" t="str">
         <f aca="false">IF(OR(C10="",D10=""),"",D10-C10)</f>
@@ -2825,7 +2920,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="7" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="C15" s="18" t="str">
         <f aca="false">IF(OR(D10="",E10=""),"",E10-D10)</f>
@@ -2834,7 +2929,7 @@
     </row>
     <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="4" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="C16" s="26" t="str">
         <f aca="false">IF(OR(C14="",C15=""),"",LN(ABS(C15/C14))/LN(C12))</f>
@@ -2843,7 +2938,7 @@
     </row>
     <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="4" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="C17" s="18" t="str">
         <f aca="false">IF(C16="","",(C12^C16*C10-D10)/(C12^C16-1))</f>
@@ -2852,89 +2947,89 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="C18" s="37" t="str">
+        <v>147</v>
+      </c>
+      <c r="C18" s="39" t="str">
         <f aca="false">IF(OR(C10="",D10=""),"",ABS((C10-D10)/C10))</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="7" t="s">
-        <v>141</v>
-      </c>
-      <c r="C19" s="37" t="str">
+        <v>148</v>
+      </c>
+      <c r="C19" s="39" t="str">
         <f aca="false">IF(C17="","",ABS((C17-C10)/C17))</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C20" s="38" t="str">
+        <v>149</v>
+      </c>
+      <c r="C20" s="40" t="str">
         <f aca="false">IF(OR(C16="",C18=""),"",1.25*C18/(C12^C16-1))</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="12" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="C21" s="12"/>
       <c r="D21" s="12"/>
       <c r="E21" s="12"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="35" t="s">
-        <v>144</v>
-      </c>
-      <c r="C23" s="35"/>
-      <c r="D23" s="35"/>
-      <c r="E23" s="35"/>
+      <c r="B23" s="37" t="s">
+        <v>151</v>
+      </c>
+      <c r="C23" s="37"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="37"/>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="C25" s="36" t="n">
-        <f aca="false">'Mesh Levels'!$E$21</f>
+        <v>139</v>
+      </c>
+      <c r="C25" s="38" t="n">
+        <f aca="false">'Mesh Levels'!$E$29</f>
         <v>3.43167571948627</v>
       </c>
-      <c r="D25" s="36" t="n">
-        <f aca="false">'Mesh Levels'!$D$21</f>
+      <c r="D25" s="38" t="n">
+        <f aca="false">'Mesh Levels'!$D$29</f>
         <v>4.8393110188735</v>
       </c>
-      <c r="E25" s="36" t="n">
-        <f aca="false">'Mesh Levels'!$C$21</f>
+      <c r="E25" s="38" t="n">
+        <f aca="false">'Mesh Levels'!$C$29</f>
         <v>6.72473347933769</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="7" t="s">
-        <v>145</v>
-      </c>
-      <c r="C26" s="33"/>
-      <c r="D26" s="33"/>
-      <c r="E26" s="33"/>
+        <v>152</v>
+      </c>
+      <c r="C26" s="35"/>
+      <c r="D26" s="35"/>
+      <c r="E26" s="35"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="7" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C28" s="26" t="n">
         <f aca="false">D25/C25</f>
@@ -2943,7 +3038,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="7" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="C29" s="26" t="n">
         <f aca="false">E25/D25</f>
@@ -2952,7 +3047,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="7" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="C30" s="18" t="str">
         <f aca="false">IF(OR(C26="",D26=""),"",D26-C26)</f>
@@ -2961,7 +3056,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="7" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="C31" s="18" t="str">
         <f aca="false">IF(OR(D26="",E26=""),"",E26-D26)</f>
@@ -2970,7 +3065,7 @@
     </row>
     <row r="32" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="4" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="C32" s="26" t="str">
         <f aca="false">IF(OR(C30="",C31=""),"",LN(ABS(C31/C30))/LN(C28))</f>
@@ -2979,7 +3074,7 @@
     </row>
     <row r="33" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="4" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="C33" s="18" t="str">
         <f aca="false">IF(C32="","",(C28^C32*C26-D26)/(C28^C32-1))</f>
@@ -2988,34 +3083,34 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="C34" s="37" t="str">
+        <v>147</v>
+      </c>
+      <c r="C34" s="39" t="str">
         <f aca="false">IF(OR(C26="",D26=""),"",ABS((C26-D26)/C26))</f>
         <v/>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="7" t="s">
-        <v>141</v>
-      </c>
-      <c r="C35" s="37" t="str">
+        <v>148</v>
+      </c>
+      <c r="C35" s="39" t="str">
         <f aca="false">IF(C33="","",ABS((C33-C26)/C33))</f>
         <v/>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C36" s="38" t="str">
+        <v>149</v>
+      </c>
+      <c r="C36" s="40" t="str">
         <f aca="false">IF(OR(C32="",C34=""),"",1.25*C34/(C28^C32-1))</f>
         <v/>
       </c>
     </row>
     <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="12" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="C37" s="12"/>
       <c r="D37" s="12"/>
@@ -3075,12 +3170,12 @@
   <sheetData>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="12" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -3094,7 +3189,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="7" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C5" s="11" t="n">
         <v>39.2</v>
@@ -3102,300 +3197,300 @@
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="D7" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="42" t="n">
+        <v>933.7</v>
+      </c>
+      <c r="D8" s="42" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E8" s="42" t="n">
+        <v>102.2</v>
+      </c>
+      <c r="F8" s="42" t="n">
+        <v>47.7</v>
+      </c>
+      <c r="G8" s="42" t="n">
+        <v>124</v>
+      </c>
+      <c r="H8" s="29" t="n">
+        <v>72.51</v>
+      </c>
+      <c r="I8" s="35"/>
+      <c r="J8" s="35"/>
+      <c r="K8" s="36" t="str">
+        <f aca="false">IF(J8="","",ABS(J8-H8)/H8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="42" t="n">
+        <v>968.2</v>
+      </c>
+      <c r="D9" s="42" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="E9" s="42" t="n">
         <v>151</v>
       </c>
-      <c r="E7" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="J7" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="K7" s="6" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="39" t="n">
+      <c r="F9" s="42" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="G9" s="42" t="n">
+        <v>173.3</v>
+      </c>
+      <c r="H9" s="29" t="n">
+        <v>70.9</v>
+      </c>
+      <c r="I9" s="35"/>
+      <c r="J9" s="35"/>
+      <c r="K9" s="36" t="str">
+        <f aca="false">IF(J9="","",ABS(J9-H9)/H9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="41" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="42" t="n">
+        <v>982.3</v>
+      </c>
+      <c r="D10" s="42" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E10" s="42" t="n">
+        <v>197.5</v>
+      </c>
+      <c r="F10" s="42" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="G10" s="42" t="n">
+        <v>219.5</v>
+      </c>
+      <c r="H10" s="29" t="n">
+        <v>70.17</v>
+      </c>
+      <c r="I10" s="35"/>
+      <c r="J10" s="35"/>
+      <c r="K10" s="36" t="str">
+        <f aca="false">IF(J10="","",ABS(J10-H10)/H10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="41" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" s="42" t="n">
+        <v>906.6</v>
+      </c>
+      <c r="D11" s="42" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="E11" s="42" t="n">
+        <v>250.7</v>
+      </c>
+      <c r="F11" s="42" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="G11" s="42" t="n">
+        <v>269.4</v>
+      </c>
+      <c r="H11" s="29" t="n">
+        <v>70.25</v>
+      </c>
+      <c r="I11" s="35"/>
+      <c r="J11" s="35"/>
+      <c r="K11" s="36" t="str">
+        <f aca="false">IF(J11="","",ABS(J11-H11)/H11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="41" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" s="42" t="n">
+        <v>937.9</v>
+      </c>
+      <c r="D12" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="40" t="n">
-        <v>933.7</v>
-      </c>
-      <c r="D8" s="40" t="n">
+      <c r="E12" s="42" t="n">
+        <v>297.8</v>
+      </c>
+      <c r="F12" s="42" t="n">
+        <v>55.5</v>
+      </c>
+      <c r="G12" s="42" t="n">
+        <v>316.9</v>
+      </c>
+      <c r="H12" s="29" t="n">
+        <v>67.98</v>
+      </c>
+      <c r="I12" s="35"/>
+      <c r="J12" s="35"/>
+      <c r="K12" s="36" t="str">
+        <f aca="false">IF(J12="","",ABS(J12-H12)/H12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="41" t="n">
+        <v>6</v>
+      </c>
+      <c r="C13" s="42" t="n">
+        <v>880.6</v>
+      </c>
+      <c r="D13" s="42" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="E13" s="42" t="n">
+        <v>299</v>
+      </c>
+      <c r="F13" s="42" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="G13" s="42" t="n">
+        <v>317.2</v>
+      </c>
+      <c r="H13" s="29" t="n">
+        <v>68.92</v>
+      </c>
+      <c r="I13" s="35"/>
+      <c r="J13" s="35"/>
+      <c r="K13" s="36" t="str">
+        <f aca="false">IF(J13="","",ABS(J13-H13)/H13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="41" t="n">
+        <v>7</v>
+      </c>
+      <c r="C14" s="42" t="n">
+        <v>920.9</v>
+      </c>
+      <c r="D14" s="42" t="n">
         <v>2.6</v>
       </c>
-      <c r="E8" s="40" t="n">
-        <v>102.2</v>
-      </c>
-      <c r="F8" s="40" t="n">
-        <v>47.7</v>
-      </c>
-      <c r="G8" s="40" t="n">
-        <v>124</v>
-      </c>
-      <c r="H8" s="41" t="n">
-        <v>72.51</v>
-      </c>
-      <c r="I8" s="33"/>
-      <c r="J8" s="33"/>
-      <c r="K8" s="34" t="str">
-        <f aca="false">IF(J8="","",ABS(J8-H8)/H8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="39" t="n">
-        <v>2</v>
-      </c>
-      <c r="C9" s="40" t="n">
-        <v>968.2</v>
-      </c>
-      <c r="D9" s="40" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="E9" s="40" t="n">
-        <v>151</v>
-      </c>
-      <c r="F9" s="40" t="n">
-        <v>47.8</v>
-      </c>
-      <c r="G9" s="40" t="n">
-        <v>173.3</v>
-      </c>
-      <c r="H9" s="41" t="n">
-        <v>70.9</v>
-      </c>
-      <c r="I9" s="33"/>
-      <c r="J9" s="33"/>
-      <c r="K9" s="34" t="str">
-        <f aca="false">IF(J9="","",ABS(J9-H9)/H9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="39" t="n">
-        <v>3</v>
-      </c>
-      <c r="C10" s="40" t="n">
-        <v>982.3</v>
-      </c>
-      <c r="D10" s="40" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E10" s="40" t="n">
-        <v>197.5</v>
-      </c>
-      <c r="F10" s="40" t="n">
-        <v>49.1</v>
-      </c>
-      <c r="G10" s="40" t="n">
-        <v>219.5</v>
-      </c>
-      <c r="H10" s="41" t="n">
-        <v>70.17</v>
-      </c>
-      <c r="I10" s="33"/>
-      <c r="J10" s="33"/>
-      <c r="K10" s="34" t="str">
-        <f aca="false">IF(J10="","",ABS(J10-H10)/H10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="39" t="n">
-        <v>4</v>
-      </c>
-      <c r="C11" s="40" t="n">
-        <v>906.6</v>
-      </c>
-      <c r="D11" s="40" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="E11" s="40" t="n">
-        <v>250.7</v>
-      </c>
-      <c r="F11" s="40" t="n">
-        <v>54.7</v>
-      </c>
-      <c r="G11" s="40" t="n">
-        <v>269.4</v>
-      </c>
-      <c r="H11" s="41" t="n">
-        <v>70.25</v>
-      </c>
-      <c r="I11" s="33"/>
-      <c r="J11" s="33"/>
-      <c r="K11" s="34" t="str">
-        <f aca="false">IF(J11="","",ABS(J11-H11)/H11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="39" t="n">
-        <v>5</v>
-      </c>
-      <c r="C12" s="40" t="n">
-        <v>937.9</v>
-      </c>
-      <c r="D12" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="40" t="n">
-        <v>297.8</v>
-      </c>
-      <c r="F12" s="40" t="n">
-        <v>55.5</v>
-      </c>
-      <c r="G12" s="40" t="n">
-        <v>316.9</v>
-      </c>
-      <c r="H12" s="41" t="n">
-        <v>67.98</v>
-      </c>
-      <c r="I12" s="33"/>
-      <c r="J12" s="33"/>
-      <c r="K12" s="34" t="str">
-        <f aca="false">IF(J12="","",ABS(J12-H12)/H12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="39" t="n">
-        <v>6</v>
-      </c>
-      <c r="C13" s="40" t="n">
-        <v>880.6</v>
-      </c>
-      <c r="D13" s="40" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="E13" s="40" t="n">
-        <v>299</v>
-      </c>
-      <c r="F13" s="40" t="n">
-        <v>55.6</v>
-      </c>
-      <c r="G13" s="40" t="n">
-        <v>317.2</v>
-      </c>
-      <c r="H13" s="41" t="n">
-        <v>68.92</v>
-      </c>
-      <c r="I13" s="33"/>
-      <c r="J13" s="33"/>
-      <c r="K13" s="34" t="str">
-        <f aca="false">IF(J13="","",ABS(J13-H13)/H13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="39" t="n">
-        <v>7</v>
-      </c>
-      <c r="C14" s="40" t="n">
+      <c r="E14" s="42" t="n">
+        <v>379.5</v>
+      </c>
+      <c r="F14" s="42" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="G14" s="42" t="n">
+        <v>398</v>
+      </c>
+      <c r="H14" s="29" t="n">
+        <v>62.34</v>
+      </c>
+      <c r="I14" s="35"/>
+      <c r="J14" s="35"/>
+      <c r="K14" s="36" t="str">
+        <f aca="false">IF(J14="","",ABS(J14-H14)/H14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="41" t="n">
+        <v>8</v>
+      </c>
+      <c r="C15" s="42" t="n">
+        <v>903.2</v>
+      </c>
+      <c r="D15" s="42" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E15" s="42" t="n">
+        <v>355.9</v>
+      </c>
+      <c r="F15" s="42" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="G15" s="42" t="n">
+        <v>374</v>
+      </c>
+      <c r="H15" s="29" t="n">
+        <v>63.82</v>
+      </c>
+      <c r="I15" s="35"/>
+      <c r="J15" s="35"/>
+      <c r="K15" s="36" t="str">
+        <f aca="false">IF(J15="","",ABS(J15-H15)/H15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="41" t="n">
+        <v>9</v>
+      </c>
+      <c r="C16" s="42" t="n">
         <v>920.9</v>
       </c>
-      <c r="D14" s="40" t="n">
+      <c r="D16" s="42" t="n">
         <v>2.6</v>
       </c>
-      <c r="E14" s="40" t="n">
+      <c r="E16" s="42" t="n">
         <v>379.5</v>
       </c>
-      <c r="F14" s="40" t="n">
+      <c r="F16" s="42" t="n">
         <v>56.8</v>
       </c>
-      <c r="G14" s="40" t="n">
+      <c r="G16" s="42" t="n">
         <v>398</v>
       </c>
-      <c r="H14" s="41" t="n">
+      <c r="H16" s="29" t="n">
         <v>62.34</v>
       </c>
-      <c r="I14" s="33"/>
-      <c r="J14" s="33"/>
-      <c r="K14" s="34" t="str">
-        <f aca="false">IF(J14="","",ABS(J14-H14)/H14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="39" t="n">
-        <v>8</v>
-      </c>
-      <c r="C15" s="40" t="n">
-        <v>903.2</v>
-      </c>
-      <c r="D15" s="40" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="E15" s="40" t="n">
-        <v>355.9</v>
-      </c>
-      <c r="F15" s="40" t="n">
-        <v>56.3</v>
-      </c>
-      <c r="G15" s="40" t="n">
-        <v>374</v>
-      </c>
-      <c r="H15" s="41" t="n">
-        <v>63.82</v>
-      </c>
-      <c r="I15" s="33"/>
-      <c r="J15" s="33"/>
-      <c r="K15" s="34" t="str">
-        <f aca="false">IF(J15="","",ABS(J15-H15)/H15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="39" t="n">
-        <v>9</v>
-      </c>
-      <c r="C16" s="40" t="n">
-        <v>920.9</v>
-      </c>
-      <c r="D16" s="40" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="E16" s="40" t="n">
-        <v>379.5</v>
-      </c>
-      <c r="F16" s="40" t="n">
-        <v>56.8</v>
-      </c>
-      <c r="G16" s="40" t="n">
-        <v>398</v>
-      </c>
-      <c r="H16" s="41" t="n">
-        <v>62.34</v>
-      </c>
-      <c r="I16" s="33"/>
-      <c r="J16" s="33"/>
-      <c r="K16" s="34" t="str">
+      <c r="I16" s="35"/>
+      <c r="J16" s="35"/>
+      <c r="K16" s="36" t="str">
         <f aca="false">IF(J16="","",ABS(J16-H16)/H16)</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="12" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>
@@ -3445,12 +3540,12 @@
   <sheetData>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="12" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -3470,1215 +3565,1215 @@
       <c r="R3" s="12"/>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="42" t="s">
-        <v>162</v>
-      </c>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="33"/>
+      <c r="B5" s="43" t="s">
+        <v>169</v>
+      </c>
+      <c r="C5" s="43"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="35"/>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="42" t="s">
-        <v>163</v>
-      </c>
-      <c r="C6" s="42"/>
-      <c r="D6" s="42"/>
-      <c r="E6" s="42"/>
-      <c r="F6" s="42"/>
-      <c r="G6" s="33"/>
+      <c r="B6" s="43" t="s">
+        <v>170</v>
+      </c>
+      <c r="C6" s="43"/>
+      <c r="D6" s="43"/>
+      <c r="E6" s="43"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="35"/>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="N8" s="6" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="O8" s="6" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="P8" s="6" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="Q8" s="6" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="R8" s="6" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="39" t="n">
+      <c r="B9" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="41" t="n">
+      <c r="C9" s="29" t="n">
         <v>3.03</v>
       </c>
-      <c r="D9" s="41" t="n">
+      <c r="D9" s="29" t="n">
         <v>0.23</v>
       </c>
-      <c r="E9" s="41" t="n">
+      <c r="E9" s="29" t="n">
         <v>0.04</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>181</v>
-      </c>
-      <c r="G9" s="40" t="n">
+        <v>188</v>
+      </c>
+      <c r="G9" s="42" t="n">
         <v>0.5</v>
       </c>
-      <c r="H9" s="39" t="n">
+      <c r="H9" s="41" t="n">
         <v>200</v>
       </c>
-      <c r="I9" s="39" t="n">
+      <c r="I9" s="41" t="n">
         <v>15</v>
       </c>
-      <c r="J9" s="40" t="n">
+      <c r="J9" s="42" t="n">
         <v>0.6</v>
       </c>
-      <c r="K9" s="40" t="n">
+      <c r="K9" s="42" t="n">
         <v>13.8</v>
       </c>
-      <c r="L9" s="33"/>
-      <c r="M9" s="33"/>
+      <c r="L9" s="35"/>
+      <c r="M9" s="35"/>
       <c r="N9" s="26" t="str">
         <f aca="false">IF(OR(L9="",M9="",$G$5="",$G$6=""),"",(L9/$G$5)/(M9/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O9" s="33"/>
-      <c r="P9" s="33"/>
-      <c r="Q9" s="33"/>
-      <c r="R9" s="33"/>
+      <c r="O9" s="35"/>
+      <c r="P9" s="35"/>
+      <c r="Q9" s="35"/>
+      <c r="R9" s="35"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="39" t="n">
+      <c r="B10" s="41" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="41" t="n">
+      <c r="C10" s="29" t="n">
         <v>3.03</v>
       </c>
-      <c r="D10" s="41" t="n">
+      <c r="D10" s="29" t="n">
         <v>0.23</v>
       </c>
-      <c r="E10" s="41" t="n">
+      <c r="E10" s="29" t="n">
         <v>0.08</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="G10" s="40" t="n">
+        <v>189</v>
+      </c>
+      <c r="G10" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="39" t="n">
+      <c r="H10" s="41" t="n">
         <v>200</v>
       </c>
-      <c r="I10" s="39" t="n">
+      <c r="I10" s="41" t="n">
         <v>15</v>
       </c>
-      <c r="J10" s="40" t="n">
+      <c r="J10" s="42" t="n">
         <v>1.2</v>
       </c>
-      <c r="K10" s="40" t="n">
+      <c r="K10" s="42" t="n">
         <v>12.6</v>
       </c>
-      <c r="L10" s="33"/>
-      <c r="M10" s="33"/>
+      <c r="L10" s="35"/>
+      <c r="M10" s="35"/>
       <c r="N10" s="26" t="str">
         <f aca="false">IF(OR(L10="",M10="",$G$5="",$G$6=""),"",(L10/$G$5)/(M10/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O10" s="33"/>
-      <c r="P10" s="33"/>
-      <c r="Q10" s="33"/>
-      <c r="R10" s="33"/>
+      <c r="O10" s="35"/>
+      <c r="P10" s="35"/>
+      <c r="Q10" s="35"/>
+      <c r="R10" s="35"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="39" t="n">
+      <c r="B11" s="41" t="n">
         <v>3</v>
       </c>
-      <c r="C11" s="41" t="n">
+      <c r="C11" s="29" t="n">
         <v>3.03</v>
       </c>
-      <c r="D11" s="41" t="n">
+      <c r="D11" s="29" t="n">
         <v>0.23</v>
       </c>
-      <c r="E11" s="41" t="n">
+      <c r="E11" s="29" t="n">
         <v>0.12</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>183</v>
-      </c>
-      <c r="G11" s="40" t="n">
+        <v>190</v>
+      </c>
+      <c r="G11" s="42" t="n">
         <v>2</v>
       </c>
-      <c r="H11" s="39" t="n">
+      <c r="H11" s="41" t="n">
         <v>200</v>
       </c>
-      <c r="I11" s="39" t="n">
+      <c r="I11" s="41" t="n">
         <v>15</v>
       </c>
-      <c r="J11" s="40" t="n">
+      <c r="J11" s="42" t="n">
         <v>1.8</v>
       </c>
-      <c r="K11" s="40" t="n">
+      <c r="K11" s="42" t="n">
         <v>11.4</v>
       </c>
-      <c r="L11" s="33"/>
-      <c r="M11" s="33"/>
+      <c r="L11" s="35"/>
+      <c r="M11" s="35"/>
       <c r="N11" s="26" t="str">
         <f aca="false">IF(OR(L11="",M11="",$G$5="",$G$6=""),"",(L11/$G$5)/(M11/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O11" s="33"/>
-      <c r="P11" s="33"/>
-      <c r="Q11" s="33"/>
-      <c r="R11" s="33"/>
+      <c r="O11" s="35"/>
+      <c r="P11" s="35"/>
+      <c r="Q11" s="35"/>
+      <c r="R11" s="35"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="39" t="n">
+      <c r="B12" s="41" t="n">
         <v>4</v>
       </c>
-      <c r="C12" s="41" t="n">
+      <c r="C12" s="29" t="n">
         <v>3.03</v>
       </c>
-      <c r="D12" s="41" t="n">
+      <c r="D12" s="29" t="n">
         <v>0.38</v>
       </c>
-      <c r="E12" s="41" t="n">
+      <c r="E12" s="29" t="n">
         <v>0.04</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="G12" s="40" t="n">
+        <v>189</v>
+      </c>
+      <c r="G12" s="42" t="n">
         <v>2</v>
       </c>
-      <c r="H12" s="39" t="n">
+      <c r="H12" s="41" t="n">
         <v>200</v>
       </c>
-      <c r="I12" s="39" t="n">
+      <c r="I12" s="41" t="n">
         <v>25</v>
       </c>
-      <c r="J12" s="40" t="n">
+      <c r="J12" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="K12" s="40" t="n">
+      <c r="K12" s="42" t="n">
         <v>23</v>
       </c>
-      <c r="L12" s="33"/>
-      <c r="M12" s="33"/>
+      <c r="L12" s="35"/>
+      <c r="M12" s="35"/>
       <c r="N12" s="26" t="str">
         <f aca="false">IF(OR(L12="",M12="",$G$5="",$G$6=""),"",(L12/$G$5)/(M12/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O12" s="33"/>
-      <c r="P12" s="33"/>
-      <c r="Q12" s="33"/>
-      <c r="R12" s="33"/>
+      <c r="O12" s="35"/>
+      <c r="P12" s="35"/>
+      <c r="Q12" s="35"/>
+      <c r="R12" s="35"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="39" t="n">
+      <c r="B13" s="41" t="n">
         <v>5</v>
       </c>
-      <c r="C13" s="41" t="n">
+      <c r="C13" s="29" t="n">
         <v>3.03</v>
       </c>
-      <c r="D13" s="41" t="n">
+      <c r="D13" s="29" t="n">
         <v>0.38</v>
       </c>
-      <c r="E13" s="41" t="n">
+      <c r="E13" s="29" t="n">
         <v>0.08</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>183</v>
-      </c>
-      <c r="G13" s="40" t="n">
+        <v>190</v>
+      </c>
+      <c r="G13" s="42" t="n">
         <v>0.5</v>
       </c>
-      <c r="H13" s="39" t="n">
+      <c r="H13" s="41" t="n">
         <v>200</v>
       </c>
-      <c r="I13" s="39" t="n">
+      <c r="I13" s="41" t="n">
         <v>25</v>
       </c>
-      <c r="J13" s="40" t="n">
+      <c r="J13" s="42" t="n">
         <v>2</v>
       </c>
-      <c r="K13" s="40" t="n">
+      <c r="K13" s="42" t="n">
         <v>21</v>
       </c>
-      <c r="L13" s="33"/>
-      <c r="M13" s="33"/>
+      <c r="L13" s="35"/>
+      <c r="M13" s="35"/>
       <c r="N13" s="26" t="str">
         <f aca="false">IF(OR(L13="",M13="",$G$5="",$G$6=""),"",(L13/$G$5)/(M13/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O13" s="33"/>
-      <c r="P13" s="33"/>
-      <c r="Q13" s="33"/>
-      <c r="R13" s="33"/>
+      <c r="O13" s="35"/>
+      <c r="P13" s="35"/>
+      <c r="Q13" s="35"/>
+      <c r="R13" s="35"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="39" t="n">
+      <c r="B14" s="41" t="n">
         <v>6</v>
       </c>
-      <c r="C14" s="41" t="n">
+      <c r="C14" s="29" t="n">
         <v>3.03</v>
       </c>
-      <c r="D14" s="41" t="n">
+      <c r="D14" s="29" t="n">
         <v>0.38</v>
       </c>
-      <c r="E14" s="41" t="n">
+      <c r="E14" s="29" t="n">
         <v>0.12</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>181</v>
-      </c>
-      <c r="G14" s="40" t="n">
+        <v>188</v>
+      </c>
+      <c r="G14" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="H14" s="39" t="n">
+      <c r="H14" s="41" t="n">
         <v>200</v>
       </c>
-      <c r="I14" s="39" t="n">
+      <c r="I14" s="41" t="n">
         <v>25</v>
       </c>
-      <c r="J14" s="40" t="n">
+      <c r="J14" s="42" t="n">
         <v>3</v>
       </c>
-      <c r="K14" s="40" t="n">
+      <c r="K14" s="42" t="n">
         <v>19</v>
       </c>
-      <c r="L14" s="33"/>
-      <c r="M14" s="33"/>
+      <c r="L14" s="35"/>
+      <c r="M14" s="35"/>
       <c r="N14" s="26" t="str">
         <f aca="false">IF(OR(L14="",M14="",$G$5="",$G$6=""),"",(L14/$G$5)/(M14/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O14" s="33"/>
-      <c r="P14" s="33"/>
-      <c r="Q14" s="33"/>
-      <c r="R14" s="33"/>
+      <c r="O14" s="35"/>
+      <c r="P14" s="35"/>
+      <c r="Q14" s="35"/>
+      <c r="R14" s="35"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="39" t="n">
+      <c r="B15" s="41" t="n">
         <v>7</v>
       </c>
-      <c r="C15" s="41" t="n">
+      <c r="C15" s="29" t="n">
         <v>3.03</v>
       </c>
-      <c r="D15" s="41" t="n">
+      <c r="D15" s="29" t="n">
         <v>0.53</v>
       </c>
-      <c r="E15" s="41" t="n">
+      <c r="E15" s="29" t="n">
         <v>0.04</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>183</v>
-      </c>
-      <c r="G15" s="40" t="n">
+        <v>190</v>
+      </c>
+      <c r="G15" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="H15" s="39" t="n">
+      <c r="H15" s="41" t="n">
         <v>200</v>
       </c>
-      <c r="I15" s="39" t="n">
+      <c r="I15" s="41" t="n">
         <v>35</v>
       </c>
-      <c r="J15" s="40" t="n">
+      <c r="J15" s="42" t="n">
         <v>1.4</v>
       </c>
-      <c r="K15" s="40" t="n">
+      <c r="K15" s="42" t="n">
         <v>32.2</v>
       </c>
-      <c r="L15" s="33"/>
-      <c r="M15" s="33"/>
+      <c r="L15" s="35"/>
+      <c r="M15" s="35"/>
       <c r="N15" s="26" t="str">
         <f aca="false">IF(OR(L15="",M15="",$G$5="",$G$6=""),"",(L15/$G$5)/(M15/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O15" s="33"/>
-      <c r="P15" s="33"/>
-      <c r="Q15" s="33"/>
-      <c r="R15" s="33"/>
+      <c r="O15" s="35"/>
+      <c r="P15" s="35"/>
+      <c r="Q15" s="35"/>
+      <c r="R15" s="35"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="39" t="n">
+      <c r="B16" s="41" t="n">
         <v>8</v>
       </c>
-      <c r="C16" s="41" t="n">
+      <c r="C16" s="29" t="n">
         <v>3.03</v>
       </c>
-      <c r="D16" s="41" t="n">
+      <c r="D16" s="29" t="n">
         <v>0.53</v>
       </c>
-      <c r="E16" s="41" t="n">
+      <c r="E16" s="29" t="n">
         <v>0.08</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>181</v>
-      </c>
-      <c r="G16" s="40" t="n">
+        <v>188</v>
+      </c>
+      <c r="G16" s="42" t="n">
         <v>2</v>
       </c>
-      <c r="H16" s="39" t="n">
+      <c r="H16" s="41" t="n">
         <v>200</v>
       </c>
-      <c r="I16" s="39" t="n">
+      <c r="I16" s="41" t="n">
         <v>35</v>
       </c>
-      <c r="J16" s="40" t="n">
+      <c r="J16" s="42" t="n">
         <v>2.8</v>
       </c>
-      <c r="K16" s="40" t="n">
+      <c r="K16" s="42" t="n">
         <v>29.4</v>
       </c>
-      <c r="L16" s="33"/>
-      <c r="M16" s="33"/>
+      <c r="L16" s="35"/>
+      <c r="M16" s="35"/>
       <c r="N16" s="26" t="str">
         <f aca="false">IF(OR(L16="",M16="",$G$5="",$G$6=""),"",(L16/$G$5)/(M16/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O16" s="33"/>
-      <c r="P16" s="33"/>
-      <c r="Q16" s="33"/>
-      <c r="R16" s="33"/>
+      <c r="O16" s="35"/>
+      <c r="P16" s="35"/>
+      <c r="Q16" s="35"/>
+      <c r="R16" s="35"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="39" t="n">
+      <c r="B17" s="41" t="n">
         <v>9</v>
       </c>
-      <c r="C17" s="41" t="n">
+      <c r="C17" s="29" t="n">
         <v>3.03</v>
       </c>
-      <c r="D17" s="41" t="n">
+      <c r="D17" s="29" t="n">
         <v>0.53</v>
       </c>
-      <c r="E17" s="41" t="n">
+      <c r="E17" s="29" t="n">
         <v>0.12</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="G17" s="40" t="n">
+        <v>189</v>
+      </c>
+      <c r="G17" s="42" t="n">
         <v>0.5</v>
       </c>
-      <c r="H17" s="39" t="n">
+      <c r="H17" s="41" t="n">
         <v>200</v>
       </c>
-      <c r="I17" s="39" t="n">
+      <c r="I17" s="41" t="n">
         <v>35</v>
       </c>
-      <c r="J17" s="40" t="n">
+      <c r="J17" s="42" t="n">
         <v>4.2</v>
       </c>
-      <c r="K17" s="40" t="n">
+      <c r="K17" s="42" t="n">
         <v>26.6</v>
       </c>
-      <c r="L17" s="33"/>
-      <c r="M17" s="33"/>
+      <c r="L17" s="35"/>
+      <c r="M17" s="35"/>
       <c r="N17" s="26" t="str">
         <f aca="false">IF(OR(L17="",M17="",$G$5="",$G$6=""),"",(L17/$G$5)/(M17/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O17" s="33"/>
-      <c r="P17" s="33"/>
-      <c r="Q17" s="33"/>
-      <c r="R17" s="33"/>
+      <c r="O17" s="35"/>
+      <c r="P17" s="35"/>
+      <c r="Q17" s="35"/>
+      <c r="R17" s="35"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="39" t="n">
+      <c r="B18" s="41" t="n">
         <v>10</v>
       </c>
-      <c r="C18" s="41" t="n">
+      <c r="C18" s="29" t="n">
         <v>4.55</v>
       </c>
-      <c r="D18" s="41" t="n">
+      <c r="D18" s="29" t="n">
         <v>0.23</v>
       </c>
-      <c r="E18" s="41" t="n">
+      <c r="E18" s="29" t="n">
         <v>0.04</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="G18" s="40" t="n">
+        <v>189</v>
+      </c>
+      <c r="G18" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="H18" s="39" t="n">
+      <c r="H18" s="41" t="n">
         <v>300</v>
       </c>
-      <c r="I18" s="39" t="n">
+      <c r="I18" s="41" t="n">
         <v>15</v>
       </c>
-      <c r="J18" s="40" t="n">
+      <c r="J18" s="42" t="n">
         <v>0.6</v>
       </c>
-      <c r="K18" s="40" t="n">
+      <c r="K18" s="42" t="n">
         <v>13.8</v>
       </c>
-      <c r="L18" s="33"/>
-      <c r="M18" s="33"/>
+      <c r="L18" s="35"/>
+      <c r="M18" s="35"/>
       <c r="N18" s="26" t="str">
         <f aca="false">IF(OR(L18="",M18="",$G$5="",$G$6=""),"",(L18/$G$5)/(M18/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O18" s="33"/>
-      <c r="P18" s="33"/>
-      <c r="Q18" s="33"/>
-      <c r="R18" s="33"/>
+      <c r="O18" s="35"/>
+      <c r="P18" s="35"/>
+      <c r="Q18" s="35"/>
+      <c r="R18" s="35"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="39" t="n">
+      <c r="B19" s="41" t="n">
         <v>11</v>
       </c>
-      <c r="C19" s="41" t="n">
+      <c r="C19" s="29" t="n">
         <v>4.55</v>
       </c>
-      <c r="D19" s="41" t="n">
+      <c r="D19" s="29" t="n">
         <v>0.23</v>
       </c>
-      <c r="E19" s="41" t="n">
+      <c r="E19" s="29" t="n">
         <v>0.08</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>183</v>
-      </c>
-      <c r="G19" s="40" t="n">
+        <v>190</v>
+      </c>
+      <c r="G19" s="42" t="n">
         <v>2</v>
       </c>
-      <c r="H19" s="39" t="n">
+      <c r="H19" s="41" t="n">
         <v>300</v>
       </c>
-      <c r="I19" s="39" t="n">
+      <c r="I19" s="41" t="n">
         <v>15</v>
       </c>
-      <c r="J19" s="40" t="n">
+      <c r="J19" s="42" t="n">
         <v>1.2</v>
       </c>
-      <c r="K19" s="40" t="n">
+      <c r="K19" s="42" t="n">
         <v>12.6</v>
       </c>
-      <c r="L19" s="33"/>
-      <c r="M19" s="33"/>
+      <c r="L19" s="35"/>
+      <c r="M19" s="35"/>
       <c r="N19" s="26" t="str">
         <f aca="false">IF(OR(L19="",M19="",$G$5="",$G$6=""),"",(L19/$G$5)/(M19/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O19" s="33"/>
-      <c r="P19" s="33"/>
-      <c r="Q19" s="33"/>
-      <c r="R19" s="33"/>
+      <c r="O19" s="35"/>
+      <c r="P19" s="35"/>
+      <c r="Q19" s="35"/>
+      <c r="R19" s="35"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="39" t="n">
+      <c r="B20" s="41" t="n">
         <v>12</v>
       </c>
-      <c r="C20" s="41" t="n">
+      <c r="C20" s="29" t="n">
         <v>4.55</v>
       </c>
-      <c r="D20" s="41" t="n">
+      <c r="D20" s="29" t="n">
         <v>0.23</v>
       </c>
-      <c r="E20" s="41" t="n">
+      <c r="E20" s="29" t="n">
         <v>0.12</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>181</v>
-      </c>
-      <c r="G20" s="40" t="n">
+        <v>188</v>
+      </c>
+      <c r="G20" s="42" t="n">
         <v>0.5</v>
       </c>
-      <c r="H20" s="39" t="n">
+      <c r="H20" s="41" t="n">
         <v>300</v>
       </c>
-      <c r="I20" s="39" t="n">
+      <c r="I20" s="41" t="n">
         <v>15</v>
       </c>
-      <c r="J20" s="40" t="n">
+      <c r="J20" s="42" t="n">
         <v>1.8</v>
       </c>
-      <c r="K20" s="40" t="n">
+      <c r="K20" s="42" t="n">
         <v>11.4</v>
       </c>
-      <c r="L20" s="33"/>
-      <c r="M20" s="33"/>
+      <c r="L20" s="35"/>
+      <c r="M20" s="35"/>
       <c r="N20" s="26" t="str">
         <f aca="false">IF(OR(L20="",M20="",$G$5="",$G$6=""),"",(L20/$G$5)/(M20/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O20" s="33"/>
-      <c r="P20" s="33"/>
-      <c r="Q20" s="33"/>
-      <c r="R20" s="33"/>
+      <c r="O20" s="35"/>
+      <c r="P20" s="35"/>
+      <c r="Q20" s="35"/>
+      <c r="R20" s="35"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="39" t="n">
+      <c r="B21" s="41" t="n">
         <v>13</v>
       </c>
-      <c r="C21" s="41" t="n">
+      <c r="C21" s="29" t="n">
         <v>4.55</v>
       </c>
-      <c r="D21" s="41" t="n">
+      <c r="D21" s="29" t="n">
         <v>0.38</v>
       </c>
-      <c r="E21" s="41" t="n">
+      <c r="E21" s="29" t="n">
         <v>0.04</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>183</v>
-      </c>
-      <c r="G21" s="40" t="n">
+        <v>190</v>
+      </c>
+      <c r="G21" s="42" t="n">
         <v>0.5</v>
       </c>
-      <c r="H21" s="39" t="n">
+      <c r="H21" s="41" t="n">
         <v>300</v>
       </c>
-      <c r="I21" s="39" t="n">
+      <c r="I21" s="41" t="n">
         <v>25</v>
       </c>
-      <c r="J21" s="40" t="n">
+      <c r="J21" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="K21" s="40" t="n">
+      <c r="K21" s="42" t="n">
         <v>23</v>
       </c>
-      <c r="L21" s="33"/>
-      <c r="M21" s="33"/>
+      <c r="L21" s="35"/>
+      <c r="M21" s="35"/>
       <c r="N21" s="26" t="str">
         <f aca="false">IF(OR(L21="",M21="",$G$5="",$G$6=""),"",(L21/$G$5)/(M21/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O21" s="33"/>
-      <c r="P21" s="33"/>
-      <c r="Q21" s="33"/>
-      <c r="R21" s="33"/>
+      <c r="O21" s="35"/>
+      <c r="P21" s="35"/>
+      <c r="Q21" s="35"/>
+      <c r="R21" s="35"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="39" t="n">
+      <c r="B22" s="41" t="n">
         <v>14</v>
       </c>
-      <c r="C22" s="41" t="n">
+      <c r="C22" s="29" t="n">
         <v>4.55</v>
       </c>
-      <c r="D22" s="41" t="n">
+      <c r="D22" s="29" t="n">
         <v>0.38</v>
       </c>
-      <c r="E22" s="41" t="n">
+      <c r="E22" s="29" t="n">
         <v>0.08</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>181</v>
-      </c>
-      <c r="G22" s="40" t="n">
+        <v>188</v>
+      </c>
+      <c r="G22" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="H22" s="39" t="n">
+      <c r="H22" s="41" t="n">
         <v>300</v>
       </c>
-      <c r="I22" s="39" t="n">
+      <c r="I22" s="41" t="n">
         <v>25</v>
       </c>
-      <c r="J22" s="40" t="n">
+      <c r="J22" s="42" t="n">
         <v>2</v>
       </c>
-      <c r="K22" s="40" t="n">
+      <c r="K22" s="42" t="n">
         <v>21</v>
       </c>
-      <c r="L22" s="33"/>
-      <c r="M22" s="33"/>
+      <c r="L22" s="35"/>
+      <c r="M22" s="35"/>
       <c r="N22" s="26" t="str">
         <f aca="false">IF(OR(L22="",M22="",$G$5="",$G$6=""),"",(L22/$G$5)/(M22/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O22" s="33"/>
-      <c r="P22" s="33"/>
-      <c r="Q22" s="33"/>
-      <c r="R22" s="33"/>
+      <c r="O22" s="35"/>
+      <c r="P22" s="35"/>
+      <c r="Q22" s="35"/>
+      <c r="R22" s="35"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="39" t="n">
+      <c r="B23" s="41" t="n">
         <v>15</v>
       </c>
-      <c r="C23" s="41" t="n">
+      <c r="C23" s="29" t="n">
         <v>4.55</v>
       </c>
-      <c r="D23" s="41" t="n">
+      <c r="D23" s="29" t="n">
         <v>0.38</v>
       </c>
-      <c r="E23" s="41" t="n">
+      <c r="E23" s="29" t="n">
         <v>0.12</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="G23" s="40" t="n">
+        <v>189</v>
+      </c>
+      <c r="G23" s="42" t="n">
         <v>2</v>
       </c>
-      <c r="H23" s="39" t="n">
+      <c r="H23" s="41" t="n">
         <v>300</v>
       </c>
-      <c r="I23" s="39" t="n">
+      <c r="I23" s="41" t="n">
         <v>25</v>
       </c>
-      <c r="J23" s="40" t="n">
+      <c r="J23" s="42" t="n">
         <v>3</v>
       </c>
-      <c r="K23" s="40" t="n">
+      <c r="K23" s="42" t="n">
         <v>19</v>
       </c>
-      <c r="L23" s="33"/>
-      <c r="M23" s="33"/>
+      <c r="L23" s="35"/>
+      <c r="M23" s="35"/>
       <c r="N23" s="26" t="str">
         <f aca="false">IF(OR(L23="",M23="",$G$5="",$G$6=""),"",(L23/$G$5)/(M23/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O23" s="33"/>
-      <c r="P23" s="33"/>
-      <c r="Q23" s="33"/>
-      <c r="R23" s="33"/>
+      <c r="O23" s="35"/>
+      <c r="P23" s="35"/>
+      <c r="Q23" s="35"/>
+      <c r="R23" s="35"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="39" t="n">
+      <c r="B24" s="41" t="n">
         <v>16</v>
       </c>
-      <c r="C24" s="41" t="n">
+      <c r="C24" s="29" t="n">
         <v>4.55</v>
       </c>
-      <c r="D24" s="41" t="n">
+      <c r="D24" s="29" t="n">
         <v>0.53</v>
       </c>
-      <c r="E24" s="41" t="n">
+      <c r="E24" s="29" t="n">
         <v>0.04</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>181</v>
-      </c>
-      <c r="G24" s="40" t="n">
+        <v>188</v>
+      </c>
+      <c r="G24" s="42" t="n">
         <v>2</v>
       </c>
-      <c r="H24" s="39" t="n">
+      <c r="H24" s="41" t="n">
         <v>300</v>
       </c>
-      <c r="I24" s="39" t="n">
+      <c r="I24" s="41" t="n">
         <v>35</v>
       </c>
-      <c r="J24" s="40" t="n">
+      <c r="J24" s="42" t="n">
         <v>1.4</v>
       </c>
-      <c r="K24" s="40" t="n">
+      <c r="K24" s="42" t="n">
         <v>32.2</v>
       </c>
-      <c r="L24" s="33"/>
-      <c r="M24" s="33"/>
+      <c r="L24" s="35"/>
+      <c r="M24" s="35"/>
       <c r="N24" s="26" t="str">
         <f aca="false">IF(OR(L24="",M24="",$G$5="",$G$6=""),"",(L24/$G$5)/(M24/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O24" s="33"/>
-      <c r="P24" s="33"/>
-      <c r="Q24" s="33"/>
-      <c r="R24" s="33"/>
+      <c r="O24" s="35"/>
+      <c r="P24" s="35"/>
+      <c r="Q24" s="35"/>
+      <c r="R24" s="35"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="39" t="n">
+      <c r="B25" s="41" t="n">
         <v>17</v>
       </c>
-      <c r="C25" s="41" t="n">
+      <c r="C25" s="29" t="n">
         <v>4.55</v>
       </c>
-      <c r="D25" s="41" t="n">
+      <c r="D25" s="29" t="n">
         <v>0.53</v>
       </c>
-      <c r="E25" s="41" t="n">
+      <c r="E25" s="29" t="n">
         <v>0.08</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="G25" s="40" t="n">
+        <v>189</v>
+      </c>
+      <c r="G25" s="42" t="n">
         <v>0.5</v>
       </c>
-      <c r="H25" s="39" t="n">
+      <c r="H25" s="41" t="n">
         <v>300</v>
       </c>
-      <c r="I25" s="39" t="n">
+      <c r="I25" s="41" t="n">
         <v>35</v>
       </c>
-      <c r="J25" s="40" t="n">
+      <c r="J25" s="42" t="n">
         <v>2.8</v>
       </c>
-      <c r="K25" s="40" t="n">
+      <c r="K25" s="42" t="n">
         <v>29.4</v>
       </c>
-      <c r="L25" s="33"/>
-      <c r="M25" s="33"/>
+      <c r="L25" s="35"/>
+      <c r="M25" s="35"/>
       <c r="N25" s="26" t="str">
         <f aca="false">IF(OR(L25="",M25="",$G$5="",$G$6=""),"",(L25/$G$5)/(M25/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O25" s="33"/>
-      <c r="P25" s="33"/>
-      <c r="Q25" s="33"/>
-      <c r="R25" s="33"/>
+      <c r="O25" s="35"/>
+      <c r="P25" s="35"/>
+      <c r="Q25" s="35"/>
+      <c r="R25" s="35"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="39" t="n">
+      <c r="B26" s="41" t="n">
         <v>18</v>
       </c>
-      <c r="C26" s="41" t="n">
+      <c r="C26" s="29" t="n">
         <v>4.55</v>
       </c>
-      <c r="D26" s="41" t="n">
+      <c r="D26" s="29" t="n">
         <v>0.53</v>
       </c>
-      <c r="E26" s="41" t="n">
+      <c r="E26" s="29" t="n">
         <v>0.12</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>183</v>
-      </c>
-      <c r="G26" s="40" t="n">
+        <v>190</v>
+      </c>
+      <c r="G26" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="H26" s="39" t="n">
+      <c r="H26" s="41" t="n">
         <v>300</v>
       </c>
-      <c r="I26" s="39" t="n">
+      <c r="I26" s="41" t="n">
         <v>35</v>
       </c>
-      <c r="J26" s="40" t="n">
+      <c r="J26" s="42" t="n">
         <v>4.2</v>
       </c>
-      <c r="K26" s="40" t="n">
+      <c r="K26" s="42" t="n">
         <v>26.6</v>
       </c>
-      <c r="L26" s="33"/>
-      <c r="M26" s="33"/>
+      <c r="L26" s="35"/>
+      <c r="M26" s="35"/>
       <c r="N26" s="26" t="str">
         <f aca="false">IF(OR(L26="",M26="",$G$5="",$G$6=""),"",(L26/$G$5)/(M26/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O26" s="33"/>
-      <c r="P26" s="33"/>
-      <c r="Q26" s="33"/>
-      <c r="R26" s="33"/>
+      <c r="O26" s="35"/>
+      <c r="P26" s="35"/>
+      <c r="Q26" s="35"/>
+      <c r="R26" s="35"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="39" t="n">
+      <c r="B27" s="41" t="n">
         <v>19</v>
       </c>
-      <c r="C27" s="41" t="n">
+      <c r="C27" s="29" t="n">
         <v>6.06</v>
       </c>
-      <c r="D27" s="41" t="n">
+      <c r="D27" s="29" t="n">
         <v>0.23</v>
       </c>
-      <c r="E27" s="41" t="n">
+      <c r="E27" s="29" t="n">
         <v>0.04</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>183</v>
-      </c>
-      <c r="G27" s="40" t="n">
+        <v>190</v>
+      </c>
+      <c r="G27" s="42" t="n">
         <v>2</v>
       </c>
-      <c r="H27" s="39" t="n">
+      <c r="H27" s="41" t="n">
         <v>400</v>
       </c>
-      <c r="I27" s="39" t="n">
+      <c r="I27" s="41" t="n">
         <v>15</v>
       </c>
-      <c r="J27" s="40" t="n">
+      <c r="J27" s="42" t="n">
         <v>0.6</v>
       </c>
-      <c r="K27" s="40" t="n">
+      <c r="K27" s="42" t="n">
         <v>13.8</v>
       </c>
-      <c r="L27" s="33"/>
-      <c r="M27" s="33"/>
+      <c r="L27" s="35"/>
+      <c r="M27" s="35"/>
       <c r="N27" s="26" t="str">
         <f aca="false">IF(OR(L27="",M27="",$G$5="",$G$6=""),"",(L27/$G$5)/(M27/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O27" s="33"/>
-      <c r="P27" s="33"/>
-      <c r="Q27" s="33"/>
-      <c r="R27" s="33"/>
+      <c r="O27" s="35"/>
+      <c r="P27" s="35"/>
+      <c r="Q27" s="35"/>
+      <c r="R27" s="35"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="39" t="n">
+      <c r="B28" s="41" t="n">
         <v>20</v>
       </c>
-      <c r="C28" s="41" t="n">
+      <c r="C28" s="29" t="n">
         <v>6.06</v>
       </c>
-      <c r="D28" s="41" t="n">
+      <c r="D28" s="29" t="n">
         <v>0.23</v>
       </c>
-      <c r="E28" s="41" t="n">
+      <c r="E28" s="29" t="n">
         <v>0.08</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>181</v>
-      </c>
-      <c r="G28" s="40" t="n">
+        <v>188</v>
+      </c>
+      <c r="G28" s="42" t="n">
         <v>0.5</v>
       </c>
-      <c r="H28" s="39" t="n">
+      <c r="H28" s="41" t="n">
         <v>400</v>
       </c>
-      <c r="I28" s="39" t="n">
+      <c r="I28" s="41" t="n">
         <v>15</v>
       </c>
-      <c r="J28" s="40" t="n">
+      <c r="J28" s="42" t="n">
         <v>1.2</v>
       </c>
-      <c r="K28" s="40" t="n">
+      <c r="K28" s="42" t="n">
         <v>12.6</v>
       </c>
-      <c r="L28" s="33"/>
-      <c r="M28" s="33"/>
+      <c r="L28" s="35"/>
+      <c r="M28" s="35"/>
       <c r="N28" s="26" t="str">
         <f aca="false">IF(OR(L28="",M28="",$G$5="",$G$6=""),"",(L28/$G$5)/(M28/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O28" s="33"/>
-      <c r="P28" s="33"/>
-      <c r="Q28" s="33"/>
-      <c r="R28" s="33"/>
+      <c r="O28" s="35"/>
+      <c r="P28" s="35"/>
+      <c r="Q28" s="35"/>
+      <c r="R28" s="35"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="39" t="n">
+      <c r="B29" s="41" t="n">
         <v>21</v>
       </c>
-      <c r="C29" s="41" t="n">
+      <c r="C29" s="29" t="n">
         <v>6.06</v>
       </c>
-      <c r="D29" s="41" t="n">
+      <c r="D29" s="29" t="n">
         <v>0.23</v>
       </c>
-      <c r="E29" s="41" t="n">
+      <c r="E29" s="29" t="n">
         <v>0.12</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="G29" s="40" t="n">
+        <v>189</v>
+      </c>
+      <c r="G29" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="H29" s="39" t="n">
+      <c r="H29" s="41" t="n">
         <v>400</v>
       </c>
-      <c r="I29" s="39" t="n">
+      <c r="I29" s="41" t="n">
         <v>15</v>
       </c>
-      <c r="J29" s="40" t="n">
+      <c r="J29" s="42" t="n">
         <v>1.8</v>
       </c>
-      <c r="K29" s="40" t="n">
+      <c r="K29" s="42" t="n">
         <v>11.4</v>
       </c>
-      <c r="L29" s="33"/>
-      <c r="M29" s="33"/>
+      <c r="L29" s="35"/>
+      <c r="M29" s="35"/>
       <c r="N29" s="26" t="str">
         <f aca="false">IF(OR(L29="",M29="",$G$5="",$G$6=""),"",(L29/$G$5)/(M29/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O29" s="33"/>
-      <c r="P29" s="33"/>
-      <c r="Q29" s="33"/>
-      <c r="R29" s="33"/>
+      <c r="O29" s="35"/>
+      <c r="P29" s="35"/>
+      <c r="Q29" s="35"/>
+      <c r="R29" s="35"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="39" t="n">
+      <c r="B30" s="41" t="n">
         <v>22</v>
       </c>
-      <c r="C30" s="41" t="n">
+      <c r="C30" s="29" t="n">
         <v>6.06</v>
       </c>
-      <c r="D30" s="41" t="n">
+      <c r="D30" s="29" t="n">
         <v>0.38</v>
       </c>
-      <c r="E30" s="41" t="n">
+      <c r="E30" s="29" t="n">
         <v>0.04</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>181</v>
-      </c>
-      <c r="G30" s="40" t="n">
+        <v>188</v>
+      </c>
+      <c r="G30" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="H30" s="39" t="n">
+      <c r="H30" s="41" t="n">
         <v>400</v>
       </c>
-      <c r="I30" s="39" t="n">
+      <c r="I30" s="41" t="n">
         <v>25</v>
       </c>
-      <c r="J30" s="40" t="n">
+      <c r="J30" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="K30" s="40" t="n">
+      <c r="K30" s="42" t="n">
         <v>23</v>
       </c>
-      <c r="L30" s="33"/>
-      <c r="M30" s="33"/>
+      <c r="L30" s="35"/>
+      <c r="M30" s="35"/>
       <c r="N30" s="26" t="str">
         <f aca="false">IF(OR(L30="",M30="",$G$5="",$G$6=""),"",(L30/$G$5)/(M30/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O30" s="33"/>
-      <c r="P30" s="33"/>
-      <c r="Q30" s="33"/>
-      <c r="R30" s="33"/>
+      <c r="O30" s="35"/>
+      <c r="P30" s="35"/>
+      <c r="Q30" s="35"/>
+      <c r="R30" s="35"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="39" t="n">
+      <c r="B31" s="41" t="n">
         <v>23</v>
       </c>
-      <c r="C31" s="41" t="n">
+      <c r="C31" s="29" t="n">
         <v>6.06</v>
       </c>
-      <c r="D31" s="41" t="n">
+      <c r="D31" s="29" t="n">
         <v>0.38</v>
       </c>
-      <c r="E31" s="41" t="n">
+      <c r="E31" s="29" t="n">
         <v>0.08</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="G31" s="40" t="n">
+        <v>189</v>
+      </c>
+      <c r="G31" s="42" t="n">
         <v>2</v>
       </c>
-      <c r="H31" s="39" t="n">
+      <c r="H31" s="41" t="n">
         <v>400</v>
       </c>
-      <c r="I31" s="39" t="n">
+      <c r="I31" s="41" t="n">
         <v>25</v>
       </c>
-      <c r="J31" s="40" t="n">
+      <c r="J31" s="42" t="n">
         <v>2</v>
       </c>
-      <c r="K31" s="40" t="n">
+      <c r="K31" s="42" t="n">
         <v>21</v>
       </c>
-      <c r="L31" s="33"/>
-      <c r="M31" s="33"/>
+      <c r="L31" s="35"/>
+      <c r="M31" s="35"/>
       <c r="N31" s="26" t="str">
         <f aca="false">IF(OR(L31="",M31="",$G$5="",$G$6=""),"",(L31/$G$5)/(M31/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O31" s="33"/>
-      <c r="P31" s="33"/>
-      <c r="Q31" s="33"/>
-      <c r="R31" s="33"/>
+      <c r="O31" s="35"/>
+      <c r="P31" s="35"/>
+      <c r="Q31" s="35"/>
+      <c r="R31" s="35"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="39" t="n">
+      <c r="B32" s="41" t="n">
         <v>24</v>
       </c>
-      <c r="C32" s="41" t="n">
+      <c r="C32" s="29" t="n">
         <v>6.06</v>
       </c>
-      <c r="D32" s="41" t="n">
+      <c r="D32" s="29" t="n">
         <v>0.38</v>
       </c>
-      <c r="E32" s="41" t="n">
+      <c r="E32" s="29" t="n">
         <v>0.12</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>183</v>
-      </c>
-      <c r="G32" s="40" t="n">
+        <v>190</v>
+      </c>
+      <c r="G32" s="42" t="n">
         <v>0.5</v>
       </c>
-      <c r="H32" s="39" t="n">
+      <c r="H32" s="41" t="n">
         <v>400</v>
       </c>
-      <c r="I32" s="39" t="n">
+      <c r="I32" s="41" t="n">
         <v>25</v>
       </c>
-      <c r="J32" s="40" t="n">
+      <c r="J32" s="42" t="n">
         <v>3</v>
       </c>
-      <c r="K32" s="40" t="n">
+      <c r="K32" s="42" t="n">
         <v>19</v>
       </c>
-      <c r="L32" s="33"/>
-      <c r="M32" s="33"/>
+      <c r="L32" s="35"/>
+      <c r="M32" s="35"/>
       <c r="N32" s="26" t="str">
         <f aca="false">IF(OR(L32="",M32="",$G$5="",$G$6=""),"",(L32/$G$5)/(M32/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O32" s="33"/>
-      <c r="P32" s="33"/>
-      <c r="Q32" s="33"/>
-      <c r="R32" s="33"/>
+      <c r="O32" s="35"/>
+      <c r="P32" s="35"/>
+      <c r="Q32" s="35"/>
+      <c r="R32" s="35"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="39" t="n">
+      <c r="B33" s="41" t="n">
         <v>25</v>
       </c>
-      <c r="C33" s="41" t="n">
+      <c r="C33" s="29" t="n">
         <v>6.06</v>
       </c>
-      <c r="D33" s="41" t="n">
+      <c r="D33" s="29" t="n">
         <v>0.53</v>
       </c>
-      <c r="E33" s="41" t="n">
+      <c r="E33" s="29" t="n">
         <v>0.04</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="G33" s="40" t="n">
+        <v>189</v>
+      </c>
+      <c r="G33" s="42" t="n">
         <v>0.5</v>
       </c>
-      <c r="H33" s="39" t="n">
+      <c r="H33" s="41" t="n">
         <v>400</v>
       </c>
-      <c r="I33" s="39" t="n">
+      <c r="I33" s="41" t="n">
         <v>35</v>
       </c>
-      <c r="J33" s="40" t="n">
+      <c r="J33" s="42" t="n">
         <v>1.4</v>
       </c>
-      <c r="K33" s="40" t="n">
+      <c r="K33" s="42" t="n">
         <v>32.2</v>
       </c>
-      <c r="L33" s="33"/>
-      <c r="M33" s="33"/>
+      <c r="L33" s="35"/>
+      <c r="M33" s="35"/>
       <c r="N33" s="26" t="str">
         <f aca="false">IF(OR(L33="",M33="",$G$5="",$G$6=""),"",(L33/$G$5)/(M33/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O33" s="33"/>
-      <c r="P33" s="33"/>
-      <c r="Q33" s="33"/>
-      <c r="R33" s="33"/>
+      <c r="O33" s="35"/>
+      <c r="P33" s="35"/>
+      <c r="Q33" s="35"/>
+      <c r="R33" s="35"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="39" t="n">
+      <c r="B34" s="41" t="n">
         <v>26</v>
       </c>
-      <c r="C34" s="41" t="n">
+      <c r="C34" s="29" t="n">
         <v>6.06</v>
       </c>
-      <c r="D34" s="41" t="n">
+      <c r="D34" s="29" t="n">
         <v>0.53</v>
       </c>
-      <c r="E34" s="41" t="n">
+      <c r="E34" s="29" t="n">
         <v>0.08</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>183</v>
-      </c>
-      <c r="G34" s="40" t="n">
+        <v>190</v>
+      </c>
+      <c r="G34" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="H34" s="39" t="n">
+      <c r="H34" s="41" t="n">
         <v>400</v>
       </c>
-      <c r="I34" s="39" t="n">
+      <c r="I34" s="41" t="n">
         <v>35</v>
       </c>
-      <c r="J34" s="40" t="n">
+      <c r="J34" s="42" t="n">
         <v>2.8</v>
       </c>
-      <c r="K34" s="40" t="n">
+      <c r="K34" s="42" t="n">
         <v>29.4</v>
       </c>
-      <c r="L34" s="33"/>
-      <c r="M34" s="33"/>
+      <c r="L34" s="35"/>
+      <c r="M34" s="35"/>
       <c r="N34" s="26" t="str">
         <f aca="false">IF(OR(L34="",M34="",$G$5="",$G$6=""),"",(L34/$G$5)/(M34/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O34" s="33"/>
-      <c r="P34" s="33"/>
-      <c r="Q34" s="33"/>
-      <c r="R34" s="33"/>
+      <c r="O34" s="35"/>
+      <c r="P34" s="35"/>
+      <c r="Q34" s="35"/>
+      <c r="R34" s="35"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="39" t="n">
+      <c r="B35" s="41" t="n">
         <v>27</v>
       </c>
-      <c r="C35" s="41" t="n">
+      <c r="C35" s="29" t="n">
         <v>6.06</v>
       </c>
-      <c r="D35" s="41" t="n">
+      <c r="D35" s="29" t="n">
         <v>0.53</v>
       </c>
-      <c r="E35" s="41" t="n">
+      <c r="E35" s="29" t="n">
         <v>0.12</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>181</v>
-      </c>
-      <c r="G35" s="40" t="n">
+        <v>188</v>
+      </c>
+      <c r="G35" s="42" t="n">
         <v>2</v>
       </c>
-      <c r="H35" s="39" t="n">
+      <c r="H35" s="41" t="n">
         <v>400</v>
       </c>
-      <c r="I35" s="39" t="n">
+      <c r="I35" s="41" t="n">
         <v>35</v>
       </c>
-      <c r="J35" s="40" t="n">
+      <c r="J35" s="42" t="n">
         <v>4.2</v>
       </c>
-      <c r="K35" s="40" t="n">
+      <c r="K35" s="42" t="n">
         <v>26.6</v>
       </c>
-      <c r="L35" s="33"/>
-      <c r="M35" s="33"/>
+      <c r="L35" s="35"/>
+      <c r="M35" s="35"/>
       <c r="N35" s="26" t="str">
         <f aca="false">IF(OR(L35="",M35="",$G$5="",$G$6=""),"",(L35/$G$5)/(M35/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O35" s="33"/>
-      <c r="P35" s="33"/>
-      <c r="Q35" s="33"/>
-      <c r="R35" s="33"/>
+      <c r="O35" s="35"/>
+      <c r="P35" s="35"/>
+      <c r="Q35" s="35"/>
+      <c r="R35" s="35"/>
     </row>
     <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="12" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="C37" s="12"/>
       <c r="D37" s="12"/>

</xml_diff>

<commit_message>
Add Results Calculator sheet: single place to compute h, Nu, dP, f
New "Results Calculator" sheet holds one row per Fluent run (3 GCI
mesh levels + 8 Correlation Validation Re points). Paste T_out,
T_wall, p_in, p_out once per row; V, Tb, h, Nu, dP, f compute there.
GCI sheet and Correlation Validation sheet now link their Nu/f from
this table instead of duplicating the raw-to-derived formula chain,
so raw Fluent numbers are entered in exactly one place.

Moved the existing Coarse mesh result (Nu=511.69, f=0.01723) into
its new home at Results Calculator row 8.
</commit_message>
<xml_diff>
--- a/thesis/mesh-validation/Mesh_and_Validation_Workbook.xlsx
+++ b/thesis/mesh-validation/Mesh_and_Validation_Workbook.xlsx
@@ -13,10 +13,11 @@
     <sheet name="Fluid Properties" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="YPlus Inflation" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Mesh Levels" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Correlation Validation" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="GCI Mesh Independence" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="Dudley D1 Validation" sheetId="8" state="visible" r:id="rId10"/>
-    <sheet name="L27 Run Log" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="Results Calculator" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Correlation Validation" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="GCI Mesh Independence" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Dudley D1 Validation" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="L27 Run Log" sheetId="10" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="234">
   <si>
     <t xml:space="preserve">PTSC-HTSP Thesis — Meshing &amp; Validation Workbook</t>
   </si>
@@ -402,10 +403,100 @@
     <t xml:space="preserve">What to change between levels: circumferential divisions, core-block radial divisions, and axial divisions (rows above) -- these control the mesh away from the wall. What must stay fixed: first-layer height, growth rate, number of inflation layers (blue-shaded block above) -- these are a physics requirement (y+), not a discretisation choice. In ANSYS Meshing this maps to: change the Sizing/Method divisions per level; leave the Inflation control's 'First Layer Thickness', 'Growth Rate' and 'Number of Layers' identical in all three.</t>
   </si>
   <si>
+    <t xml:space="preserve">Results Calculator -- one place for h, Nu, dP, f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One row per Fluent run. Paste T_out, T_wall, p_in, p_out here from your Report Definitions (Compute button) -- V, Tb, h, Nu, dP and f compute automatically. The GCI sheet and Correlation Validation sheet both read their Nu/f from this table, so you only enter raw numbers once, here.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q''
+(W/m2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T_out (K)
+PASTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T_wall (K)
+PASTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p_in (Pa)
+PASTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p_out (Pa)
+PASTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V
+(m/s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tb
+(K)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">h
+(W/m2K)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dP
+(Pa)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GCI -- Fine mesh (Re=100,000 design point)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GCI -- Medium mesh (Re=100,000 design point)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GCI -- Coarse mesh (Re=100,000 design point)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correlation Validation Re sweep (Tin = 500K design point held fixed for every point)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correlation Validation -- Re=5,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correlation Validation -- Re=7,500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correlation Validation -- Re=10,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correlation Validation -- Re=20,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correlation Validation -- Re=30,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correlation Validation -- Re=50,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correlation Validation -- Re=70,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correlation Validation -- Re=100,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q'' pulls from the single wall-heat-flux input on the GCI sheet -- keep it identical across every run. V = Re . nu / D (kinematic viscosity, Fluid Properties sheet). f uses this row's own V, so it is correct at every Re, not just the Re=100,000 GCI design point.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Smooth-Tube Validation vs Gnielinski / Petukhov</t>
   </si>
   <si>
-    <t xml:space="preserve">Yellow cells: paste your Fluent results here after each run, at the matching Re. Deviation % and PASS/FAIL compute automatically against the thresholds in your solver_and_formulas.md (Nu &lt;= 9%, f &lt;= 5%).</t>
+    <t xml:space="preserve">Nu CFD and f CFD pull automatically from the Results Calculator sheet (enter your raw T_out/T_wall/p_in/p_out there, per Re). Deviation % and PASS/FAIL compute automatically against the thresholds in your solver_and_formulas.md (Nu &lt;= 9%, f &lt;= 5%).</t>
   </si>
   <si>
     <t xml:space="preserve">f Petukhov
@@ -442,13 +533,13 @@
     <t xml:space="preserve">Grid Convergence Index (Celik et al. 2008)</t>
   </si>
   <si>
-    <t xml:space="preserve">Run your smooth-tube geometry at ALL THREE mesh levels (Mesh Levels sheet), at ONE fixed Re (recommended: 100,000, your y+ design point). Paste the resulting Nu and f into the yellow cells. Everything else computes automatically.</t>
+    <t xml:space="preserve">Run your smooth-tube geometry at ALL THREE mesh levels (Mesh Levels sheet), at ONE fixed Re (recommended: 100,000, your y+ design point). Enter your raw T_out/T_wall/p_in/p_out on the Results Calculator sheet (rows 6-8) -- everything below pulls from there automatically.</t>
   </si>
   <si>
     <t xml:space="preserve">Validation Re used for this mesh-independence study</t>
   </si>
   <si>
-    <t xml:space="preserve">Raw Fluent Extraction (paste report values here -- Nu and f below compute automatically)</t>
+    <t xml:space="preserve">Raw Fluent Extraction (linked from Results Calculator -- enter raw numbers there, rows 6-8)</t>
   </si>
   <si>
     <t xml:space="preserve">Wall heat flux, q'' (W/m²) -- must match your Fluent Wall BC, same for every mesh level</t>
@@ -463,16 +554,16 @@
     <t xml:space="preserve">Coarse (3)</t>
   </si>
   <si>
-    <t xml:space="preserve">Outlet bulk temperature, T_out (K)  --  PASTE from Fluent t_out report</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wall temperature, T_wall (K)  --  PASTE from Fluent t_wall report</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inlet pressure, p_in (Pa)  --  PASTE from Fluent p_inlet report</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Outlet pressure, p_out (Pa)  --  PASTE from Fluent p_out report</t>
+    <t xml:space="preserve">Outlet bulk temperature, T_out (K)  --  linked from Results Calculator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wall temperature, T_wall (K)  --  linked from Results Calculator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inlet pressure, p_in (Pa)  --  linked from Results Calculator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outlet pressure, p_out (Pa)  --  linked from Results Calculator</t>
   </si>
   <si>
     <t xml:space="preserve">Bulk temperature, Tb = (T_in + T_out) / 2  (K)</t>
@@ -494,12 +585,6 @@
   </si>
   <si>
     <t xml:space="preserve">Mesh Comparison Summary -- Nu and f across mesh levels (this is where you see the difference)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">f</t>
   </si>
   <si>
     <t xml:space="preserve">% change in Nu, Fine -&gt; Medium  /  Medium -&gt; Coarse</t>
@@ -617,9 +702,6 @@
   </si>
   <si>
     <t xml:space="preserve">Plain-tube reference f_plain (same Re as production runs, fill in after validation)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Run</t>
   </si>
   <si>
     <t xml:space="preserve">A
@@ -890,7 +972,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="50">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1031,7 +1113,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1047,23 +1145,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="174" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="174" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="175" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="175" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1072,6 +1162,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="176" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1505,6 +1599,1298 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="B2:R37"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="8" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="12" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="3"/>
+  </cols>
+  <sheetData>
+    <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B3" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="12"/>
+      <c r="L3" s="12"/>
+      <c r="M3" s="12"/>
+      <c r="N3" s="12"/>
+      <c r="O3" s="12"/>
+      <c r="P3" s="12"/>
+      <c r="Q3" s="12"/>
+      <c r="R3" s="12"/>
+    </row>
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="49" t="s">
+        <v>212</v>
+      </c>
+      <c r="C5" s="49"/>
+      <c r="D5" s="49"/>
+      <c r="E5" s="49"/>
+      <c r="F5" s="49"/>
+      <c r="G5" s="48"/>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="49" t="s">
+        <v>213</v>
+      </c>
+      <c r="C6" s="49"/>
+      <c r="D6" s="49"/>
+      <c r="E6" s="49"/>
+      <c r="F6" s="49"/>
+      <c r="G6" s="48"/>
+    </row>
+    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="L8" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="M8" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="N8" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="O8" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="P8" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="Q8" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="R8" s="6" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="29" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="D9" s="29" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="E9" s="29" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="G9" s="47" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H9" s="42" t="n">
+        <v>200</v>
+      </c>
+      <c r="I9" s="42" t="n">
+        <v>15</v>
+      </c>
+      <c r="J9" s="47" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K9" s="47" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="L9" s="48"/>
+      <c r="M9" s="48"/>
+      <c r="N9" s="26" t="str">
+        <f aca="false">IF(OR(L9="",M9="",$G$5="",$G$6=""),"",(L9/$G$5)/(M9/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O9" s="48"/>
+      <c r="P9" s="48"/>
+      <c r="Q9" s="48"/>
+      <c r="R9" s="48"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="42" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" s="29" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="D10" s="29" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="E10" s="29" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="G10" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="42" t="n">
+        <v>200</v>
+      </c>
+      <c r="I10" s="42" t="n">
+        <v>15</v>
+      </c>
+      <c r="J10" s="47" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="K10" s="47" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="L10" s="48"/>
+      <c r="M10" s="48"/>
+      <c r="N10" s="26" t="str">
+        <f aca="false">IF(OR(L10="",M10="",$G$5="",$G$6=""),"",(L10/$G$5)/(M10/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O10" s="48"/>
+      <c r="P10" s="48"/>
+      <c r="Q10" s="48"/>
+      <c r="R10" s="48"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" s="29" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="D11" s="29" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="E11" s="29" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="G11" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" s="42" t="n">
+        <v>200</v>
+      </c>
+      <c r="I11" s="42" t="n">
+        <v>15</v>
+      </c>
+      <c r="J11" s="47" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="K11" s="47" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="L11" s="48"/>
+      <c r="M11" s="48"/>
+      <c r="N11" s="26" t="str">
+        <f aca="false">IF(OR(L11="",M11="",$G$5="",$G$6=""),"",(L11/$G$5)/(M11/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O11" s="48"/>
+      <c r="P11" s="48"/>
+      <c r="Q11" s="48"/>
+      <c r="R11" s="48"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="42" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" s="29" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="D12" s="29" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="E12" s="29" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="G12" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="H12" s="42" t="n">
+        <v>200</v>
+      </c>
+      <c r="I12" s="42" t="n">
+        <v>25</v>
+      </c>
+      <c r="J12" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="47" t="n">
+        <v>23</v>
+      </c>
+      <c r="L12" s="48"/>
+      <c r="M12" s="48"/>
+      <c r="N12" s="26" t="str">
+        <f aca="false">IF(OR(L12="",M12="",$G$5="",$G$6=""),"",(L12/$G$5)/(M12/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O12" s="48"/>
+      <c r="P12" s="48"/>
+      <c r="Q12" s="48"/>
+      <c r="R12" s="48"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="42" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" s="29" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="D13" s="29" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="E13" s="29" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="G13" s="47" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H13" s="42" t="n">
+        <v>200</v>
+      </c>
+      <c r="I13" s="42" t="n">
+        <v>25</v>
+      </c>
+      <c r="J13" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="K13" s="47" t="n">
+        <v>21</v>
+      </c>
+      <c r="L13" s="48"/>
+      <c r="M13" s="48"/>
+      <c r="N13" s="26" t="str">
+        <f aca="false">IF(OR(L13="",M13="",$G$5="",$G$6=""),"",(L13/$G$5)/(M13/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O13" s="48"/>
+      <c r="P13" s="48"/>
+      <c r="Q13" s="48"/>
+      <c r="R13" s="48"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="42" t="n">
+        <v>6</v>
+      </c>
+      <c r="C14" s="29" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="D14" s="29" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="E14" s="29" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="G14" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="42" t="n">
+        <v>200</v>
+      </c>
+      <c r="I14" s="42" t="n">
+        <v>25</v>
+      </c>
+      <c r="J14" s="47" t="n">
+        <v>3</v>
+      </c>
+      <c r="K14" s="47" t="n">
+        <v>19</v>
+      </c>
+      <c r="L14" s="48"/>
+      <c r="M14" s="48"/>
+      <c r="N14" s="26" t="str">
+        <f aca="false">IF(OR(L14="",M14="",$G$5="",$G$6=""),"",(L14/$G$5)/(M14/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O14" s="48"/>
+      <c r="P14" s="48"/>
+      <c r="Q14" s="48"/>
+      <c r="R14" s="48"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="42" t="n">
+        <v>7</v>
+      </c>
+      <c r="C15" s="29" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="D15" s="29" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="E15" s="29" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="G15" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="42" t="n">
+        <v>200</v>
+      </c>
+      <c r="I15" s="42" t="n">
+        <v>35</v>
+      </c>
+      <c r="J15" s="47" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="K15" s="47" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="L15" s="48"/>
+      <c r="M15" s="48"/>
+      <c r="N15" s="26" t="str">
+        <f aca="false">IF(OR(L15="",M15="",$G$5="",$G$6=""),"",(L15/$G$5)/(M15/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O15" s="48"/>
+      <c r="P15" s="48"/>
+      <c r="Q15" s="48"/>
+      <c r="R15" s="48"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="42" t="n">
+        <v>8</v>
+      </c>
+      <c r="C16" s="29" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="D16" s="29" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="E16" s="29" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="G16" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="H16" s="42" t="n">
+        <v>200</v>
+      </c>
+      <c r="I16" s="42" t="n">
+        <v>35</v>
+      </c>
+      <c r="J16" s="47" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K16" s="47" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="L16" s="48"/>
+      <c r="M16" s="48"/>
+      <c r="N16" s="26" t="str">
+        <f aca="false">IF(OR(L16="",M16="",$G$5="",$G$6=""),"",(L16/$G$5)/(M16/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O16" s="48"/>
+      <c r="P16" s="48"/>
+      <c r="Q16" s="48"/>
+      <c r="R16" s="48"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="42" t="n">
+        <v>9</v>
+      </c>
+      <c r="C17" s="29" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="D17" s="29" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="E17" s="29" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="G17" s="47" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H17" s="42" t="n">
+        <v>200</v>
+      </c>
+      <c r="I17" s="42" t="n">
+        <v>35</v>
+      </c>
+      <c r="J17" s="47" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="K17" s="47" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="L17" s="48"/>
+      <c r="M17" s="48"/>
+      <c r="N17" s="26" t="str">
+        <f aca="false">IF(OR(L17="",M17="",$G$5="",$G$6=""),"",(L17/$G$5)/(M17/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O17" s="48"/>
+      <c r="P17" s="48"/>
+      <c r="Q17" s="48"/>
+      <c r="R17" s="48"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="42" t="n">
+        <v>10</v>
+      </c>
+      <c r="C18" s="29" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="D18" s="29" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="E18" s="29" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="G18" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="42" t="n">
+        <v>300</v>
+      </c>
+      <c r="I18" s="42" t="n">
+        <v>15</v>
+      </c>
+      <c r="J18" s="47" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K18" s="47" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="L18" s="48"/>
+      <c r="M18" s="48"/>
+      <c r="N18" s="26" t="str">
+        <f aca="false">IF(OR(L18="",M18="",$G$5="",$G$6=""),"",(L18/$G$5)/(M18/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O18" s="48"/>
+      <c r="P18" s="48"/>
+      <c r="Q18" s="48"/>
+      <c r="R18" s="48"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="42" t="n">
+        <v>11</v>
+      </c>
+      <c r="C19" s="29" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="D19" s="29" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="E19" s="29" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="G19" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="H19" s="42" t="n">
+        <v>300</v>
+      </c>
+      <c r="I19" s="42" t="n">
+        <v>15</v>
+      </c>
+      <c r="J19" s="47" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="K19" s="47" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="L19" s="48"/>
+      <c r="M19" s="48"/>
+      <c r="N19" s="26" t="str">
+        <f aca="false">IF(OR(L19="",M19="",$G$5="",$G$6=""),"",(L19/$G$5)/(M19/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O19" s="48"/>
+      <c r="P19" s="48"/>
+      <c r="Q19" s="48"/>
+      <c r="R19" s="48"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="42" t="n">
+        <v>12</v>
+      </c>
+      <c r="C20" s="29" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="D20" s="29" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="E20" s="29" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="G20" s="47" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H20" s="42" t="n">
+        <v>300</v>
+      </c>
+      <c r="I20" s="42" t="n">
+        <v>15</v>
+      </c>
+      <c r="J20" s="47" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="K20" s="47" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="L20" s="48"/>
+      <c r="M20" s="48"/>
+      <c r="N20" s="26" t="str">
+        <f aca="false">IF(OR(L20="",M20="",$G$5="",$G$6=""),"",(L20/$G$5)/(M20/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O20" s="48"/>
+      <c r="P20" s="48"/>
+      <c r="Q20" s="48"/>
+      <c r="R20" s="48"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="42" t="n">
+        <v>13</v>
+      </c>
+      <c r="C21" s="29" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="D21" s="29" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="E21" s="29" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F21" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="G21" s="47" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H21" s="42" t="n">
+        <v>300</v>
+      </c>
+      <c r="I21" s="42" t="n">
+        <v>25</v>
+      </c>
+      <c r="J21" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="47" t="n">
+        <v>23</v>
+      </c>
+      <c r="L21" s="48"/>
+      <c r="M21" s="48"/>
+      <c r="N21" s="26" t="str">
+        <f aca="false">IF(OR(L21="",M21="",$G$5="",$G$6=""),"",(L21/$G$5)/(M21/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O21" s="48"/>
+      <c r="P21" s="48"/>
+      <c r="Q21" s="48"/>
+      <c r="R21" s="48"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="42" t="n">
+        <v>14</v>
+      </c>
+      <c r="C22" s="29" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="D22" s="29" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="E22" s="29" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F22" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="G22" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="42" t="n">
+        <v>300</v>
+      </c>
+      <c r="I22" s="42" t="n">
+        <v>25</v>
+      </c>
+      <c r="J22" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="K22" s="47" t="n">
+        <v>21</v>
+      </c>
+      <c r="L22" s="48"/>
+      <c r="M22" s="48"/>
+      <c r="N22" s="26" t="str">
+        <f aca="false">IF(OR(L22="",M22="",$G$5="",$G$6=""),"",(L22/$G$5)/(M22/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O22" s="48"/>
+      <c r="P22" s="48"/>
+      <c r="Q22" s="48"/>
+      <c r="R22" s="48"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="42" t="n">
+        <v>15</v>
+      </c>
+      <c r="C23" s="29" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="D23" s="29" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="E23" s="29" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F23" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="G23" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="H23" s="42" t="n">
+        <v>300</v>
+      </c>
+      <c r="I23" s="42" t="n">
+        <v>25</v>
+      </c>
+      <c r="J23" s="47" t="n">
+        <v>3</v>
+      </c>
+      <c r="K23" s="47" t="n">
+        <v>19</v>
+      </c>
+      <c r="L23" s="48"/>
+      <c r="M23" s="48"/>
+      <c r="N23" s="26" t="str">
+        <f aca="false">IF(OR(L23="",M23="",$G$5="",$G$6=""),"",(L23/$G$5)/(M23/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O23" s="48"/>
+      <c r="P23" s="48"/>
+      <c r="Q23" s="48"/>
+      <c r="R23" s="48"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="42" t="n">
+        <v>16</v>
+      </c>
+      <c r="C24" s="29" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="D24" s="29" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="E24" s="29" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="G24" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="H24" s="42" t="n">
+        <v>300</v>
+      </c>
+      <c r="I24" s="42" t="n">
+        <v>35</v>
+      </c>
+      <c r="J24" s="47" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="K24" s="47" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="L24" s="48"/>
+      <c r="M24" s="48"/>
+      <c r="N24" s="26" t="str">
+        <f aca="false">IF(OR(L24="",M24="",$G$5="",$G$6=""),"",(L24/$G$5)/(M24/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O24" s="48"/>
+      <c r="P24" s="48"/>
+      <c r="Q24" s="48"/>
+      <c r="R24" s="48"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="42" t="n">
+        <v>17</v>
+      </c>
+      <c r="C25" s="29" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="D25" s="29" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="E25" s="29" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F25" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="G25" s="47" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H25" s="42" t="n">
+        <v>300</v>
+      </c>
+      <c r="I25" s="42" t="n">
+        <v>35</v>
+      </c>
+      <c r="J25" s="47" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K25" s="47" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="L25" s="48"/>
+      <c r="M25" s="48"/>
+      <c r="N25" s="26" t="str">
+        <f aca="false">IF(OR(L25="",M25="",$G$5="",$G$6=""),"",(L25/$G$5)/(M25/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O25" s="48"/>
+      <c r="P25" s="48"/>
+      <c r="Q25" s="48"/>
+      <c r="R25" s="48"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="42" t="n">
+        <v>18</v>
+      </c>
+      <c r="C26" s="29" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="D26" s="29" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="E26" s="29" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F26" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="G26" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" s="42" t="n">
+        <v>300</v>
+      </c>
+      <c r="I26" s="42" t="n">
+        <v>35</v>
+      </c>
+      <c r="J26" s="47" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="K26" s="47" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="L26" s="48"/>
+      <c r="M26" s="48"/>
+      <c r="N26" s="26" t="str">
+        <f aca="false">IF(OR(L26="",M26="",$G$5="",$G$6=""),"",(L26/$G$5)/(M26/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O26" s="48"/>
+      <c r="P26" s="48"/>
+      <c r="Q26" s="48"/>
+      <c r="R26" s="48"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="42" t="n">
+        <v>19</v>
+      </c>
+      <c r="C27" s="29" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="D27" s="29" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="E27" s="29" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F27" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="G27" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="H27" s="42" t="n">
+        <v>400</v>
+      </c>
+      <c r="I27" s="42" t="n">
+        <v>15</v>
+      </c>
+      <c r="J27" s="47" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K27" s="47" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="L27" s="48"/>
+      <c r="M27" s="48"/>
+      <c r="N27" s="26" t="str">
+        <f aca="false">IF(OR(L27="",M27="",$G$5="",$G$6=""),"",(L27/$G$5)/(M27/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O27" s="48"/>
+      <c r="P27" s="48"/>
+      <c r="Q27" s="48"/>
+      <c r="R27" s="48"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="42" t="n">
+        <v>20</v>
+      </c>
+      <c r="C28" s="29" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="D28" s="29" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="E28" s="29" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F28" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="G28" s="47" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H28" s="42" t="n">
+        <v>400</v>
+      </c>
+      <c r="I28" s="42" t="n">
+        <v>15</v>
+      </c>
+      <c r="J28" s="47" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="K28" s="47" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="L28" s="48"/>
+      <c r="M28" s="48"/>
+      <c r="N28" s="26" t="str">
+        <f aca="false">IF(OR(L28="",M28="",$G$5="",$G$6=""),"",(L28/$G$5)/(M28/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O28" s="48"/>
+      <c r="P28" s="48"/>
+      <c r="Q28" s="48"/>
+      <c r="R28" s="48"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="42" t="n">
+        <v>21</v>
+      </c>
+      <c r="C29" s="29" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="D29" s="29" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="E29" s="29" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F29" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="G29" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="H29" s="42" t="n">
+        <v>400</v>
+      </c>
+      <c r="I29" s="42" t="n">
+        <v>15</v>
+      </c>
+      <c r="J29" s="47" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="K29" s="47" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="L29" s="48"/>
+      <c r="M29" s="48"/>
+      <c r="N29" s="26" t="str">
+        <f aca="false">IF(OR(L29="",M29="",$G$5="",$G$6=""),"",(L29/$G$5)/(M29/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O29" s="48"/>
+      <c r="P29" s="48"/>
+      <c r="Q29" s="48"/>
+      <c r="R29" s="48"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="42" t="n">
+        <v>22</v>
+      </c>
+      <c r="C30" s="29" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="D30" s="29" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="E30" s="29" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F30" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="G30" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" s="42" t="n">
+        <v>400</v>
+      </c>
+      <c r="I30" s="42" t="n">
+        <v>25</v>
+      </c>
+      <c r="J30" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="K30" s="47" t="n">
+        <v>23</v>
+      </c>
+      <c r="L30" s="48"/>
+      <c r="M30" s="48"/>
+      <c r="N30" s="26" t="str">
+        <f aca="false">IF(OR(L30="",M30="",$G$5="",$G$6=""),"",(L30/$G$5)/(M30/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O30" s="48"/>
+      <c r="P30" s="48"/>
+      <c r="Q30" s="48"/>
+      <c r="R30" s="48"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="42" t="n">
+        <v>23</v>
+      </c>
+      <c r="C31" s="29" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="D31" s="29" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="E31" s="29" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F31" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="G31" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="H31" s="42" t="n">
+        <v>400</v>
+      </c>
+      <c r="I31" s="42" t="n">
+        <v>25</v>
+      </c>
+      <c r="J31" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="K31" s="47" t="n">
+        <v>21</v>
+      </c>
+      <c r="L31" s="48"/>
+      <c r="M31" s="48"/>
+      <c r="N31" s="26" t="str">
+        <f aca="false">IF(OR(L31="",M31="",$G$5="",$G$6=""),"",(L31/$G$5)/(M31/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O31" s="48"/>
+      <c r="P31" s="48"/>
+      <c r="Q31" s="48"/>
+      <c r="R31" s="48"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="42" t="n">
+        <v>24</v>
+      </c>
+      <c r="C32" s="29" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="D32" s="29" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="E32" s="29" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F32" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="G32" s="47" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H32" s="42" t="n">
+        <v>400</v>
+      </c>
+      <c r="I32" s="42" t="n">
+        <v>25</v>
+      </c>
+      <c r="J32" s="47" t="n">
+        <v>3</v>
+      </c>
+      <c r="K32" s="47" t="n">
+        <v>19</v>
+      </c>
+      <c r="L32" s="48"/>
+      <c r="M32" s="48"/>
+      <c r="N32" s="26" t="str">
+        <f aca="false">IF(OR(L32="",M32="",$G$5="",$G$6=""),"",(L32/$G$5)/(M32/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O32" s="48"/>
+      <c r="P32" s="48"/>
+      <c r="Q32" s="48"/>
+      <c r="R32" s="48"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="42" t="n">
+        <v>25</v>
+      </c>
+      <c r="C33" s="29" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="D33" s="29" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="E33" s="29" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F33" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="G33" s="47" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H33" s="42" t="n">
+        <v>400</v>
+      </c>
+      <c r="I33" s="42" t="n">
+        <v>35</v>
+      </c>
+      <c r="J33" s="47" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="K33" s="47" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="L33" s="48"/>
+      <c r="M33" s="48"/>
+      <c r="N33" s="26" t="str">
+        <f aca="false">IF(OR(L33="",M33="",$G$5="",$G$6=""),"",(L33/$G$5)/(M33/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O33" s="48"/>
+      <c r="P33" s="48"/>
+      <c r="Q33" s="48"/>
+      <c r="R33" s="48"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="42" t="n">
+        <v>26</v>
+      </c>
+      <c r="C34" s="29" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="D34" s="29" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="E34" s="29" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F34" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="G34" s="47" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" s="42" t="n">
+        <v>400</v>
+      </c>
+      <c r="I34" s="42" t="n">
+        <v>35</v>
+      </c>
+      <c r="J34" s="47" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K34" s="47" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="L34" s="48"/>
+      <c r="M34" s="48"/>
+      <c r="N34" s="26" t="str">
+        <f aca="false">IF(OR(L34="",M34="",$G$5="",$G$6=""),"",(L34/$G$5)/(M34/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O34" s="48"/>
+      <c r="P34" s="48"/>
+      <c r="Q34" s="48"/>
+      <c r="R34" s="48"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="42" t="n">
+        <v>27</v>
+      </c>
+      <c r="C35" s="29" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="D35" s="29" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="E35" s="29" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F35" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="G35" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="H35" s="42" t="n">
+        <v>400</v>
+      </c>
+      <c r="I35" s="42" t="n">
+        <v>35</v>
+      </c>
+      <c r="J35" s="47" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="K35" s="47" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="L35" s="48"/>
+      <c r="M35" s="48"/>
+      <c r="N35" s="26" t="str">
+        <f aca="false">IF(OR(L35="",M35="",$G$5="",$G$6=""),"",(L35/$G$5)/(M35/$G$6)^(1/3))</f>
+        <v/>
+      </c>
+      <c r="O35" s="48"/>
+      <c r="P35" s="48"/>
+      <c r="Q35" s="48"/>
+      <c r="R35" s="48"/>
+    </row>
+    <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B37" s="12" t="s">
+        <v>233</v>
+      </c>
+      <c r="C37" s="12"/>
+      <c r="D37" s="12"/>
+      <c r="E37" s="12"/>
+      <c r="F37" s="12"/>
+      <c r="G37" s="12"/>
+      <c r="H37" s="12"/>
+      <c r="I37" s="12"/>
+      <c r="J37" s="12"/>
+      <c r="K37" s="12"/>
+      <c r="L37" s="12"/>
+      <c r="M37" s="12"/>
+      <c r="N37" s="12"/>
+      <c r="O37" s="12"/>
+      <c r="P37" s="12"/>
+      <c r="Q37" s="12"/>
+      <c r="R37" s="12"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B3:R3"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B37:R37"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
@@ -2561,6 +3947,585 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
+  <dimension ref="B2:N19"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="7" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="3"/>
+  </cols>
+  <sheetData>
+    <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B3" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="12"/>
+      <c r="L3" s="12"/>
+      <c r="M3" s="12"/>
+      <c r="N3" s="12"/>
+    </row>
+    <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="M5" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="N5" s="6" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="C6" s="34" t="n">
+        <v>100000</v>
+      </c>
+      <c r="D6" s="35" t="n">
+        <f aca="false">'GCI Mesh Independence'!$C$8</f>
+        <v>5000</v>
+      </c>
+      <c r="E6" s="36"/>
+      <c r="F6" s="36"/>
+      <c r="G6" s="37"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="18" t="n">
+        <f aca="false">C6*'Fluid Properties'!$C$22/Inputs!$C$6</f>
+        <v>0.956659090909091</v>
+      </c>
+      <c r="J6" s="18" t="str">
+        <f aca="false">IF(E6="","",(Inputs!$C$10+E6)/2)</f>
+        <v/>
+      </c>
+      <c r="K6" s="21" t="str">
+        <f aca="false">IF(OR(F6="",J6=""),"",D6/(F6-J6))</f>
+        <v/>
+      </c>
+      <c r="L6" s="38" t="str">
+        <f aca="false">IF(K6="","",K6*Inputs!$C$6/'Fluid Properties'!$C$19)</f>
+        <v/>
+      </c>
+      <c r="M6" s="18" t="str">
+        <f aca="false">IF(OR(G6="",H6=""),"",G6-H6)</f>
+        <v/>
+      </c>
+      <c r="N6" s="39" t="str">
+        <f aca="false">IF(M6="","",2*M6*Inputs!$C$6/(Inputs!$C$7*'Fluid Properties'!$C$17*I6^2))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="C7" s="34" t="n">
+        <v>100000</v>
+      </c>
+      <c r="D7" s="35" t="n">
+        <f aca="false">'GCI Mesh Independence'!$C$8</f>
+        <v>5000</v>
+      </c>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="37"/>
+      <c r="I7" s="18" t="n">
+        <f aca="false">C7*'Fluid Properties'!$C$22/Inputs!$C$6</f>
+        <v>0.956659090909091</v>
+      </c>
+      <c r="J7" s="18" t="str">
+        <f aca="false">IF(E7="","",(Inputs!$C$10+E7)/2)</f>
+        <v/>
+      </c>
+      <c r="K7" s="21" t="str">
+        <f aca="false">IF(OR(F7="",J7=""),"",D7/(F7-J7))</f>
+        <v/>
+      </c>
+      <c r="L7" s="38" t="str">
+        <f aca="false">IF(K7="","",K7*Inputs!$C$6/'Fluid Properties'!$C$19)</f>
+        <v/>
+      </c>
+      <c r="M7" s="18" t="str">
+        <f aca="false">IF(OR(G7="",H7=""),"",G7-H7)</f>
+        <v/>
+      </c>
+      <c r="N7" s="39" t="str">
+        <f aca="false">IF(M7="","",2*M7*Inputs!$C$6/(Inputs!$C$7*'Fluid Properties'!$C$17*I7^2))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="C8" s="34" t="n">
+        <v>100000</v>
+      </c>
+      <c r="D8" s="35" t="n">
+        <f aca="false">'GCI Mesh Independence'!$C$8</f>
+        <v>5000</v>
+      </c>
+      <c r="E8" s="36" t="n">
+        <v>500.93989</v>
+      </c>
+      <c r="F8" s="36" t="n">
+        <v>506.45377</v>
+      </c>
+      <c r="G8" s="37" t="n">
+        <v>368.57945</v>
+      </c>
+      <c r="H8" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="18" t="n">
+        <f aca="false">C8*'Fluid Properties'!$C$22/Inputs!$C$6</f>
+        <v>0.956659090909091</v>
+      </c>
+      <c r="J8" s="18" t="n">
+        <f aca="false">IF(E8="","",(Inputs!$C$10+E8)/2)</f>
+        <v>500.469945</v>
+      </c>
+      <c r="K8" s="21" t="n">
+        <f aca="false">IF(OR(F8="",J8=""),"",D8/(F8-J8))</f>
+        <v>835.585933746388</v>
+      </c>
+      <c r="L8" s="38" t="n">
+        <f aca="false">IF(K8="","",K8*Inputs!$C$6/'Fluid Properties'!$C$19)</f>
+        <v>511.687650793869</v>
+      </c>
+      <c r="M8" s="18" t="n">
+        <f aca="false">IF(OR(G8="",H8=""),"",G8-H8)</f>
+        <v>368.57945</v>
+      </c>
+      <c r="N8" s="39" t="n">
+        <f aca="false">IF(M8="","",2*M8*Inputs!$C$6/(Inputs!$C$7*'Fluid Properties'!$C$17*I8^2))</f>
+        <v>0.0172303048932932</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="22"/>
+      <c r="I9" s="22"/>
+      <c r="J9" s="22"/>
+      <c r="K9" s="22"/>
+      <c r="L9" s="22"/>
+      <c r="M9" s="22"/>
+      <c r="N9" s="22"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="C10" s="34" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D10" s="35" t="n">
+        <f aca="false">'GCI Mesh Independence'!$C$8</f>
+        <v>5000</v>
+      </c>
+      <c r="E10" s="36"/>
+      <c r="F10" s="36"/>
+      <c r="G10" s="37"/>
+      <c r="H10" s="37"/>
+      <c r="I10" s="18" t="n">
+        <f aca="false">C10*'Fluid Properties'!$C$22/Inputs!$C$6</f>
+        <v>0.0478329545454545</v>
+      </c>
+      <c r="J10" s="18" t="str">
+        <f aca="false">IF(E10="","",(Inputs!$C$10+E10)/2)</f>
+        <v/>
+      </c>
+      <c r="K10" s="21" t="str">
+        <f aca="false">IF(OR(F10="",J10=""),"",D10/(F10-J10))</f>
+        <v/>
+      </c>
+      <c r="L10" s="38" t="str">
+        <f aca="false">IF(K10="","",K10*Inputs!$C$6/'Fluid Properties'!$C$19)</f>
+        <v/>
+      </c>
+      <c r="M10" s="18" t="str">
+        <f aca="false">IF(OR(G10="",H10=""),"",G10-H10)</f>
+        <v/>
+      </c>
+      <c r="N10" s="39" t="str">
+        <f aca="false">IF(M10="","",2*M10*Inputs!$C$6/(Inputs!$C$7*'Fluid Properties'!$C$17*I10^2))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="C11" s="34" t="n">
+        <v>7500</v>
+      </c>
+      <c r="D11" s="35" t="n">
+        <f aca="false">'GCI Mesh Independence'!$C$8</f>
+        <v>5000</v>
+      </c>
+      <c r="E11" s="36"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="37"/>
+      <c r="H11" s="37"/>
+      <c r="I11" s="18" t="n">
+        <f aca="false">C11*'Fluid Properties'!$C$22/Inputs!$C$6</f>
+        <v>0.0717494318181818</v>
+      </c>
+      <c r="J11" s="18" t="str">
+        <f aca="false">IF(E11="","",(Inputs!$C$10+E11)/2)</f>
+        <v/>
+      </c>
+      <c r="K11" s="21" t="str">
+        <f aca="false">IF(OR(F11="",J11=""),"",D11/(F11-J11))</f>
+        <v/>
+      </c>
+      <c r="L11" s="38" t="str">
+        <f aca="false">IF(K11="","",K11*Inputs!$C$6/'Fluid Properties'!$C$19)</f>
+        <v/>
+      </c>
+      <c r="M11" s="18" t="str">
+        <f aca="false">IF(OR(G11="",H11=""),"",G11-H11)</f>
+        <v/>
+      </c>
+      <c r="N11" s="39" t="str">
+        <f aca="false">IF(M11="","",2*M11*Inputs!$C$6/(Inputs!$C$7*'Fluid Properties'!$C$17*I11^2))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="C12" s="34" t="n">
+        <v>10000</v>
+      </c>
+      <c r="D12" s="35" t="n">
+        <f aca="false">'GCI Mesh Independence'!$C$8</f>
+        <v>5000</v>
+      </c>
+      <c r="E12" s="36"/>
+      <c r="F12" s="36"/>
+      <c r="G12" s="37"/>
+      <c r="H12" s="37"/>
+      <c r="I12" s="18" t="n">
+        <f aca="false">C12*'Fluid Properties'!$C$22/Inputs!$C$6</f>
+        <v>0.0956659090909091</v>
+      </c>
+      <c r="J12" s="18" t="str">
+        <f aca="false">IF(E12="","",(Inputs!$C$10+E12)/2)</f>
+        <v/>
+      </c>
+      <c r="K12" s="21" t="str">
+        <f aca="false">IF(OR(F12="",J12=""),"",D12/(F12-J12))</f>
+        <v/>
+      </c>
+      <c r="L12" s="38" t="str">
+        <f aca="false">IF(K12="","",K12*Inputs!$C$6/'Fluid Properties'!$C$19)</f>
+        <v/>
+      </c>
+      <c r="M12" s="18" t="str">
+        <f aca="false">IF(OR(G12="",H12=""),"",G12-H12)</f>
+        <v/>
+      </c>
+      <c r="N12" s="39" t="str">
+        <f aca="false">IF(M12="","",2*M12*Inputs!$C$6/(Inputs!$C$7*'Fluid Properties'!$C$17*I12^2))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="C13" s="34" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D13" s="35" t="n">
+        <f aca="false">'GCI Mesh Independence'!$C$8</f>
+        <v>5000</v>
+      </c>
+      <c r="E13" s="36"/>
+      <c r="F13" s="36"/>
+      <c r="G13" s="37"/>
+      <c r="H13" s="37"/>
+      <c r="I13" s="18" t="n">
+        <f aca="false">C13*'Fluid Properties'!$C$22/Inputs!$C$6</f>
+        <v>0.191331818181818</v>
+      </c>
+      <c r="J13" s="18" t="str">
+        <f aca="false">IF(E13="","",(Inputs!$C$10+E13)/2)</f>
+        <v/>
+      </c>
+      <c r="K13" s="21" t="str">
+        <f aca="false">IF(OR(F13="",J13=""),"",D13/(F13-J13))</f>
+        <v/>
+      </c>
+      <c r="L13" s="38" t="str">
+        <f aca="false">IF(K13="","",K13*Inputs!$C$6/'Fluid Properties'!$C$19)</f>
+        <v/>
+      </c>
+      <c r="M13" s="18" t="str">
+        <f aca="false">IF(OR(G13="",H13=""),"",G13-H13)</f>
+        <v/>
+      </c>
+      <c r="N13" s="39" t="str">
+        <f aca="false">IF(M13="","",2*M13*Inputs!$C$6/(Inputs!$C$7*'Fluid Properties'!$C$17*I13^2))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="C14" s="34" t="n">
+        <v>30000</v>
+      </c>
+      <c r="D14" s="35" t="n">
+        <f aca="false">'GCI Mesh Independence'!$C$8</f>
+        <v>5000</v>
+      </c>
+      <c r="E14" s="36"/>
+      <c r="F14" s="36"/>
+      <c r="G14" s="37"/>
+      <c r="H14" s="37"/>
+      <c r="I14" s="18" t="n">
+        <f aca="false">C14*'Fluid Properties'!$C$22/Inputs!$C$6</f>
+        <v>0.286997727272727</v>
+      </c>
+      <c r="J14" s="18" t="str">
+        <f aca="false">IF(E14="","",(Inputs!$C$10+E14)/2)</f>
+        <v/>
+      </c>
+      <c r="K14" s="21" t="str">
+        <f aca="false">IF(OR(F14="",J14=""),"",D14/(F14-J14))</f>
+        <v/>
+      </c>
+      <c r="L14" s="38" t="str">
+        <f aca="false">IF(K14="","",K14*Inputs!$C$6/'Fluid Properties'!$C$19)</f>
+        <v/>
+      </c>
+      <c r="M14" s="18" t="str">
+        <f aca="false">IF(OR(G14="",H14=""),"",G14-H14)</f>
+        <v/>
+      </c>
+      <c r="N14" s="39" t="str">
+        <f aca="false">IF(M14="","",2*M14*Inputs!$C$6/(Inputs!$C$7*'Fluid Properties'!$C$17*I14^2))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="C15" s="34" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D15" s="35" t="n">
+        <f aca="false">'GCI Mesh Independence'!$C$8</f>
+        <v>5000</v>
+      </c>
+      <c r="E15" s="36"/>
+      <c r="F15" s="36"/>
+      <c r="G15" s="37"/>
+      <c r="H15" s="37"/>
+      <c r="I15" s="18" t="n">
+        <f aca="false">C15*'Fluid Properties'!$C$22/Inputs!$C$6</f>
+        <v>0.478329545454545</v>
+      </c>
+      <c r="J15" s="18" t="str">
+        <f aca="false">IF(E15="","",(Inputs!$C$10+E15)/2)</f>
+        <v/>
+      </c>
+      <c r="K15" s="21" t="str">
+        <f aca="false">IF(OR(F15="",J15=""),"",D15/(F15-J15))</f>
+        <v/>
+      </c>
+      <c r="L15" s="38" t="str">
+        <f aca="false">IF(K15="","",K15*Inputs!$C$6/'Fluid Properties'!$C$19)</f>
+        <v/>
+      </c>
+      <c r="M15" s="18" t="str">
+        <f aca="false">IF(OR(G15="",H15=""),"",G15-H15)</f>
+        <v/>
+      </c>
+      <c r="N15" s="39" t="str">
+        <f aca="false">IF(M15="","",2*M15*Inputs!$C$6/(Inputs!$C$7*'Fluid Properties'!$C$17*I15^2))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="C16" s="34" t="n">
+        <v>70000</v>
+      </c>
+      <c r="D16" s="35" t="n">
+        <f aca="false">'GCI Mesh Independence'!$C$8</f>
+        <v>5000</v>
+      </c>
+      <c r="E16" s="36"/>
+      <c r="F16" s="36"/>
+      <c r="G16" s="37"/>
+      <c r="H16" s="37"/>
+      <c r="I16" s="18" t="n">
+        <f aca="false">C16*'Fluid Properties'!$C$22/Inputs!$C$6</f>
+        <v>0.669661363636363</v>
+      </c>
+      <c r="J16" s="18" t="str">
+        <f aca="false">IF(E16="","",(Inputs!$C$10+E16)/2)</f>
+        <v/>
+      </c>
+      <c r="K16" s="21" t="str">
+        <f aca="false">IF(OR(F16="",J16=""),"",D16/(F16-J16))</f>
+        <v/>
+      </c>
+      <c r="L16" s="38" t="str">
+        <f aca="false">IF(K16="","",K16*Inputs!$C$6/'Fluid Properties'!$C$19)</f>
+        <v/>
+      </c>
+      <c r="M16" s="18" t="str">
+        <f aca="false">IF(OR(G16="",H16=""),"",G16-H16)</f>
+        <v/>
+      </c>
+      <c r="N16" s="39" t="str">
+        <f aca="false">IF(M16="","",2*M16*Inputs!$C$6/(Inputs!$C$7*'Fluid Properties'!$C$17*I16^2))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="C17" s="34" t="n">
+        <v>100000</v>
+      </c>
+      <c r="D17" s="35" t="n">
+        <f aca="false">'GCI Mesh Independence'!$C$8</f>
+        <v>5000</v>
+      </c>
+      <c r="E17" s="36"/>
+      <c r="F17" s="36"/>
+      <c r="G17" s="37"/>
+      <c r="H17" s="37"/>
+      <c r="I17" s="18" t="n">
+        <f aca="false">C17*'Fluid Properties'!$C$22/Inputs!$C$6</f>
+        <v>0.956659090909091</v>
+      </c>
+      <c r="J17" s="18" t="str">
+        <f aca="false">IF(E17="","",(Inputs!$C$10+E17)/2)</f>
+        <v/>
+      </c>
+      <c r="K17" s="21" t="str">
+        <f aca="false">IF(OR(F17="",J17=""),"",D17/(F17-J17))</f>
+        <v/>
+      </c>
+      <c r="L17" s="38" t="str">
+        <f aca="false">IF(K17="","",K17*Inputs!$C$6/'Fluid Properties'!$C$19)</f>
+        <v/>
+      </c>
+      <c r="M17" s="18" t="str">
+        <f aca="false">IF(OR(G17="",H17=""),"",G17-H17)</f>
+        <v/>
+      </c>
+      <c r="N17" s="39" t="str">
+        <f aca="false">IF(M17="","",2*M17*Inputs!$C$6/(Inputs!$C$7*'Fluid Properties'!$C$17*I17^2))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="12"/>
+      <c r="K19" s="12"/>
+      <c r="L19" s="12"/>
+      <c r="M19" s="12"/>
+      <c r="N19" s="12"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B3:N3"/>
+    <mergeCell ref="B9:N9"/>
+    <mergeCell ref="B19:N19"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
   <dimension ref="B2:I15"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -2576,12 +4541,12 @@
   <sheetData>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>122</v>
+        <v>149</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="12" t="s">
-        <v>123</v>
+        <v>150</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -2596,25 +4561,25 @@
         <v>79</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>124</v>
+        <v>151</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>125</v>
+        <v>152</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>126</v>
+        <v>153</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>127</v>
+        <v>154</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>128</v>
+        <v>155</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>129</v>
+        <v>156</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>130</v>
+        <v>157</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2633,13 +4598,19 @@
         <f aca="false">0.023*B6^0.8*'Fluid Properties'!$C$24^0.4</f>
         <v>50.2911752463619</v>
       </c>
-      <c r="F6" s="35"/>
-      <c r="G6" s="36" t="str">
+      <c r="F6" s="17" t="str">
+        <f aca="false">IF('Results Calculator'!L10="","",'Results Calculator'!L10)</f>
+        <v/>
+      </c>
+      <c r="G6" s="40" t="str">
         <f aca="false">IF(F6="","",ABS(F6-D6)/D6)</f>
         <v/>
       </c>
-      <c r="H6" s="35"/>
-      <c r="I6" s="36" t="str">
+      <c r="H6" s="17" t="str">
+        <f aca="false">IF('Results Calculator'!N10="","",'Results Calculator'!N10)</f>
+        <v/>
+      </c>
+      <c r="I6" s="40" t="str">
         <f aca="false">IF(H6="","",ABS(H6-C6)/C6)</f>
         <v/>
       </c>
@@ -2660,13 +4631,19 @@
         <f aca="false">0.023*B7^0.8*'Fluid Properties'!$C$24^0.4</f>
         <v>69.5608358585765</v>
       </c>
-      <c r="F7" s="35"/>
-      <c r="G7" s="36" t="str">
+      <c r="F7" s="17" t="str">
+        <f aca="false">IF('Results Calculator'!L11="","",'Results Calculator'!L11)</f>
+        <v/>
+      </c>
+      <c r="G7" s="40" t="str">
         <f aca="false">IF(F7="","",ABS(F7-D7)/D7)</f>
         <v/>
       </c>
-      <c r="H7" s="35"/>
-      <c r="I7" s="36" t="str">
+      <c r="H7" s="17" t="str">
+        <f aca="false">IF('Results Calculator'!N11="","",'Results Calculator'!N11)</f>
+        <v/>
+      </c>
+      <c r="I7" s="40" t="str">
         <f aca="false">IF(H7="","",ABS(H7-C7)/C7)</f>
         <v/>
       </c>
@@ -2687,13 +4664,19 @@
         <f aca="false">0.023*B8^0.8*'Fluid Properties'!$C$24^0.4</f>
         <v>87.5620218790889</v>
       </c>
-      <c r="F8" s="35"/>
-      <c r="G8" s="36" t="str">
+      <c r="F8" s="17" t="str">
+        <f aca="false">IF('Results Calculator'!L12="","",'Results Calculator'!L12)</f>
+        <v/>
+      </c>
+      <c r="G8" s="40" t="str">
         <f aca="false">IF(F8="","",ABS(F8-D8)/D8)</f>
         <v/>
       </c>
-      <c r="H8" s="35"/>
-      <c r="I8" s="36" t="str">
+      <c r="H8" s="17" t="str">
+        <f aca="false">IF('Results Calculator'!N12="","",'Results Calculator'!N12)</f>
+        <v/>
+      </c>
+      <c r="I8" s="40" t="str">
         <f aca="false">IF(H8="","",ABS(H8-C8)/C8)</f>
         <v/>
       </c>
@@ -2714,13 +4697,19 @@
         <f aca="false">0.023*B9^0.8*'Fluid Properties'!$C$24^0.4</f>
         <v>152.454334940377</v>
       </c>
-      <c r="F9" s="35"/>
-      <c r="G9" s="36" t="str">
+      <c r="F9" s="17" t="str">
+        <f aca="false">IF('Results Calculator'!L13="","",'Results Calculator'!L13)</f>
+        <v/>
+      </c>
+      <c r="G9" s="40" t="str">
         <f aca="false">IF(F9="","",ABS(F9-D9)/D9)</f>
         <v/>
       </c>
-      <c r="H9" s="35"/>
-      <c r="I9" s="36" t="str">
+      <c r="H9" s="17" t="str">
+        <f aca="false">IF('Results Calculator'!N13="","",'Results Calculator'!N13)</f>
+        <v/>
+      </c>
+      <c r="I9" s="40" t="str">
         <f aca="false">IF(H9="","",ABS(H9-C9)/C9)</f>
         <v/>
       </c>
@@ -2741,13 +4730,19 @@
         <f aca="false">0.023*B10^0.8*'Fluid Properties'!$C$24^0.4</f>
         <v>210.86902258231</v>
       </c>
-      <c r="F10" s="35"/>
-      <c r="G10" s="36" t="str">
+      <c r="F10" s="17" t="str">
+        <f aca="false">IF('Results Calculator'!L14="","",'Results Calculator'!L14)</f>
+        <v/>
+      </c>
+      <c r="G10" s="40" t="str">
         <f aca="false">IF(F10="","",ABS(F10-D10)/D10)</f>
         <v/>
       </c>
-      <c r="H10" s="35"/>
-      <c r="I10" s="36" t="str">
+      <c r="H10" s="17" t="str">
+        <f aca="false">IF('Results Calculator'!N14="","",'Results Calculator'!N14)</f>
+        <v/>
+      </c>
+      <c r="I10" s="40" t="str">
         <f aca="false">IF(H10="","",ABS(H10-C10)/C10)</f>
         <v/>
       </c>
@@ -2768,13 +4763,19 @@
         <f aca="false">0.023*B11^0.8*'Fluid Properties'!$C$24^0.4</f>
         <v>317.315863842325</v>
       </c>
-      <c r="F11" s="35"/>
-      <c r="G11" s="36" t="str">
+      <c r="F11" s="17" t="str">
+        <f aca="false">IF('Results Calculator'!L15="","",'Results Calculator'!L15)</f>
+        <v/>
+      </c>
+      <c r="G11" s="40" t="str">
         <f aca="false">IF(F11="","",ABS(F11-D11)/D11)</f>
         <v/>
       </c>
-      <c r="H11" s="35"/>
-      <c r="I11" s="36" t="str">
+      <c r="H11" s="17" t="str">
+        <f aca="false">IF('Results Calculator'!N15="","",'Results Calculator'!N15)</f>
+        <v/>
+      </c>
+      <c r="I11" s="40" t="str">
         <f aca="false">IF(H11="","",ABS(H11-C11)/C11)</f>
         <v/>
       </c>
@@ -2795,13 +4796,19 @@
         <f aca="false">0.023*B12^0.8*'Fluid Properties'!$C$24^0.4</f>
         <v>415.330871372776</v>
       </c>
-      <c r="F12" s="35"/>
-      <c r="G12" s="36" t="str">
+      <c r="F12" s="17" t="str">
+        <f aca="false">IF('Results Calculator'!L16="","",'Results Calculator'!L16)</f>
+        <v/>
+      </c>
+      <c r="G12" s="40" t="str">
         <f aca="false">IF(F12="","",ABS(F12-D12)/D12)</f>
         <v/>
       </c>
-      <c r="H12" s="35"/>
-      <c r="I12" s="36" t="str">
+      <c r="H12" s="17" t="str">
+        <f aca="false">IF('Results Calculator'!N16="","",'Results Calculator'!N16)</f>
+        <v/>
+      </c>
+      <c r="I12" s="40" t="str">
         <f aca="false">IF(H12="","",ABS(H12-C12)/C12)</f>
         <v/>
       </c>
@@ -2822,20 +4829,26 @@
         <f aca="false">0.023*B13^0.8*'Fluid Properties'!$C$24^0.4</f>
         <v>552.479008021465</v>
       </c>
-      <c r="F13" s="35"/>
-      <c r="G13" s="36" t="str">
+      <c r="F13" s="17" t="str">
+        <f aca="false">IF('Results Calculator'!L17="","",'Results Calculator'!L17)</f>
+        <v/>
+      </c>
+      <c r="G13" s="40" t="str">
         <f aca="false">IF(F13="","",ABS(F13-D13)/D13)</f>
         <v/>
       </c>
-      <c r="H13" s="35"/>
-      <c r="I13" s="36" t="str">
+      <c r="H13" s="17" t="str">
+        <f aca="false">IF('Results Calculator'!N17="","",'Results Calculator'!N17)</f>
+        <v/>
+      </c>
+      <c r="I13" s="40" t="str">
         <f aca="false">IF(H13="","",ABS(H13-C13)/C13)</f>
         <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="12" t="s">
-        <v>131</v>
+        <v>158</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="12"/>
@@ -2876,7 +4889,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
@@ -2892,12 +4905,12 @@
   <sheetData>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>132</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="12" t="s">
-        <v>133</v>
+        <v>160</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -2905,25 +4918,25 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="7" t="s">
-        <v>134</v>
+        <v>161</v>
       </c>
       <c r="C5" s="34" t="n">
         <v>100000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="37" t="s">
-        <v>135</v>
-      </c>
-      <c r="C7" s="37"/>
-      <c r="D7" s="37"/>
-      <c r="E7" s="37"/>
+      <c r="B7" s="41" t="s">
+        <v>162</v>
+      </c>
+      <c r="C7" s="41"/>
+      <c r="D7" s="41"/>
+      <c r="E7" s="41"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="C8" s="38" t="n">
+        <v>163</v>
+      </c>
+      <c r="C8" s="42" t="n">
         <v>5000</v>
       </c>
     </row>
@@ -2932,58 +4945,86 @@
         <v>30</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>137</v>
+        <v>164</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>138</v>
+        <v>165</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>139</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="C11" s="35"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="35" t="n">
+        <v>167</v>
+      </c>
+      <c r="C11" s="43" t="str">
+        <f aca="false">IF('Results Calculator'!E6="","",'Results Calculator'!E6)</f>
+        <v/>
+      </c>
+      <c r="D11" s="43" t="str">
+        <f aca="false">IF('Results Calculator'!E7="","",'Results Calculator'!E7)</f>
+        <v/>
+      </c>
+      <c r="E11" s="43" t="n">
+        <f aca="false">IF('Results Calculator'!E8="","",'Results Calculator'!E8)</f>
         <v>500.93989</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="7" t="s">
-        <v>141</v>
-      </c>
-      <c r="C12" s="35"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="35" t="n">
+        <v>168</v>
+      </c>
+      <c r="C12" s="43" t="str">
+        <f aca="false">IF('Results Calculator'!F6="","",'Results Calculator'!F6)</f>
+        <v/>
+      </c>
+      <c r="D12" s="43" t="str">
+        <f aca="false">IF('Results Calculator'!F7="","",'Results Calculator'!F7)</f>
+        <v/>
+      </c>
+      <c r="E12" s="43" t="n">
+        <f aca="false">IF('Results Calculator'!F8="","",'Results Calculator'!F8)</f>
         <v>506.45377</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="35" t="n">
+        <v>169</v>
+      </c>
+      <c r="C13" s="44" t="str">
+        <f aca="false">IF('Results Calculator'!G6="","",'Results Calculator'!G6)</f>
+        <v/>
+      </c>
+      <c r="D13" s="44" t="str">
+        <f aca="false">IF('Results Calculator'!G7="","",'Results Calculator'!G7)</f>
+        <v/>
+      </c>
+      <c r="E13" s="44" t="n">
+        <f aca="false">IF('Results Calculator'!G8="","",'Results Calculator'!G8)</f>
         <v>368.57945</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="7" t="s">
-        <v>143</v>
-      </c>
-      <c r="C14" s="35"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="35" t="n">
+        <v>170</v>
+      </c>
+      <c r="C14" s="44" t="str">
+        <f aca="false">IF('Results Calculator'!H6="","",'Results Calculator'!H6)</f>
+        <v/>
+      </c>
+      <c r="D14" s="44" t="str">
+        <f aca="false">IF('Results Calculator'!H7="","",'Results Calculator'!H7)</f>
+        <v/>
+      </c>
+      <c r="E14" s="44" t="n">
+        <f aca="false">IF('Results Calculator'!H8="","",'Results Calculator'!H8)</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="7" t="s">
-        <v>144</v>
+        <v>171</v>
       </c>
       <c r="C16" s="18" t="str">
         <f aca="false">IF(C11="","",(Inputs!$C$10+C11)/2)</f>
@@ -3000,7 +5041,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="7" t="s">
-        <v>145</v>
+        <v>172</v>
       </c>
       <c r="C17" s="21" t="str">
         <f aca="false">IF(OR(C12="",C16=""),"",$C$8/(C12-C16))</f>
@@ -3017,24 +5058,24 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="C18" s="39" t="str">
+        <v>173</v>
+      </c>
+      <c r="C18" s="38" t="str">
         <f aca="false">IF(C17="","",C17*Inputs!$C$6/'Fluid Properties'!$C$19)</f>
         <v/>
       </c>
-      <c r="D18" s="39" t="str">
+      <c r="D18" s="38" t="str">
         <f aca="false">IF(D17="","",D17*Inputs!$C$6/'Fluid Properties'!$C$19)</f>
         <v/>
       </c>
-      <c r="E18" s="39" t="n">
+      <c r="E18" s="38" t="n">
         <f aca="false">IF(E17="","",E17*Inputs!$C$6/'Fluid Properties'!$C$19)</f>
         <v>511.687650793869</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="7" t="s">
-        <v>147</v>
+        <v>174</v>
       </c>
       <c r="C19" s="18" t="str">
         <f aca="false">IF(OR(C13="",C14=""),"",C13-C14)</f>
@@ -3051,54 +5092,54 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="C20" s="40" t="str">
+        <v>175</v>
+      </c>
+      <c r="C20" s="39" t="str">
         <f aca="false">IF(C19="","",2*C19*Inputs!$C$6/(Inputs!$C$7*'Fluid Properties'!$C$17*'YPlus Inflation'!$D$10^2))</f>
         <v/>
       </c>
-      <c r="D20" s="40" t="str">
+      <c r="D20" s="39" t="str">
         <f aca="false">IF(D19="","",2*D19*Inputs!$C$6/(Inputs!$C$7*'Fluid Properties'!$C$17*'YPlus Inflation'!$D$10^2))</f>
         <v/>
       </c>
-      <c r="E20" s="40" t="n">
+      <c r="E20" s="39" t="n">
         <f aca="false">IF(E19="","",2*E19*Inputs!$C$6/(Inputs!$C$7*'Fluid Properties'!$C$17*'YPlus Inflation'!$D$10^2))</f>
         <v>0.0172303048932932</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="12" t="s">
-        <v>149</v>
+        <v>176</v>
       </c>
       <c r="C21" s="12"/>
       <c r="D21" s="12"/>
       <c r="E21" s="12"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="37" t="s">
-        <v>150</v>
-      </c>
-      <c r="C23" s="37"/>
-      <c r="D23" s="37"/>
-      <c r="E23" s="37"/>
+      <c r="B23" s="41" t="s">
+        <v>177</v>
+      </c>
+      <c r="C23" s="41"/>
+      <c r="D23" s="41"/>
+      <c r="E23" s="41"/>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>137</v>
+        <v>164</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>138</v>
+        <v>165</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>139</v>
+        <v>166</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="3" t="s">
-        <v>151</v>
+        <v>133</v>
       </c>
       <c r="C25" s="17" t="str">
         <f aca="false">IF(C18="","",C18)</f>
@@ -3115,114 +5156,114 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="C26" s="41" t="str">
+        <v>135</v>
+      </c>
+      <c r="C26" s="43" t="str">
         <f aca="false">IF(C20="","",C20)</f>
         <v/>
       </c>
-      <c r="D26" s="41" t="str">
+      <c r="D26" s="43" t="str">
         <f aca="false">IF(D20="","",D20)</f>
         <v/>
       </c>
-      <c r="E26" s="41" t="n">
+      <c r="E26" s="43" t="n">
         <f aca="false">IF(E20="","",E20)</f>
         <v>0.0172303048932932</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="C28" s="42" t="str">
+        <v>178</v>
+      </c>
+      <c r="C28" s="45" t="str">
         <f aca="false">IF(OR(C25="",D25=""),"",(D25-C25)/C25)</f>
         <v/>
       </c>
-      <c r="D28" s="42" t="str">
+      <c r="D28" s="45" t="str">
         <f aca="false">IF(OR(D25="",E25=""),"",(E25-D25)/D25)</f>
         <v/>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="C29" s="42" t="str">
+        <v>179</v>
+      </c>
+      <c r="C29" s="45" t="str">
         <f aca="false">IF(OR(C26="",D26=""),"",(D26-C26)/C26)</f>
         <v/>
       </c>
-      <c r="D29" s="42" t="str">
+      <c r="D29" s="45" t="str">
         <f aca="false">IF(OR(D26="",E26=""),"",(E26-D26)/D26)</f>
         <v/>
       </c>
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="12" t="s">
-        <v>155</v>
+        <v>180</v>
       </c>
       <c r="C30" s="12"/>
       <c r="D30" s="12"/>
       <c r="E30" s="12"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="37" t="s">
-        <v>156</v>
-      </c>
-      <c r="C32" s="37"/>
-      <c r="D32" s="37"/>
-      <c r="E32" s="37"/>
+      <c r="B32" s="41" t="s">
+        <v>181</v>
+      </c>
+      <c r="C32" s="41"/>
+      <c r="D32" s="41"/>
+      <c r="E32" s="41"/>
     </row>
     <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>137</v>
+        <v>164</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>138</v>
+        <v>165</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>139</v>
+        <v>166</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="C34" s="43" t="n">
+        <v>182</v>
+      </c>
+      <c r="C34" s="44" t="n">
         <f aca="false">'Mesh Levels'!$E$29</f>
         <v>3.43167571948627</v>
       </c>
-      <c r="D34" s="43" t="n">
+      <c r="D34" s="44" t="n">
         <f aca="false">'Mesh Levels'!$D$29</f>
         <v>4.8393110188735</v>
       </c>
-      <c r="E34" s="43" t="n">
+      <c r="E34" s="44" t="n">
         <f aca="false">'Mesh Levels'!$C$29</f>
         <v>6.72473347933769</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="C35" s="41" t="str">
+        <v>183</v>
+      </c>
+      <c r="C35" s="43" t="str">
         <f aca="false">IF(C18="","",C18)</f>
         <v/>
       </c>
-      <c r="D35" s="41" t="str">
+      <c r="D35" s="43" t="str">
         <f aca="false">IF(D18="","",D18)</f>
         <v/>
       </c>
-      <c r="E35" s="41" t="n">
+      <c r="E35" s="43" t="n">
         <f aca="false">IF(E18="","",E18)</f>
         <v>511.687650793869</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="7" t="s">
-        <v>159</v>
+        <v>184</v>
       </c>
       <c r="C37" s="26" t="n">
         <f aca="false">D34/C34</f>
@@ -3231,7 +5272,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="7" t="s">
-        <v>160</v>
+        <v>185</v>
       </c>
       <c r="C38" s="26" t="n">
         <f aca="false">E34/D34</f>
@@ -3240,7 +5281,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="7" t="s">
-        <v>161</v>
+        <v>186</v>
       </c>
       <c r="C39" s="18" t="str">
         <f aca="false">IF(OR(C35="",D35=""),"",D35-C35)</f>
@@ -3249,7 +5290,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="7" t="s">
-        <v>162</v>
+        <v>187</v>
       </c>
       <c r="C40" s="18" t="str">
         <f aca="false">IF(OR(D35="",E35=""),"",E35-D35)</f>
@@ -3258,7 +5299,7 @@
     </row>
     <row r="41" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="4" t="s">
-        <v>163</v>
+        <v>188</v>
       </c>
       <c r="C41" s="26" t="str">
         <f aca="false">IF(OR(C39="",C40=""),"",LN(ABS(C40/C39))/LN(C37))</f>
@@ -3267,7 +5308,7 @@
     </row>
     <row r="42" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="4" t="s">
-        <v>164</v>
+        <v>189</v>
       </c>
       <c r="C42" s="18" t="str">
         <f aca="false">IF(C41="","",(C37^C41*C35-D35)/(C37^C41-1))</f>
@@ -3276,98 +5317,98 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="C43" s="42" t="str">
+        <v>190</v>
+      </c>
+      <c r="C43" s="45" t="str">
         <f aca="false">IF(OR(C35="",D35=""),"",ABS((C35-D35)/C35))</f>
         <v/>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="C44" s="42" t="str">
+        <v>191</v>
+      </c>
+      <c r="C44" s="45" t="str">
         <f aca="false">IF(C42="","",ABS((C42-C35)/C42))</f>
         <v/>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="C45" s="44" t="str">
+        <v>192</v>
+      </c>
+      <c r="C45" s="46" t="str">
         <f aca="false">IF(OR(C41="",C43=""),"",1.25*C43/(C37^C41-1))</f>
         <v/>
       </c>
     </row>
     <row r="46" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="12" t="s">
-        <v>168</v>
+        <v>193</v>
       </c>
       <c r="C46" s="12"/>
       <c r="D46" s="12"/>
       <c r="E46" s="12"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="37" t="s">
-        <v>169</v>
-      </c>
-      <c r="C48" s="37"/>
-      <c r="D48" s="37"/>
-      <c r="E48" s="37"/>
+      <c r="B48" s="41" t="s">
+        <v>194</v>
+      </c>
+      <c r="C48" s="41"/>
+      <c r="D48" s="41"/>
+      <c r="E48" s="41"/>
     </row>
     <row r="49" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B49" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>137</v>
+        <v>164</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>138</v>
+        <v>165</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>139</v>
+        <v>166</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="C50" s="43" t="n">
+        <v>182</v>
+      </c>
+      <c r="C50" s="44" t="n">
         <f aca="false">'Mesh Levels'!$E$29</f>
         <v>3.43167571948627</v>
       </c>
-      <c r="D50" s="43" t="n">
+      <c r="D50" s="44" t="n">
         <f aca="false">'Mesh Levels'!$D$29</f>
         <v>4.8393110188735</v>
       </c>
-      <c r="E50" s="43" t="n">
+      <c r="E50" s="44" t="n">
         <f aca="false">'Mesh Levels'!$C$29</f>
         <v>6.72473347933769</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="7" t="s">
-        <v>170</v>
-      </c>
-      <c r="C51" s="41" t="str">
+        <v>195</v>
+      </c>
+      <c r="C51" s="43" t="str">
         <f aca="false">IF(C20="","",C20)</f>
         <v/>
       </c>
-      <c r="D51" s="41" t="str">
+      <c r="D51" s="43" t="str">
         <f aca="false">IF(D20="","",D20)</f>
         <v/>
       </c>
-      <c r="E51" s="41" t="n">
+      <c r="E51" s="43" t="n">
         <f aca="false">IF(E20="","",E20)</f>
         <v>0.0172303048932932</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="7" t="s">
-        <v>159</v>
+        <v>184</v>
       </c>
       <c r="C53" s="26" t="n">
         <f aca="false">D50/C50</f>
@@ -3376,7 +5417,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="7" t="s">
-        <v>160</v>
+        <v>185</v>
       </c>
       <c r="C54" s="26" t="n">
         <f aca="false">E50/D50</f>
@@ -3385,7 +5426,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="7" t="s">
-        <v>161</v>
+        <v>186</v>
       </c>
       <c r="C55" s="18" t="str">
         <f aca="false">IF(OR(C51="",D51=""),"",D51-C51)</f>
@@ -3394,7 +5435,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="7" t="s">
-        <v>162</v>
+        <v>187</v>
       </c>
       <c r="C56" s="18" t="str">
         <f aca="false">IF(OR(D51="",E51=""),"",E51-D51)</f>
@@ -3403,7 +5444,7 @@
     </row>
     <row r="57" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B57" s="4" t="s">
-        <v>163</v>
+        <v>188</v>
       </c>
       <c r="C57" s="26" t="str">
         <f aca="false">IF(OR(C55="",C56=""),"",LN(ABS(C56/C55))/LN(C53))</f>
@@ -3412,7 +5453,7 @@
     </row>
     <row r="58" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B58" s="4" t="s">
-        <v>164</v>
+        <v>189</v>
       </c>
       <c r="C58" s="18" t="str">
         <f aca="false">IF(C57="","",(C53^C57*C51-D51)/(C53^C57-1))</f>
@@ -3421,34 +5462,34 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="C59" s="42" t="str">
+        <v>190</v>
+      </c>
+      <c r="C59" s="45" t="str">
         <f aca="false">IF(OR(C51="",D51=""),"",ABS((C51-D51)/C51))</f>
         <v/>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="C60" s="42" t="str">
+        <v>191</v>
+      </c>
+      <c r="C60" s="45" t="str">
         <f aca="false">IF(C58="","",ABS((C58-C51)/C58))</f>
         <v/>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="C61" s="44" t="str">
+        <v>192</v>
+      </c>
+      <c r="C61" s="46" t="str">
         <f aca="false">IF(OR(C57="",C59=""),"",1.25*C59/(C53^C57-1))</f>
         <v/>
       </c>
     </row>
     <row r="62" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B62" s="12" t="s">
-        <v>168</v>
+        <v>193</v>
       </c>
       <c r="C62" s="12"/>
       <c r="D62" s="12"/>
@@ -3492,7 +5533,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
@@ -3512,12 +5553,12 @@
   <sheetData>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>171</v>
+        <v>196</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="12" t="s">
-        <v>172</v>
+        <v>197</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -3531,7 +5572,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="7" t="s">
-        <v>173</v>
+        <v>198</v>
       </c>
       <c r="C5" s="11" t="n">
         <v>39.2</v>
@@ -3539,300 +5580,300 @@
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>174</v>
+        <v>199</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>175</v>
+        <v>200</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>176</v>
+        <v>201</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>177</v>
+        <v>202</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>178</v>
+        <v>203</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>181</v>
+        <v>206</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>182</v>
+        <v>207</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>183</v>
+        <v>208</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="38" t="n">
+      <c r="B8" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="45" t="n">
+      <c r="C8" s="47" t="n">
         <v>933.7</v>
       </c>
-      <c r="D8" s="45" t="n">
+      <c r="D8" s="47" t="n">
         <v>2.6</v>
       </c>
-      <c r="E8" s="45" t="n">
+      <c r="E8" s="47" t="n">
         <v>102.2</v>
       </c>
-      <c r="F8" s="45" t="n">
+      <c r="F8" s="47" t="n">
         <v>47.7</v>
       </c>
-      <c r="G8" s="45" t="n">
+      <c r="G8" s="47" t="n">
         <v>124</v>
       </c>
       <c r="H8" s="29" t="n">
         <v>72.51</v>
       </c>
-      <c r="I8" s="35"/>
-      <c r="J8" s="35"/>
-      <c r="K8" s="36" t="str">
+      <c r="I8" s="48"/>
+      <c r="J8" s="48"/>
+      <c r="K8" s="40" t="str">
         <f aca="false">IF(J8="","",ABS(J8-H8)/H8)</f>
         <v/>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="38" t="n">
+      <c r="B9" s="42" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="45" t="n">
+      <c r="C9" s="47" t="n">
         <v>968.2</v>
       </c>
-      <c r="D9" s="45" t="n">
+      <c r="D9" s="47" t="n">
         <v>3.7</v>
       </c>
-      <c r="E9" s="45" t="n">
+      <c r="E9" s="47" t="n">
         <v>151</v>
       </c>
-      <c r="F9" s="45" t="n">
+      <c r="F9" s="47" t="n">
         <v>47.8</v>
       </c>
-      <c r="G9" s="45" t="n">
+      <c r="G9" s="47" t="n">
         <v>173.3</v>
       </c>
       <c r="H9" s="29" t="n">
         <v>70.9</v>
       </c>
-      <c r="I9" s="35"/>
-      <c r="J9" s="35"/>
-      <c r="K9" s="36" t="str">
+      <c r="I9" s="48"/>
+      <c r="J9" s="48"/>
+      <c r="K9" s="40" t="str">
         <f aca="false">IF(J9="","",ABS(J9-H9)/H9)</f>
         <v/>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="38" t="n">
+      <c r="B10" s="42" t="n">
         <v>3</v>
       </c>
-      <c r="C10" s="45" t="n">
+      <c r="C10" s="47" t="n">
         <v>982.3</v>
       </c>
-      <c r="D10" s="45" t="n">
+      <c r="D10" s="47" t="n">
         <v>2.5</v>
       </c>
-      <c r="E10" s="45" t="n">
+      <c r="E10" s="47" t="n">
         <v>197.5</v>
       </c>
-      <c r="F10" s="45" t="n">
+      <c r="F10" s="47" t="n">
         <v>49.1</v>
       </c>
-      <c r="G10" s="45" t="n">
+      <c r="G10" s="47" t="n">
         <v>219.5</v>
       </c>
       <c r="H10" s="29" t="n">
         <v>70.17</v>
       </c>
-      <c r="I10" s="35"/>
-      <c r="J10" s="35"/>
-      <c r="K10" s="36" t="str">
+      <c r="I10" s="48"/>
+      <c r="J10" s="48"/>
+      <c r="K10" s="40" t="str">
         <f aca="false">IF(J10="","",ABS(J10-H10)/H10)</f>
         <v/>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="38" t="n">
+      <c r="B11" s="42" t="n">
         <v>4</v>
       </c>
-      <c r="C11" s="45" t="n">
+      <c r="C11" s="47" t="n">
         <v>906.6</v>
       </c>
-      <c r="D11" s="45" t="n">
+      <c r="D11" s="47" t="n">
         <v>3.3</v>
       </c>
-      <c r="E11" s="45" t="n">
+      <c r="E11" s="47" t="n">
         <v>250.7</v>
       </c>
-      <c r="F11" s="45" t="n">
+      <c r="F11" s="47" t="n">
         <v>54.7</v>
       </c>
-      <c r="G11" s="45" t="n">
+      <c r="G11" s="47" t="n">
         <v>269.4</v>
       </c>
       <c r="H11" s="29" t="n">
         <v>70.25</v>
       </c>
-      <c r="I11" s="35"/>
-      <c r="J11" s="35"/>
-      <c r="K11" s="36" t="str">
+      <c r="I11" s="48"/>
+      <c r="J11" s="48"/>
+      <c r="K11" s="40" t="str">
         <f aca="false">IF(J11="","",ABS(J11-H11)/H11)</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="38" t="n">
+      <c r="B12" s="42" t="n">
         <v>5</v>
       </c>
-      <c r="C12" s="45" t="n">
+      <c r="C12" s="47" t="n">
         <v>937.9</v>
       </c>
-      <c r="D12" s="45" t="n">
+      <c r="D12" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="45" t="n">
+      <c r="E12" s="47" t="n">
         <v>297.8</v>
       </c>
-      <c r="F12" s="45" t="n">
+      <c r="F12" s="47" t="n">
         <v>55.5</v>
       </c>
-      <c r="G12" s="45" t="n">
+      <c r="G12" s="47" t="n">
         <v>316.9</v>
       </c>
       <c r="H12" s="29" t="n">
         <v>67.98</v>
       </c>
-      <c r="I12" s="35"/>
-      <c r="J12" s="35"/>
-      <c r="K12" s="36" t="str">
+      <c r="I12" s="48"/>
+      <c r="J12" s="48"/>
+      <c r="K12" s="40" t="str">
         <f aca="false">IF(J12="","",ABS(J12-H12)/H12)</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="38" t="n">
+      <c r="B13" s="42" t="n">
         <v>6</v>
       </c>
-      <c r="C13" s="45" t="n">
+      <c r="C13" s="47" t="n">
         <v>880.6</v>
       </c>
-      <c r="D13" s="45" t="n">
+      <c r="D13" s="47" t="n">
         <v>2.9</v>
       </c>
-      <c r="E13" s="45" t="n">
+      <c r="E13" s="47" t="n">
         <v>299</v>
       </c>
-      <c r="F13" s="45" t="n">
+      <c r="F13" s="47" t="n">
         <v>55.6</v>
       </c>
-      <c r="G13" s="45" t="n">
+      <c r="G13" s="47" t="n">
         <v>317.2</v>
       </c>
       <c r="H13" s="29" t="n">
         <v>68.92</v>
       </c>
-      <c r="I13" s="35"/>
-      <c r="J13" s="35"/>
-      <c r="K13" s="36" t="str">
+      <c r="I13" s="48"/>
+      <c r="J13" s="48"/>
+      <c r="K13" s="40" t="str">
         <f aca="false">IF(J13="","",ABS(J13-H13)/H13)</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="38" t="n">
+      <c r="B14" s="42" t="n">
         <v>7</v>
       </c>
-      <c r="C14" s="45" t="n">
+      <c r="C14" s="47" t="n">
         <v>920.9</v>
       </c>
-      <c r="D14" s="45" t="n">
+      <c r="D14" s="47" t="n">
         <v>2.6</v>
       </c>
-      <c r="E14" s="45" t="n">
+      <c r="E14" s="47" t="n">
         <v>379.5</v>
       </c>
-      <c r="F14" s="45" t="n">
+      <c r="F14" s="47" t="n">
         <v>56.8</v>
       </c>
-      <c r="G14" s="45" t="n">
+      <c r="G14" s="47" t="n">
         <v>398</v>
       </c>
       <c r="H14" s="29" t="n">
         <v>62.34</v>
       </c>
-      <c r="I14" s="35"/>
-      <c r="J14" s="35"/>
-      <c r="K14" s="36" t="str">
+      <c r="I14" s="48"/>
+      <c r="J14" s="48"/>
+      <c r="K14" s="40" t="str">
         <f aca="false">IF(J14="","",ABS(J14-H14)/H14)</f>
         <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="38" t="n">
+      <c r="B15" s="42" t="n">
         <v>8</v>
       </c>
-      <c r="C15" s="45" t="n">
+      <c r="C15" s="47" t="n">
         <v>903.2</v>
       </c>
-      <c r="D15" s="45" t="n">
+      <c r="D15" s="47" t="n">
         <v>4.2</v>
       </c>
-      <c r="E15" s="45" t="n">
+      <c r="E15" s="47" t="n">
         <v>355.9</v>
       </c>
-      <c r="F15" s="45" t="n">
+      <c r="F15" s="47" t="n">
         <v>56.3</v>
       </c>
-      <c r="G15" s="45" t="n">
+      <c r="G15" s="47" t="n">
         <v>374</v>
       </c>
       <c r="H15" s="29" t="n">
         <v>63.82</v>
       </c>
-      <c r="I15" s="35"/>
-      <c r="J15" s="35"/>
-      <c r="K15" s="36" t="str">
+      <c r="I15" s="48"/>
+      <c r="J15" s="48"/>
+      <c r="K15" s="40" t="str">
         <f aca="false">IF(J15="","",ABS(J15-H15)/H15)</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="38" t="n">
+      <c r="B16" s="42" t="n">
         <v>9</v>
       </c>
-      <c r="C16" s="45" t="n">
+      <c r="C16" s="47" t="n">
         <v>920.9</v>
       </c>
-      <c r="D16" s="45" t="n">
+      <c r="D16" s="47" t="n">
         <v>2.6</v>
       </c>
-      <c r="E16" s="45" t="n">
+      <c r="E16" s="47" t="n">
         <v>379.5</v>
       </c>
-      <c r="F16" s="45" t="n">
+      <c r="F16" s="47" t="n">
         <v>56.8</v>
       </c>
-      <c r="G16" s="45" t="n">
+      <c r="G16" s="47" t="n">
         <v>398</v>
       </c>
       <c r="H16" s="29" t="n">
         <v>62.34</v>
       </c>
-      <c r="I16" s="35"/>
-      <c r="J16" s="35"/>
-      <c r="K16" s="36" t="str">
+      <c r="I16" s="48"/>
+      <c r="J16" s="48"/>
+      <c r="K16" s="40" t="str">
         <f aca="false">IF(J16="","",ABS(J16-H16)/H16)</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="12" t="s">
-        <v>184</v>
+        <v>209</v>
       </c>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>
@@ -3857,1296 +5898,4 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="true"/>
-  </sheetPr>
-  <dimension ref="B2:R37"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="8" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="12" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="3"/>
-  </cols>
-  <sheetData>
-    <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="12" t="s">
-        <v>186</v>
-      </c>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-      <c r="L3" s="12"/>
-      <c r="M3" s="12"/>
-      <c r="N3" s="12"/>
-      <c r="O3" s="12"/>
-      <c r="P3" s="12"/>
-      <c r="Q3" s="12"/>
-      <c r="R3" s="12"/>
-    </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="46" t="s">
-        <v>187</v>
-      </c>
-      <c r="C5" s="46"/>
-      <c r="D5" s="46"/>
-      <c r="E5" s="46"/>
-      <c r="F5" s="46"/>
-      <c r="G5" s="35"/>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="46" t="s">
-        <v>188</v>
-      </c>
-      <c r="C6" s="46"/>
-      <c r="D6" s="46"/>
-      <c r="E6" s="46"/>
-      <c r="F6" s="46"/>
-      <c r="G6" s="35"/>
-    </row>
-    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="K8" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="L8" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="M8" s="6" t="s">
-        <v>200</v>
-      </c>
-      <c r="N8" s="6" t="s">
-        <v>201</v>
-      </c>
-      <c r="O8" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="P8" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="Q8" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="R8" s="6" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="38" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" s="29" t="n">
-        <v>3.03</v>
-      </c>
-      <c r="D9" s="29" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="E9" s="29" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="F9" s="11" t="s">
-        <v>206</v>
-      </c>
-      <c r="G9" s="45" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H9" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="I9" s="38" t="n">
-        <v>15</v>
-      </c>
-      <c r="J9" s="45" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="K9" s="45" t="n">
-        <v>13.8</v>
-      </c>
-      <c r="L9" s="35"/>
-      <c r="M9" s="35"/>
-      <c r="N9" s="26" t="str">
-        <f aca="false">IF(OR(L9="",M9="",$G$5="",$G$6=""),"",(L9/$G$5)/(M9/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O9" s="35"/>
-      <c r="P9" s="35"/>
-      <c r="Q9" s="35"/>
-      <c r="R9" s="35"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="38" t="n">
-        <v>2</v>
-      </c>
-      <c r="C10" s="29" t="n">
-        <v>3.03</v>
-      </c>
-      <c r="D10" s="29" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="E10" s="29" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="F10" s="11" t="s">
-        <v>207</v>
-      </c>
-      <c r="G10" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="I10" s="38" t="n">
-        <v>15</v>
-      </c>
-      <c r="J10" s="45" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="K10" s="45" t="n">
-        <v>12.6</v>
-      </c>
-      <c r="L10" s="35"/>
-      <c r="M10" s="35"/>
-      <c r="N10" s="26" t="str">
-        <f aca="false">IF(OR(L10="",M10="",$G$5="",$G$6=""),"",(L10/$G$5)/(M10/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O10" s="35"/>
-      <c r="P10" s="35"/>
-      <c r="Q10" s="35"/>
-      <c r="R10" s="35"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="38" t="n">
-        <v>3</v>
-      </c>
-      <c r="C11" s="29" t="n">
-        <v>3.03</v>
-      </c>
-      <c r="D11" s="29" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="E11" s="29" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="F11" s="11" t="s">
-        <v>208</v>
-      </c>
-      <c r="G11" s="45" t="n">
-        <v>2</v>
-      </c>
-      <c r="H11" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="I11" s="38" t="n">
-        <v>15</v>
-      </c>
-      <c r="J11" s="45" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="K11" s="45" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="L11" s="35"/>
-      <c r="M11" s="35"/>
-      <c r="N11" s="26" t="str">
-        <f aca="false">IF(OR(L11="",M11="",$G$5="",$G$6=""),"",(L11/$G$5)/(M11/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O11" s="35"/>
-      <c r="P11" s="35"/>
-      <c r="Q11" s="35"/>
-      <c r="R11" s="35"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="38" t="n">
-        <v>4</v>
-      </c>
-      <c r="C12" s="29" t="n">
-        <v>3.03</v>
-      </c>
-      <c r="D12" s="29" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="E12" s="29" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="F12" s="11" t="s">
-        <v>207</v>
-      </c>
-      <c r="G12" s="45" t="n">
-        <v>2</v>
-      </c>
-      <c r="H12" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="I12" s="38" t="n">
-        <v>25</v>
-      </c>
-      <c r="J12" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" s="45" t="n">
-        <v>23</v>
-      </c>
-      <c r="L12" s="35"/>
-      <c r="M12" s="35"/>
-      <c r="N12" s="26" t="str">
-        <f aca="false">IF(OR(L12="",M12="",$G$5="",$G$6=""),"",(L12/$G$5)/(M12/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O12" s="35"/>
-      <c r="P12" s="35"/>
-      <c r="Q12" s="35"/>
-      <c r="R12" s="35"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="38" t="n">
-        <v>5</v>
-      </c>
-      <c r="C13" s="29" t="n">
-        <v>3.03</v>
-      </c>
-      <c r="D13" s="29" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="E13" s="29" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="F13" s="11" t="s">
-        <v>208</v>
-      </c>
-      <c r="G13" s="45" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H13" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="I13" s="38" t="n">
-        <v>25</v>
-      </c>
-      <c r="J13" s="45" t="n">
-        <v>2</v>
-      </c>
-      <c r="K13" s="45" t="n">
-        <v>21</v>
-      </c>
-      <c r="L13" s="35"/>
-      <c r="M13" s="35"/>
-      <c r="N13" s="26" t="str">
-        <f aca="false">IF(OR(L13="",M13="",$G$5="",$G$6=""),"",(L13/$G$5)/(M13/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O13" s="35"/>
-      <c r="P13" s="35"/>
-      <c r="Q13" s="35"/>
-      <c r="R13" s="35"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="38" t="n">
-        <v>6</v>
-      </c>
-      <c r="C14" s="29" t="n">
-        <v>3.03</v>
-      </c>
-      <c r="D14" s="29" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="E14" s="29" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="F14" s="11" t="s">
-        <v>206</v>
-      </c>
-      <c r="G14" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="H14" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="I14" s="38" t="n">
-        <v>25</v>
-      </c>
-      <c r="J14" s="45" t="n">
-        <v>3</v>
-      </c>
-      <c r="K14" s="45" t="n">
-        <v>19</v>
-      </c>
-      <c r="L14" s="35"/>
-      <c r="M14" s="35"/>
-      <c r="N14" s="26" t="str">
-        <f aca="false">IF(OR(L14="",M14="",$G$5="",$G$6=""),"",(L14/$G$5)/(M14/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O14" s="35"/>
-      <c r="P14" s="35"/>
-      <c r="Q14" s="35"/>
-      <c r="R14" s="35"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="38" t="n">
-        <v>7</v>
-      </c>
-      <c r="C15" s="29" t="n">
-        <v>3.03</v>
-      </c>
-      <c r="D15" s="29" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="E15" s="29" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="F15" s="11" t="s">
-        <v>208</v>
-      </c>
-      <c r="G15" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="H15" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="I15" s="38" t="n">
-        <v>35</v>
-      </c>
-      <c r="J15" s="45" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="K15" s="45" t="n">
-        <v>32.2</v>
-      </c>
-      <c r="L15" s="35"/>
-      <c r="M15" s="35"/>
-      <c r="N15" s="26" t="str">
-        <f aca="false">IF(OR(L15="",M15="",$G$5="",$G$6=""),"",(L15/$G$5)/(M15/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O15" s="35"/>
-      <c r="P15" s="35"/>
-      <c r="Q15" s="35"/>
-      <c r="R15" s="35"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="38" t="n">
-        <v>8</v>
-      </c>
-      <c r="C16" s="29" t="n">
-        <v>3.03</v>
-      </c>
-      <c r="D16" s="29" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="E16" s="29" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="F16" s="11" t="s">
-        <v>206</v>
-      </c>
-      <c r="G16" s="45" t="n">
-        <v>2</v>
-      </c>
-      <c r="H16" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="I16" s="38" t="n">
-        <v>35</v>
-      </c>
-      <c r="J16" s="45" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K16" s="45" t="n">
-        <v>29.4</v>
-      </c>
-      <c r="L16" s="35"/>
-      <c r="M16" s="35"/>
-      <c r="N16" s="26" t="str">
-        <f aca="false">IF(OR(L16="",M16="",$G$5="",$G$6=""),"",(L16/$G$5)/(M16/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O16" s="35"/>
-      <c r="P16" s="35"/>
-      <c r="Q16" s="35"/>
-      <c r="R16" s="35"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="38" t="n">
-        <v>9</v>
-      </c>
-      <c r="C17" s="29" t="n">
-        <v>3.03</v>
-      </c>
-      <c r="D17" s="29" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="E17" s="29" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="F17" s="11" t="s">
-        <v>207</v>
-      </c>
-      <c r="G17" s="45" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H17" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="I17" s="38" t="n">
-        <v>35</v>
-      </c>
-      <c r="J17" s="45" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="K17" s="45" t="n">
-        <v>26.6</v>
-      </c>
-      <c r="L17" s="35"/>
-      <c r="M17" s="35"/>
-      <c r="N17" s="26" t="str">
-        <f aca="false">IF(OR(L17="",M17="",$G$5="",$G$6=""),"",(L17/$G$5)/(M17/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O17" s="35"/>
-      <c r="P17" s="35"/>
-      <c r="Q17" s="35"/>
-      <c r="R17" s="35"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="38" t="n">
-        <v>10</v>
-      </c>
-      <c r="C18" s="29" t="n">
-        <v>4.55</v>
-      </c>
-      <c r="D18" s="29" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="E18" s="29" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="F18" s="11" t="s">
-        <v>207</v>
-      </c>
-      <c r="G18" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="H18" s="38" t="n">
-        <v>300</v>
-      </c>
-      <c r="I18" s="38" t="n">
-        <v>15</v>
-      </c>
-      <c r="J18" s="45" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="K18" s="45" t="n">
-        <v>13.8</v>
-      </c>
-      <c r="L18" s="35"/>
-      <c r="M18" s="35"/>
-      <c r="N18" s="26" t="str">
-        <f aca="false">IF(OR(L18="",M18="",$G$5="",$G$6=""),"",(L18/$G$5)/(M18/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O18" s="35"/>
-      <c r="P18" s="35"/>
-      <c r="Q18" s="35"/>
-      <c r="R18" s="35"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="38" t="n">
-        <v>11</v>
-      </c>
-      <c r="C19" s="29" t="n">
-        <v>4.55</v>
-      </c>
-      <c r="D19" s="29" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="E19" s="29" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="F19" s="11" t="s">
-        <v>208</v>
-      </c>
-      <c r="G19" s="45" t="n">
-        <v>2</v>
-      </c>
-      <c r="H19" s="38" t="n">
-        <v>300</v>
-      </c>
-      <c r="I19" s="38" t="n">
-        <v>15</v>
-      </c>
-      <c r="J19" s="45" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="K19" s="45" t="n">
-        <v>12.6</v>
-      </c>
-      <c r="L19" s="35"/>
-      <c r="M19" s="35"/>
-      <c r="N19" s="26" t="str">
-        <f aca="false">IF(OR(L19="",M19="",$G$5="",$G$6=""),"",(L19/$G$5)/(M19/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O19" s="35"/>
-      <c r="P19" s="35"/>
-      <c r="Q19" s="35"/>
-      <c r="R19" s="35"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="38" t="n">
-        <v>12</v>
-      </c>
-      <c r="C20" s="29" t="n">
-        <v>4.55</v>
-      </c>
-      <c r="D20" s="29" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="E20" s="29" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="F20" s="11" t="s">
-        <v>206</v>
-      </c>
-      <c r="G20" s="45" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H20" s="38" t="n">
-        <v>300</v>
-      </c>
-      <c r="I20" s="38" t="n">
-        <v>15</v>
-      </c>
-      <c r="J20" s="45" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="K20" s="45" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="L20" s="35"/>
-      <c r="M20" s="35"/>
-      <c r="N20" s="26" t="str">
-        <f aca="false">IF(OR(L20="",M20="",$G$5="",$G$6=""),"",(L20/$G$5)/(M20/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O20" s="35"/>
-      <c r="P20" s="35"/>
-      <c r="Q20" s="35"/>
-      <c r="R20" s="35"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="38" t="n">
-        <v>13</v>
-      </c>
-      <c r="C21" s="29" t="n">
-        <v>4.55</v>
-      </c>
-      <c r="D21" s="29" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="E21" s="29" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="F21" s="11" t="s">
-        <v>208</v>
-      </c>
-      <c r="G21" s="45" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H21" s="38" t="n">
-        <v>300</v>
-      </c>
-      <c r="I21" s="38" t="n">
-        <v>25</v>
-      </c>
-      <c r="J21" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="K21" s="45" t="n">
-        <v>23</v>
-      </c>
-      <c r="L21" s="35"/>
-      <c r="M21" s="35"/>
-      <c r="N21" s="26" t="str">
-        <f aca="false">IF(OR(L21="",M21="",$G$5="",$G$6=""),"",(L21/$G$5)/(M21/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O21" s="35"/>
-      <c r="P21" s="35"/>
-      <c r="Q21" s="35"/>
-      <c r="R21" s="35"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="38" t="n">
-        <v>14</v>
-      </c>
-      <c r="C22" s="29" t="n">
-        <v>4.55</v>
-      </c>
-      <c r="D22" s="29" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="E22" s="29" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="F22" s="11" t="s">
-        <v>206</v>
-      </c>
-      <c r="G22" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="H22" s="38" t="n">
-        <v>300</v>
-      </c>
-      <c r="I22" s="38" t="n">
-        <v>25</v>
-      </c>
-      <c r="J22" s="45" t="n">
-        <v>2</v>
-      </c>
-      <c r="K22" s="45" t="n">
-        <v>21</v>
-      </c>
-      <c r="L22" s="35"/>
-      <c r="M22" s="35"/>
-      <c r="N22" s="26" t="str">
-        <f aca="false">IF(OR(L22="",M22="",$G$5="",$G$6=""),"",(L22/$G$5)/(M22/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O22" s="35"/>
-      <c r="P22" s="35"/>
-      <c r="Q22" s="35"/>
-      <c r="R22" s="35"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="38" t="n">
-        <v>15</v>
-      </c>
-      <c r="C23" s="29" t="n">
-        <v>4.55</v>
-      </c>
-      <c r="D23" s="29" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="E23" s="29" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="F23" s="11" t="s">
-        <v>207</v>
-      </c>
-      <c r="G23" s="45" t="n">
-        <v>2</v>
-      </c>
-      <c r="H23" s="38" t="n">
-        <v>300</v>
-      </c>
-      <c r="I23" s="38" t="n">
-        <v>25</v>
-      </c>
-      <c r="J23" s="45" t="n">
-        <v>3</v>
-      </c>
-      <c r="K23" s="45" t="n">
-        <v>19</v>
-      </c>
-      <c r="L23" s="35"/>
-      <c r="M23" s="35"/>
-      <c r="N23" s="26" t="str">
-        <f aca="false">IF(OR(L23="",M23="",$G$5="",$G$6=""),"",(L23/$G$5)/(M23/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O23" s="35"/>
-      <c r="P23" s="35"/>
-      <c r="Q23" s="35"/>
-      <c r="R23" s="35"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="38" t="n">
-        <v>16</v>
-      </c>
-      <c r="C24" s="29" t="n">
-        <v>4.55</v>
-      </c>
-      <c r="D24" s="29" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="E24" s="29" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="F24" s="11" t="s">
-        <v>206</v>
-      </c>
-      <c r="G24" s="45" t="n">
-        <v>2</v>
-      </c>
-      <c r="H24" s="38" t="n">
-        <v>300</v>
-      </c>
-      <c r="I24" s="38" t="n">
-        <v>35</v>
-      </c>
-      <c r="J24" s="45" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="K24" s="45" t="n">
-        <v>32.2</v>
-      </c>
-      <c r="L24" s="35"/>
-      <c r="M24" s="35"/>
-      <c r="N24" s="26" t="str">
-        <f aca="false">IF(OR(L24="",M24="",$G$5="",$G$6=""),"",(L24/$G$5)/(M24/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O24" s="35"/>
-      <c r="P24" s="35"/>
-      <c r="Q24" s="35"/>
-      <c r="R24" s="35"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="38" t="n">
-        <v>17</v>
-      </c>
-      <c r="C25" s="29" t="n">
-        <v>4.55</v>
-      </c>
-      <c r="D25" s="29" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="E25" s="29" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="F25" s="11" t="s">
-        <v>207</v>
-      </c>
-      <c r="G25" s="45" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H25" s="38" t="n">
-        <v>300</v>
-      </c>
-      <c r="I25" s="38" t="n">
-        <v>35</v>
-      </c>
-      <c r="J25" s="45" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K25" s="45" t="n">
-        <v>29.4</v>
-      </c>
-      <c r="L25" s="35"/>
-      <c r="M25" s="35"/>
-      <c r="N25" s="26" t="str">
-        <f aca="false">IF(OR(L25="",M25="",$G$5="",$G$6=""),"",(L25/$G$5)/(M25/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O25" s="35"/>
-      <c r="P25" s="35"/>
-      <c r="Q25" s="35"/>
-      <c r="R25" s="35"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="38" t="n">
-        <v>18</v>
-      </c>
-      <c r="C26" s="29" t="n">
-        <v>4.55</v>
-      </c>
-      <c r="D26" s="29" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="E26" s="29" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="F26" s="11" t="s">
-        <v>208</v>
-      </c>
-      <c r="G26" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="H26" s="38" t="n">
-        <v>300</v>
-      </c>
-      <c r="I26" s="38" t="n">
-        <v>35</v>
-      </c>
-      <c r="J26" s="45" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="K26" s="45" t="n">
-        <v>26.6</v>
-      </c>
-      <c r="L26" s="35"/>
-      <c r="M26" s="35"/>
-      <c r="N26" s="26" t="str">
-        <f aca="false">IF(OR(L26="",M26="",$G$5="",$G$6=""),"",(L26/$G$5)/(M26/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O26" s="35"/>
-      <c r="P26" s="35"/>
-      <c r="Q26" s="35"/>
-      <c r="R26" s="35"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="38" t="n">
-        <v>19</v>
-      </c>
-      <c r="C27" s="29" t="n">
-        <v>6.06</v>
-      </c>
-      <c r="D27" s="29" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="E27" s="29" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="F27" s="11" t="s">
-        <v>208</v>
-      </c>
-      <c r="G27" s="45" t="n">
-        <v>2</v>
-      </c>
-      <c r="H27" s="38" t="n">
-        <v>400</v>
-      </c>
-      <c r="I27" s="38" t="n">
-        <v>15</v>
-      </c>
-      <c r="J27" s="45" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="K27" s="45" t="n">
-        <v>13.8</v>
-      </c>
-      <c r="L27" s="35"/>
-      <c r="M27" s="35"/>
-      <c r="N27" s="26" t="str">
-        <f aca="false">IF(OR(L27="",M27="",$G$5="",$G$6=""),"",(L27/$G$5)/(M27/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O27" s="35"/>
-      <c r="P27" s="35"/>
-      <c r="Q27" s="35"/>
-      <c r="R27" s="35"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="38" t="n">
-        <v>20</v>
-      </c>
-      <c r="C28" s="29" t="n">
-        <v>6.06</v>
-      </c>
-      <c r="D28" s="29" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="E28" s="29" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="F28" s="11" t="s">
-        <v>206</v>
-      </c>
-      <c r="G28" s="45" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H28" s="38" t="n">
-        <v>400</v>
-      </c>
-      <c r="I28" s="38" t="n">
-        <v>15</v>
-      </c>
-      <c r="J28" s="45" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="K28" s="45" t="n">
-        <v>12.6</v>
-      </c>
-      <c r="L28" s="35"/>
-      <c r="M28" s="35"/>
-      <c r="N28" s="26" t="str">
-        <f aca="false">IF(OR(L28="",M28="",$G$5="",$G$6=""),"",(L28/$G$5)/(M28/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O28" s="35"/>
-      <c r="P28" s="35"/>
-      <c r="Q28" s="35"/>
-      <c r="R28" s="35"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="38" t="n">
-        <v>21</v>
-      </c>
-      <c r="C29" s="29" t="n">
-        <v>6.06</v>
-      </c>
-      <c r="D29" s="29" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="E29" s="29" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="F29" s="11" t="s">
-        <v>207</v>
-      </c>
-      <c r="G29" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="H29" s="38" t="n">
-        <v>400</v>
-      </c>
-      <c r="I29" s="38" t="n">
-        <v>15</v>
-      </c>
-      <c r="J29" s="45" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="K29" s="45" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="L29" s="35"/>
-      <c r="M29" s="35"/>
-      <c r="N29" s="26" t="str">
-        <f aca="false">IF(OR(L29="",M29="",$G$5="",$G$6=""),"",(L29/$G$5)/(M29/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O29" s="35"/>
-      <c r="P29" s="35"/>
-      <c r="Q29" s="35"/>
-      <c r="R29" s="35"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="38" t="n">
-        <v>22</v>
-      </c>
-      <c r="C30" s="29" t="n">
-        <v>6.06</v>
-      </c>
-      <c r="D30" s="29" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="E30" s="29" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="F30" s="11" t="s">
-        <v>206</v>
-      </c>
-      <c r="G30" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="H30" s="38" t="n">
-        <v>400</v>
-      </c>
-      <c r="I30" s="38" t="n">
-        <v>25</v>
-      </c>
-      <c r="J30" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="K30" s="45" t="n">
-        <v>23</v>
-      </c>
-      <c r="L30" s="35"/>
-      <c r="M30" s="35"/>
-      <c r="N30" s="26" t="str">
-        <f aca="false">IF(OR(L30="",M30="",$G$5="",$G$6=""),"",(L30/$G$5)/(M30/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O30" s="35"/>
-      <c r="P30" s="35"/>
-      <c r="Q30" s="35"/>
-      <c r="R30" s="35"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="38" t="n">
-        <v>23</v>
-      </c>
-      <c r="C31" s="29" t="n">
-        <v>6.06</v>
-      </c>
-      <c r="D31" s="29" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="E31" s="29" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="F31" s="11" t="s">
-        <v>207</v>
-      </c>
-      <c r="G31" s="45" t="n">
-        <v>2</v>
-      </c>
-      <c r="H31" s="38" t="n">
-        <v>400</v>
-      </c>
-      <c r="I31" s="38" t="n">
-        <v>25</v>
-      </c>
-      <c r="J31" s="45" t="n">
-        <v>2</v>
-      </c>
-      <c r="K31" s="45" t="n">
-        <v>21</v>
-      </c>
-      <c r="L31" s="35"/>
-      <c r="M31" s="35"/>
-      <c r="N31" s="26" t="str">
-        <f aca="false">IF(OR(L31="",M31="",$G$5="",$G$6=""),"",(L31/$G$5)/(M31/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O31" s="35"/>
-      <c r="P31" s="35"/>
-      <c r="Q31" s="35"/>
-      <c r="R31" s="35"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="38" t="n">
-        <v>24</v>
-      </c>
-      <c r="C32" s="29" t="n">
-        <v>6.06</v>
-      </c>
-      <c r="D32" s="29" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="E32" s="29" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="F32" s="11" t="s">
-        <v>208</v>
-      </c>
-      <c r="G32" s="45" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H32" s="38" t="n">
-        <v>400</v>
-      </c>
-      <c r="I32" s="38" t="n">
-        <v>25</v>
-      </c>
-      <c r="J32" s="45" t="n">
-        <v>3</v>
-      </c>
-      <c r="K32" s="45" t="n">
-        <v>19</v>
-      </c>
-      <c r="L32" s="35"/>
-      <c r="M32" s="35"/>
-      <c r="N32" s="26" t="str">
-        <f aca="false">IF(OR(L32="",M32="",$G$5="",$G$6=""),"",(L32/$G$5)/(M32/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O32" s="35"/>
-      <c r="P32" s="35"/>
-      <c r="Q32" s="35"/>
-      <c r="R32" s="35"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="38" t="n">
-        <v>25</v>
-      </c>
-      <c r="C33" s="29" t="n">
-        <v>6.06</v>
-      </c>
-      <c r="D33" s="29" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="E33" s="29" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="F33" s="11" t="s">
-        <v>207</v>
-      </c>
-      <c r="G33" s="45" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H33" s="38" t="n">
-        <v>400</v>
-      </c>
-      <c r="I33" s="38" t="n">
-        <v>35</v>
-      </c>
-      <c r="J33" s="45" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="K33" s="45" t="n">
-        <v>32.2</v>
-      </c>
-      <c r="L33" s="35"/>
-      <c r="M33" s="35"/>
-      <c r="N33" s="26" t="str">
-        <f aca="false">IF(OR(L33="",M33="",$G$5="",$G$6=""),"",(L33/$G$5)/(M33/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O33" s="35"/>
-      <c r="P33" s="35"/>
-      <c r="Q33" s="35"/>
-      <c r="R33" s="35"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="38" t="n">
-        <v>26</v>
-      </c>
-      <c r="C34" s="29" t="n">
-        <v>6.06</v>
-      </c>
-      <c r="D34" s="29" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="E34" s="29" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="F34" s="11" t="s">
-        <v>208</v>
-      </c>
-      <c r="G34" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="H34" s="38" t="n">
-        <v>400</v>
-      </c>
-      <c r="I34" s="38" t="n">
-        <v>35</v>
-      </c>
-      <c r="J34" s="45" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K34" s="45" t="n">
-        <v>29.4</v>
-      </c>
-      <c r="L34" s="35"/>
-      <c r="M34" s="35"/>
-      <c r="N34" s="26" t="str">
-        <f aca="false">IF(OR(L34="",M34="",$G$5="",$G$6=""),"",(L34/$G$5)/(M34/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O34" s="35"/>
-      <c r="P34" s="35"/>
-      <c r="Q34" s="35"/>
-      <c r="R34" s="35"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="38" t="n">
-        <v>27</v>
-      </c>
-      <c r="C35" s="29" t="n">
-        <v>6.06</v>
-      </c>
-      <c r="D35" s="29" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="E35" s="29" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="F35" s="11" t="s">
-        <v>206</v>
-      </c>
-      <c r="G35" s="45" t="n">
-        <v>2</v>
-      </c>
-      <c r="H35" s="38" t="n">
-        <v>400</v>
-      </c>
-      <c r="I35" s="38" t="n">
-        <v>35</v>
-      </c>
-      <c r="J35" s="45" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="K35" s="45" t="n">
-        <v>26.6</v>
-      </c>
-      <c r="L35" s="35"/>
-      <c r="M35" s="35"/>
-      <c r="N35" s="26" t="str">
-        <f aca="false">IF(OR(L35="",M35="",$G$5="",$G$6=""),"",(L35/$G$5)/(M35/$G$6)^(1/3))</f>
-        <v/>
-      </c>
-      <c r="O35" s="35"/>
-      <c r="P35" s="35"/>
-      <c r="Q35" s="35"/>
-      <c r="R35" s="35"/>
-    </row>
-    <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="12" t="s">
-        <v>209</v>
-      </c>
-      <c r="C37" s="12"/>
-      <c r="D37" s="12"/>
-      <c r="E37" s="12"/>
-      <c r="F37" s="12"/>
-      <c r="G37" s="12"/>
-      <c r="H37" s="12"/>
-      <c r="I37" s="12"/>
-      <c r="J37" s="12"/>
-      <c r="K37" s="12"/>
-      <c r="L37" s="12"/>
-      <c r="M37" s="12"/>
-      <c r="N37" s="12"/>
-      <c r="O37" s="12"/>
-      <c r="P37" s="12"/>
-      <c r="Q37" s="12"/>
-      <c r="R37" s="12"/>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="B3:R3"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B37:R37"/>
-  </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add convergence ratio/classification gate; enter Fine+Medium GCI results
Convergence ratio R = e21/e32 now classifies each GCI block as
monotonic convergence (GCI valid), monotonic divergence, or
oscillatory (both invalid) before the apparent-order/GCI% numbers
are computed, so a negative or unphysical apparent order can't be
misread as a passing GCI%.

All three GCI mesh results now entered in Results Calculator:
Fine Nu=648.99/f=0.01923, Medium Nu=537.48/f=0.01704,
Coarse Nu=511.69/f=0.01723. Both Nu and f classify as FAIL
(monotonic divergence for Nu, oscillatory for f) with this data.
</commit_message>
<xml_diff>
--- a/thesis/mesh-validation/Mesh_and_Validation_Workbook.xlsx
+++ b/thesis/mesh-validation/Mesh_and_Validation_Workbook.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="236">
   <si>
     <t xml:space="preserve">PTSC-HTSP Thesis — Meshing &amp; Validation Workbook</t>
   </si>
@@ -617,6 +617,12 @@
     <t xml:space="preserve">ε32 = φ3 - φ2</t>
   </si>
   <si>
+    <t xml:space="preserve">Convergence ratio, R = ε21 / ε32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Convergence classification</t>
+  </si>
+  <si>
     <t xml:space="preserve">Apparent order, p  =  ln|ε32/ε21| / ln(r)
 (exact when r21≈r32, valid here by construction)</t>
   </si>
@@ -633,7 +639,7 @@
     <t xml:space="preserve">GCI_fine (%) = 1.25 · e_a21 / (r21^p - 1) × 100</t>
   </si>
   <si>
-    <t xml:space="preserve">Mesh-independent if GCI_fine &lt; ~1% (CLAUDE.md threshold) to ~2% (roadmap threshold). If it fails, your Fine mesh becomes the new Coarse and you add a finer 4th level.</t>
+    <t xml:space="preserve">Check Convergence classification above FIRST. If it says FAIL, the apparent order p and GCI% here are mathematical artifacts (a negative or unphysical p), not a real result -- do not use them to claim mesh independence. If it says PASS, mesh-independent when GCI_fine &lt; ~1% (CLAUDE.md threshold) to ~2% (roadmap threshold); if it fails, your Fine mesh becomes the new Coarse and you add a finer 4th level.</t>
   </si>
   <si>
     <t xml:space="preserve">Friction Factor (f) Mesh Independence</t>
@@ -972,7 +978,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="52">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1155,6 +1161,14 @@
     </xf>
     <xf numFmtId="175" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="175" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
@@ -1622,12 +1636,12 @@
   <sheetData>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="12" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -1647,76 +1661,76 @@
       <c r="R3" s="12"/>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="49" t="s">
-        <v>212</v>
-      </c>
-      <c r="C5" s="49"/>
-      <c r="D5" s="49"/>
-      <c r="E5" s="49"/>
-      <c r="F5" s="49"/>
-      <c r="G5" s="48"/>
+      <c r="B5" s="51" t="s">
+        <v>214</v>
+      </c>
+      <c r="C5" s="51"/>
+      <c r="D5" s="51"/>
+      <c r="E5" s="51"/>
+      <c r="F5" s="51"/>
+      <c r="G5" s="50"/>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="49" t="s">
-        <v>213</v>
-      </c>
-      <c r="C6" s="49"/>
-      <c r="D6" s="49"/>
-      <c r="E6" s="49"/>
-      <c r="F6" s="49"/>
-      <c r="G6" s="48"/>
+      <c r="B6" s="51" t="s">
+        <v>215</v>
+      </c>
+      <c r="C6" s="51"/>
+      <c r="D6" s="51"/>
+      <c r="E6" s="51"/>
+      <c r="F6" s="51"/>
+      <c r="G6" s="50"/>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
         <v>124</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="N8" s="6" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="O8" s="6" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="P8" s="6" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="Q8" s="6" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="R8" s="6" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1733,9 +1747,9 @@
         <v>0.04</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>230</v>
-      </c>
-      <c r="G9" s="47" t="n">
+        <v>232</v>
+      </c>
+      <c r="G9" s="49" t="n">
         <v>0.5</v>
       </c>
       <c r="H9" s="42" t="n">
@@ -1744,22 +1758,22 @@
       <c r="I9" s="42" t="n">
         <v>15</v>
       </c>
-      <c r="J9" s="47" t="n">
+      <c r="J9" s="49" t="n">
         <v>0.6</v>
       </c>
-      <c r="K9" s="47" t="n">
+      <c r="K9" s="49" t="n">
         <v>13.8</v>
       </c>
-      <c r="L9" s="48"/>
-      <c r="M9" s="48"/>
+      <c r="L9" s="50"/>
+      <c r="M9" s="50"/>
       <c r="N9" s="26" t="str">
         <f aca="false">IF(OR(L9="",M9="",$G$5="",$G$6=""),"",(L9/$G$5)/(M9/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O9" s="48"/>
-      <c r="P9" s="48"/>
-      <c r="Q9" s="48"/>
-      <c r="R9" s="48"/>
+      <c r="O9" s="50"/>
+      <c r="P9" s="50"/>
+      <c r="Q9" s="50"/>
+      <c r="R9" s="50"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="42" t="n">
@@ -1775,9 +1789,9 @@
         <v>0.08</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>231</v>
-      </c>
-      <c r="G10" s="47" t="n">
+        <v>233</v>
+      </c>
+      <c r="G10" s="49" t="n">
         <v>1</v>
       </c>
       <c r="H10" s="42" t="n">
@@ -1786,22 +1800,22 @@
       <c r="I10" s="42" t="n">
         <v>15</v>
       </c>
-      <c r="J10" s="47" t="n">
+      <c r="J10" s="49" t="n">
         <v>1.2</v>
       </c>
-      <c r="K10" s="47" t="n">
+      <c r="K10" s="49" t="n">
         <v>12.6</v>
       </c>
-      <c r="L10" s="48"/>
-      <c r="M10" s="48"/>
+      <c r="L10" s="50"/>
+      <c r="M10" s="50"/>
       <c r="N10" s="26" t="str">
         <f aca="false">IF(OR(L10="",M10="",$G$5="",$G$6=""),"",(L10/$G$5)/(M10/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O10" s="48"/>
-      <c r="P10" s="48"/>
-      <c r="Q10" s="48"/>
-      <c r="R10" s="48"/>
+      <c r="O10" s="50"/>
+      <c r="P10" s="50"/>
+      <c r="Q10" s="50"/>
+      <c r="R10" s="50"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="42" t="n">
@@ -1817,9 +1831,9 @@
         <v>0.12</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>232</v>
-      </c>
-      <c r="G11" s="47" t="n">
+        <v>234</v>
+      </c>
+      <c r="G11" s="49" t="n">
         <v>2</v>
       </c>
       <c r="H11" s="42" t="n">
@@ -1828,22 +1842,22 @@
       <c r="I11" s="42" t="n">
         <v>15</v>
       </c>
-      <c r="J11" s="47" t="n">
+      <c r="J11" s="49" t="n">
         <v>1.8</v>
       </c>
-      <c r="K11" s="47" t="n">
+      <c r="K11" s="49" t="n">
         <v>11.4</v>
       </c>
-      <c r="L11" s="48"/>
-      <c r="M11" s="48"/>
+      <c r="L11" s="50"/>
+      <c r="M11" s="50"/>
       <c r="N11" s="26" t="str">
         <f aca="false">IF(OR(L11="",M11="",$G$5="",$G$6=""),"",(L11/$G$5)/(M11/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O11" s="48"/>
-      <c r="P11" s="48"/>
-      <c r="Q11" s="48"/>
-      <c r="R11" s="48"/>
+      <c r="O11" s="50"/>
+      <c r="P11" s="50"/>
+      <c r="Q11" s="50"/>
+      <c r="R11" s="50"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="42" t="n">
@@ -1859,9 +1873,9 @@
         <v>0.04</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>231</v>
-      </c>
-      <c r="G12" s="47" t="n">
+        <v>233</v>
+      </c>
+      <c r="G12" s="49" t="n">
         <v>2</v>
       </c>
       <c r="H12" s="42" t="n">
@@ -1870,22 +1884,22 @@
       <c r="I12" s="42" t="n">
         <v>25</v>
       </c>
-      <c r="J12" s="47" t="n">
+      <c r="J12" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="K12" s="47" t="n">
+      <c r="K12" s="49" t="n">
         <v>23</v>
       </c>
-      <c r="L12" s="48"/>
-      <c r="M12" s="48"/>
+      <c r="L12" s="50"/>
+      <c r="M12" s="50"/>
       <c r="N12" s="26" t="str">
         <f aca="false">IF(OR(L12="",M12="",$G$5="",$G$6=""),"",(L12/$G$5)/(M12/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O12" s="48"/>
-      <c r="P12" s="48"/>
-      <c r="Q12" s="48"/>
-      <c r="R12" s="48"/>
+      <c r="O12" s="50"/>
+      <c r="P12" s="50"/>
+      <c r="Q12" s="50"/>
+      <c r="R12" s="50"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="42" t="n">
@@ -1901,9 +1915,9 @@
         <v>0.08</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>232</v>
-      </c>
-      <c r="G13" s="47" t="n">
+        <v>234</v>
+      </c>
+      <c r="G13" s="49" t="n">
         <v>0.5</v>
       </c>
       <c r="H13" s="42" t="n">
@@ -1912,22 +1926,22 @@
       <c r="I13" s="42" t="n">
         <v>25</v>
       </c>
-      <c r="J13" s="47" t="n">
+      <c r="J13" s="49" t="n">
         <v>2</v>
       </c>
-      <c r="K13" s="47" t="n">
+      <c r="K13" s="49" t="n">
         <v>21</v>
       </c>
-      <c r="L13" s="48"/>
-      <c r="M13" s="48"/>
+      <c r="L13" s="50"/>
+      <c r="M13" s="50"/>
       <c r="N13" s="26" t="str">
         <f aca="false">IF(OR(L13="",M13="",$G$5="",$G$6=""),"",(L13/$G$5)/(M13/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O13" s="48"/>
-      <c r="P13" s="48"/>
-      <c r="Q13" s="48"/>
-      <c r="R13" s="48"/>
+      <c r="O13" s="50"/>
+      <c r="P13" s="50"/>
+      <c r="Q13" s="50"/>
+      <c r="R13" s="50"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="42" t="n">
@@ -1943,9 +1957,9 @@
         <v>0.12</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>230</v>
-      </c>
-      <c r="G14" s="47" t="n">
+        <v>232</v>
+      </c>
+      <c r="G14" s="49" t="n">
         <v>1</v>
       </c>
       <c r="H14" s="42" t="n">
@@ -1954,22 +1968,22 @@
       <c r="I14" s="42" t="n">
         <v>25</v>
       </c>
-      <c r="J14" s="47" t="n">
+      <c r="J14" s="49" t="n">
         <v>3</v>
       </c>
-      <c r="K14" s="47" t="n">
+      <c r="K14" s="49" t="n">
         <v>19</v>
       </c>
-      <c r="L14" s="48"/>
-      <c r="M14" s="48"/>
+      <c r="L14" s="50"/>
+      <c r="M14" s="50"/>
       <c r="N14" s="26" t="str">
         <f aca="false">IF(OR(L14="",M14="",$G$5="",$G$6=""),"",(L14/$G$5)/(M14/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O14" s="48"/>
-      <c r="P14" s="48"/>
-      <c r="Q14" s="48"/>
-      <c r="R14" s="48"/>
+      <c r="O14" s="50"/>
+      <c r="P14" s="50"/>
+      <c r="Q14" s="50"/>
+      <c r="R14" s="50"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="42" t="n">
@@ -1985,9 +1999,9 @@
         <v>0.04</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>232</v>
-      </c>
-      <c r="G15" s="47" t="n">
+        <v>234</v>
+      </c>
+      <c r="G15" s="49" t="n">
         <v>1</v>
       </c>
       <c r="H15" s="42" t="n">
@@ -1996,22 +2010,22 @@
       <c r="I15" s="42" t="n">
         <v>35</v>
       </c>
-      <c r="J15" s="47" t="n">
+      <c r="J15" s="49" t="n">
         <v>1.4</v>
       </c>
-      <c r="K15" s="47" t="n">
+      <c r="K15" s="49" t="n">
         <v>32.2</v>
       </c>
-      <c r="L15" s="48"/>
-      <c r="M15" s="48"/>
+      <c r="L15" s="50"/>
+      <c r="M15" s="50"/>
       <c r="N15" s="26" t="str">
         <f aca="false">IF(OR(L15="",M15="",$G$5="",$G$6=""),"",(L15/$G$5)/(M15/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O15" s="48"/>
-      <c r="P15" s="48"/>
-      <c r="Q15" s="48"/>
-      <c r="R15" s="48"/>
+      <c r="O15" s="50"/>
+      <c r="P15" s="50"/>
+      <c r="Q15" s="50"/>
+      <c r="R15" s="50"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="42" t="n">
@@ -2027,9 +2041,9 @@
         <v>0.08</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>230</v>
-      </c>
-      <c r="G16" s="47" t="n">
+        <v>232</v>
+      </c>
+      <c r="G16" s="49" t="n">
         <v>2</v>
       </c>
       <c r="H16" s="42" t="n">
@@ -2038,22 +2052,22 @@
       <c r="I16" s="42" t="n">
         <v>35</v>
       </c>
-      <c r="J16" s="47" t="n">
+      <c r="J16" s="49" t="n">
         <v>2.8</v>
       </c>
-      <c r="K16" s="47" t="n">
+      <c r="K16" s="49" t="n">
         <v>29.4</v>
       </c>
-      <c r="L16" s="48"/>
-      <c r="M16" s="48"/>
+      <c r="L16" s="50"/>
+      <c r="M16" s="50"/>
       <c r="N16" s="26" t="str">
         <f aca="false">IF(OR(L16="",M16="",$G$5="",$G$6=""),"",(L16/$G$5)/(M16/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O16" s="48"/>
-      <c r="P16" s="48"/>
-      <c r="Q16" s="48"/>
-      <c r="R16" s="48"/>
+      <c r="O16" s="50"/>
+      <c r="P16" s="50"/>
+      <c r="Q16" s="50"/>
+      <c r="R16" s="50"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="42" t="n">
@@ -2069,9 +2083,9 @@
         <v>0.12</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>231</v>
-      </c>
-      <c r="G17" s="47" t="n">
+        <v>233</v>
+      </c>
+      <c r="G17" s="49" t="n">
         <v>0.5</v>
       </c>
       <c r="H17" s="42" t="n">
@@ -2080,22 +2094,22 @@
       <c r="I17" s="42" t="n">
         <v>35</v>
       </c>
-      <c r="J17" s="47" t="n">
+      <c r="J17" s="49" t="n">
         <v>4.2</v>
       </c>
-      <c r="K17" s="47" t="n">
+      <c r="K17" s="49" t="n">
         <v>26.6</v>
       </c>
-      <c r="L17" s="48"/>
-      <c r="M17" s="48"/>
+      <c r="L17" s="50"/>
+      <c r="M17" s="50"/>
       <c r="N17" s="26" t="str">
         <f aca="false">IF(OR(L17="",M17="",$G$5="",$G$6=""),"",(L17/$G$5)/(M17/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O17" s="48"/>
-      <c r="P17" s="48"/>
-      <c r="Q17" s="48"/>
-      <c r="R17" s="48"/>
+      <c r="O17" s="50"/>
+      <c r="P17" s="50"/>
+      <c r="Q17" s="50"/>
+      <c r="R17" s="50"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="42" t="n">
@@ -2111,9 +2125,9 @@
         <v>0.04</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>231</v>
-      </c>
-      <c r="G18" s="47" t="n">
+        <v>233</v>
+      </c>
+      <c r="G18" s="49" t="n">
         <v>1</v>
       </c>
       <c r="H18" s="42" t="n">
@@ -2122,22 +2136,22 @@
       <c r="I18" s="42" t="n">
         <v>15</v>
       </c>
-      <c r="J18" s="47" t="n">
+      <c r="J18" s="49" t="n">
         <v>0.6</v>
       </c>
-      <c r="K18" s="47" t="n">
+      <c r="K18" s="49" t="n">
         <v>13.8</v>
       </c>
-      <c r="L18" s="48"/>
-      <c r="M18" s="48"/>
+      <c r="L18" s="50"/>
+      <c r="M18" s="50"/>
       <c r="N18" s="26" t="str">
         <f aca="false">IF(OR(L18="",M18="",$G$5="",$G$6=""),"",(L18/$G$5)/(M18/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O18" s="48"/>
-      <c r="P18" s="48"/>
-      <c r="Q18" s="48"/>
-      <c r="R18" s="48"/>
+      <c r="O18" s="50"/>
+      <c r="P18" s="50"/>
+      <c r="Q18" s="50"/>
+      <c r="R18" s="50"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="42" t="n">
@@ -2153,9 +2167,9 @@
         <v>0.08</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>232</v>
-      </c>
-      <c r="G19" s="47" t="n">
+        <v>234</v>
+      </c>
+      <c r="G19" s="49" t="n">
         <v>2</v>
       </c>
       <c r="H19" s="42" t="n">
@@ -2164,22 +2178,22 @@
       <c r="I19" s="42" t="n">
         <v>15</v>
       </c>
-      <c r="J19" s="47" t="n">
+      <c r="J19" s="49" t="n">
         <v>1.2</v>
       </c>
-      <c r="K19" s="47" t="n">
+      <c r="K19" s="49" t="n">
         <v>12.6</v>
       </c>
-      <c r="L19" s="48"/>
-      <c r="M19" s="48"/>
+      <c r="L19" s="50"/>
+      <c r="M19" s="50"/>
       <c r="N19" s="26" t="str">
         <f aca="false">IF(OR(L19="",M19="",$G$5="",$G$6=""),"",(L19/$G$5)/(M19/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O19" s="48"/>
-      <c r="P19" s="48"/>
-      <c r="Q19" s="48"/>
-      <c r="R19" s="48"/>
+      <c r="O19" s="50"/>
+      <c r="P19" s="50"/>
+      <c r="Q19" s="50"/>
+      <c r="R19" s="50"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="42" t="n">
@@ -2195,9 +2209,9 @@
         <v>0.12</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>230</v>
-      </c>
-      <c r="G20" s="47" t="n">
+        <v>232</v>
+      </c>
+      <c r="G20" s="49" t="n">
         <v>0.5</v>
       </c>
       <c r="H20" s="42" t="n">
@@ -2206,22 +2220,22 @@
       <c r="I20" s="42" t="n">
         <v>15</v>
       </c>
-      <c r="J20" s="47" t="n">
+      <c r="J20" s="49" t="n">
         <v>1.8</v>
       </c>
-      <c r="K20" s="47" t="n">
+      <c r="K20" s="49" t="n">
         <v>11.4</v>
       </c>
-      <c r="L20" s="48"/>
-      <c r="M20" s="48"/>
+      <c r="L20" s="50"/>
+      <c r="M20" s="50"/>
       <c r="N20" s="26" t="str">
         <f aca="false">IF(OR(L20="",M20="",$G$5="",$G$6=""),"",(L20/$G$5)/(M20/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O20" s="48"/>
-      <c r="P20" s="48"/>
-      <c r="Q20" s="48"/>
-      <c r="R20" s="48"/>
+      <c r="O20" s="50"/>
+      <c r="P20" s="50"/>
+      <c r="Q20" s="50"/>
+      <c r="R20" s="50"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="42" t="n">
@@ -2237,9 +2251,9 @@
         <v>0.04</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>232</v>
-      </c>
-      <c r="G21" s="47" t="n">
+        <v>234</v>
+      </c>
+      <c r="G21" s="49" t="n">
         <v>0.5</v>
       </c>
       <c r="H21" s="42" t="n">
@@ -2248,22 +2262,22 @@
       <c r="I21" s="42" t="n">
         <v>25</v>
       </c>
-      <c r="J21" s="47" t="n">
+      <c r="J21" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="K21" s="47" t="n">
+      <c r="K21" s="49" t="n">
         <v>23</v>
       </c>
-      <c r="L21" s="48"/>
-      <c r="M21" s="48"/>
+      <c r="L21" s="50"/>
+      <c r="M21" s="50"/>
       <c r="N21" s="26" t="str">
         <f aca="false">IF(OR(L21="",M21="",$G$5="",$G$6=""),"",(L21/$G$5)/(M21/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O21" s="48"/>
-      <c r="P21" s="48"/>
-      <c r="Q21" s="48"/>
-      <c r="R21" s="48"/>
+      <c r="O21" s="50"/>
+      <c r="P21" s="50"/>
+      <c r="Q21" s="50"/>
+      <c r="R21" s="50"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="42" t="n">
@@ -2279,9 +2293,9 @@
         <v>0.08</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>230</v>
-      </c>
-      <c r="G22" s="47" t="n">
+        <v>232</v>
+      </c>
+      <c r="G22" s="49" t="n">
         <v>1</v>
       </c>
       <c r="H22" s="42" t="n">
@@ -2290,22 +2304,22 @@
       <c r="I22" s="42" t="n">
         <v>25</v>
       </c>
-      <c r="J22" s="47" t="n">
+      <c r="J22" s="49" t="n">
         <v>2</v>
       </c>
-      <c r="K22" s="47" t="n">
+      <c r="K22" s="49" t="n">
         <v>21</v>
       </c>
-      <c r="L22" s="48"/>
-      <c r="M22" s="48"/>
+      <c r="L22" s="50"/>
+      <c r="M22" s="50"/>
       <c r="N22" s="26" t="str">
         <f aca="false">IF(OR(L22="",M22="",$G$5="",$G$6=""),"",(L22/$G$5)/(M22/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O22" s="48"/>
-      <c r="P22" s="48"/>
-      <c r="Q22" s="48"/>
-      <c r="R22" s="48"/>
+      <c r="O22" s="50"/>
+      <c r="P22" s="50"/>
+      <c r="Q22" s="50"/>
+      <c r="R22" s="50"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="42" t="n">
@@ -2321,9 +2335,9 @@
         <v>0.12</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>231</v>
-      </c>
-      <c r="G23" s="47" t="n">
+        <v>233</v>
+      </c>
+      <c r="G23" s="49" t="n">
         <v>2</v>
       </c>
       <c r="H23" s="42" t="n">
@@ -2332,22 +2346,22 @@
       <c r="I23" s="42" t="n">
         <v>25</v>
       </c>
-      <c r="J23" s="47" t="n">
+      <c r="J23" s="49" t="n">
         <v>3</v>
       </c>
-      <c r="K23" s="47" t="n">
+      <c r="K23" s="49" t="n">
         <v>19</v>
       </c>
-      <c r="L23" s="48"/>
-      <c r="M23" s="48"/>
+      <c r="L23" s="50"/>
+      <c r="M23" s="50"/>
       <c r="N23" s="26" t="str">
         <f aca="false">IF(OR(L23="",M23="",$G$5="",$G$6=""),"",(L23/$G$5)/(M23/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O23" s="48"/>
-      <c r="P23" s="48"/>
-      <c r="Q23" s="48"/>
-      <c r="R23" s="48"/>
+      <c r="O23" s="50"/>
+      <c r="P23" s="50"/>
+      <c r="Q23" s="50"/>
+      <c r="R23" s="50"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="42" t="n">
@@ -2363,9 +2377,9 @@
         <v>0.04</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>230</v>
-      </c>
-      <c r="G24" s="47" t="n">
+        <v>232</v>
+      </c>
+      <c r="G24" s="49" t="n">
         <v>2</v>
       </c>
       <c r="H24" s="42" t="n">
@@ -2374,22 +2388,22 @@
       <c r="I24" s="42" t="n">
         <v>35</v>
       </c>
-      <c r="J24" s="47" t="n">
+      <c r="J24" s="49" t="n">
         <v>1.4</v>
       </c>
-      <c r="K24" s="47" t="n">
+      <c r="K24" s="49" t="n">
         <v>32.2</v>
       </c>
-      <c r="L24" s="48"/>
-      <c r="M24" s="48"/>
+      <c r="L24" s="50"/>
+      <c r="M24" s="50"/>
       <c r="N24" s="26" t="str">
         <f aca="false">IF(OR(L24="",M24="",$G$5="",$G$6=""),"",(L24/$G$5)/(M24/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O24" s="48"/>
-      <c r="P24" s="48"/>
-      <c r="Q24" s="48"/>
-      <c r="R24" s="48"/>
+      <c r="O24" s="50"/>
+      <c r="P24" s="50"/>
+      <c r="Q24" s="50"/>
+      <c r="R24" s="50"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="42" t="n">
@@ -2405,9 +2419,9 @@
         <v>0.08</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>231</v>
-      </c>
-      <c r="G25" s="47" t="n">
+        <v>233</v>
+      </c>
+      <c r="G25" s="49" t="n">
         <v>0.5</v>
       </c>
       <c r="H25" s="42" t="n">
@@ -2416,22 +2430,22 @@
       <c r="I25" s="42" t="n">
         <v>35</v>
       </c>
-      <c r="J25" s="47" t="n">
+      <c r="J25" s="49" t="n">
         <v>2.8</v>
       </c>
-      <c r="K25" s="47" t="n">
+      <c r="K25" s="49" t="n">
         <v>29.4</v>
       </c>
-      <c r="L25" s="48"/>
-      <c r="M25" s="48"/>
+      <c r="L25" s="50"/>
+      <c r="M25" s="50"/>
       <c r="N25" s="26" t="str">
         <f aca="false">IF(OR(L25="",M25="",$G$5="",$G$6=""),"",(L25/$G$5)/(M25/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O25" s="48"/>
-      <c r="P25" s="48"/>
-      <c r="Q25" s="48"/>
-      <c r="R25" s="48"/>
+      <c r="O25" s="50"/>
+      <c r="P25" s="50"/>
+      <c r="Q25" s="50"/>
+      <c r="R25" s="50"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="42" t="n">
@@ -2447,9 +2461,9 @@
         <v>0.12</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>232</v>
-      </c>
-      <c r="G26" s="47" t="n">
+        <v>234</v>
+      </c>
+      <c r="G26" s="49" t="n">
         <v>1</v>
       </c>
       <c r="H26" s="42" t="n">
@@ -2458,22 +2472,22 @@
       <c r="I26" s="42" t="n">
         <v>35</v>
       </c>
-      <c r="J26" s="47" t="n">
+      <c r="J26" s="49" t="n">
         <v>4.2</v>
       </c>
-      <c r="K26" s="47" t="n">
+      <c r="K26" s="49" t="n">
         <v>26.6</v>
       </c>
-      <c r="L26" s="48"/>
-      <c r="M26" s="48"/>
+      <c r="L26" s="50"/>
+      <c r="M26" s="50"/>
       <c r="N26" s="26" t="str">
         <f aca="false">IF(OR(L26="",M26="",$G$5="",$G$6=""),"",(L26/$G$5)/(M26/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O26" s="48"/>
-      <c r="P26" s="48"/>
-      <c r="Q26" s="48"/>
-      <c r="R26" s="48"/>
+      <c r="O26" s="50"/>
+      <c r="P26" s="50"/>
+      <c r="Q26" s="50"/>
+      <c r="R26" s="50"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="42" t="n">
@@ -2489,9 +2503,9 @@
         <v>0.04</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>232</v>
-      </c>
-      <c r="G27" s="47" t="n">
+        <v>234</v>
+      </c>
+      <c r="G27" s="49" t="n">
         <v>2</v>
       </c>
       <c r="H27" s="42" t="n">
@@ -2500,22 +2514,22 @@
       <c r="I27" s="42" t="n">
         <v>15</v>
       </c>
-      <c r="J27" s="47" t="n">
+      <c r="J27" s="49" t="n">
         <v>0.6</v>
       </c>
-      <c r="K27" s="47" t="n">
+      <c r="K27" s="49" t="n">
         <v>13.8</v>
       </c>
-      <c r="L27" s="48"/>
-      <c r="M27" s="48"/>
+      <c r="L27" s="50"/>
+      <c r="M27" s="50"/>
       <c r="N27" s="26" t="str">
         <f aca="false">IF(OR(L27="",M27="",$G$5="",$G$6=""),"",(L27/$G$5)/(M27/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O27" s="48"/>
-      <c r="P27" s="48"/>
-      <c r="Q27" s="48"/>
-      <c r="R27" s="48"/>
+      <c r="O27" s="50"/>
+      <c r="P27" s="50"/>
+      <c r="Q27" s="50"/>
+      <c r="R27" s="50"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="42" t="n">
@@ -2531,9 +2545,9 @@
         <v>0.08</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>230</v>
-      </c>
-      <c r="G28" s="47" t="n">
+        <v>232</v>
+      </c>
+      <c r="G28" s="49" t="n">
         <v>0.5</v>
       </c>
       <c r="H28" s="42" t="n">
@@ -2542,22 +2556,22 @@
       <c r="I28" s="42" t="n">
         <v>15</v>
       </c>
-      <c r="J28" s="47" t="n">
+      <c r="J28" s="49" t="n">
         <v>1.2</v>
       </c>
-      <c r="K28" s="47" t="n">
+      <c r="K28" s="49" t="n">
         <v>12.6</v>
       </c>
-      <c r="L28" s="48"/>
-      <c r="M28" s="48"/>
+      <c r="L28" s="50"/>
+      <c r="M28" s="50"/>
       <c r="N28" s="26" t="str">
         <f aca="false">IF(OR(L28="",M28="",$G$5="",$G$6=""),"",(L28/$G$5)/(M28/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O28" s="48"/>
-      <c r="P28" s="48"/>
-      <c r="Q28" s="48"/>
-      <c r="R28" s="48"/>
+      <c r="O28" s="50"/>
+      <c r="P28" s="50"/>
+      <c r="Q28" s="50"/>
+      <c r="R28" s="50"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="42" t="n">
@@ -2573,9 +2587,9 @@
         <v>0.12</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>231</v>
-      </c>
-      <c r="G29" s="47" t="n">
+        <v>233</v>
+      </c>
+      <c r="G29" s="49" t="n">
         <v>1</v>
       </c>
       <c r="H29" s="42" t="n">
@@ -2584,22 +2598,22 @@
       <c r="I29" s="42" t="n">
         <v>15</v>
       </c>
-      <c r="J29" s="47" t="n">
+      <c r="J29" s="49" t="n">
         <v>1.8</v>
       </c>
-      <c r="K29" s="47" t="n">
+      <c r="K29" s="49" t="n">
         <v>11.4</v>
       </c>
-      <c r="L29" s="48"/>
-      <c r="M29" s="48"/>
+      <c r="L29" s="50"/>
+      <c r="M29" s="50"/>
       <c r="N29" s="26" t="str">
         <f aca="false">IF(OR(L29="",M29="",$G$5="",$G$6=""),"",(L29/$G$5)/(M29/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O29" s="48"/>
-      <c r="P29" s="48"/>
-      <c r="Q29" s="48"/>
-      <c r="R29" s="48"/>
+      <c r="O29" s="50"/>
+      <c r="P29" s="50"/>
+      <c r="Q29" s="50"/>
+      <c r="R29" s="50"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="42" t="n">
@@ -2615,9 +2629,9 @@
         <v>0.04</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>230</v>
-      </c>
-      <c r="G30" s="47" t="n">
+        <v>232</v>
+      </c>
+      <c r="G30" s="49" t="n">
         <v>1</v>
       </c>
       <c r="H30" s="42" t="n">
@@ -2626,22 +2640,22 @@
       <c r="I30" s="42" t="n">
         <v>25</v>
       </c>
-      <c r="J30" s="47" t="n">
+      <c r="J30" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="K30" s="47" t="n">
+      <c r="K30" s="49" t="n">
         <v>23</v>
       </c>
-      <c r="L30" s="48"/>
-      <c r="M30" s="48"/>
+      <c r="L30" s="50"/>
+      <c r="M30" s="50"/>
       <c r="N30" s="26" t="str">
         <f aca="false">IF(OR(L30="",M30="",$G$5="",$G$6=""),"",(L30/$G$5)/(M30/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O30" s="48"/>
-      <c r="P30" s="48"/>
-      <c r="Q30" s="48"/>
-      <c r="R30" s="48"/>
+      <c r="O30" s="50"/>
+      <c r="P30" s="50"/>
+      <c r="Q30" s="50"/>
+      <c r="R30" s="50"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="42" t="n">
@@ -2657,9 +2671,9 @@
         <v>0.08</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>231</v>
-      </c>
-      <c r="G31" s="47" t="n">
+        <v>233</v>
+      </c>
+      <c r="G31" s="49" t="n">
         <v>2</v>
       </c>
       <c r="H31" s="42" t="n">
@@ -2668,22 +2682,22 @@
       <c r="I31" s="42" t="n">
         <v>25</v>
       </c>
-      <c r="J31" s="47" t="n">
+      <c r="J31" s="49" t="n">
         <v>2</v>
       </c>
-      <c r="K31" s="47" t="n">
+      <c r="K31" s="49" t="n">
         <v>21</v>
       </c>
-      <c r="L31" s="48"/>
-      <c r="M31" s="48"/>
+      <c r="L31" s="50"/>
+      <c r="M31" s="50"/>
       <c r="N31" s="26" t="str">
         <f aca="false">IF(OR(L31="",M31="",$G$5="",$G$6=""),"",(L31/$G$5)/(M31/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O31" s="48"/>
-      <c r="P31" s="48"/>
-      <c r="Q31" s="48"/>
-      <c r="R31" s="48"/>
+      <c r="O31" s="50"/>
+      <c r="P31" s="50"/>
+      <c r="Q31" s="50"/>
+      <c r="R31" s="50"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="42" t="n">
@@ -2699,9 +2713,9 @@
         <v>0.12</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>232</v>
-      </c>
-      <c r="G32" s="47" t="n">
+        <v>234</v>
+      </c>
+      <c r="G32" s="49" t="n">
         <v>0.5</v>
       </c>
       <c r="H32" s="42" t="n">
@@ -2710,22 +2724,22 @@
       <c r="I32" s="42" t="n">
         <v>25</v>
       </c>
-      <c r="J32" s="47" t="n">
+      <c r="J32" s="49" t="n">
         <v>3</v>
       </c>
-      <c r="K32" s="47" t="n">
+      <c r="K32" s="49" t="n">
         <v>19</v>
       </c>
-      <c r="L32" s="48"/>
-      <c r="M32" s="48"/>
+      <c r="L32" s="50"/>
+      <c r="M32" s="50"/>
       <c r="N32" s="26" t="str">
         <f aca="false">IF(OR(L32="",M32="",$G$5="",$G$6=""),"",(L32/$G$5)/(M32/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O32" s="48"/>
-      <c r="P32" s="48"/>
-      <c r="Q32" s="48"/>
-      <c r="R32" s="48"/>
+      <c r="O32" s="50"/>
+      <c r="P32" s="50"/>
+      <c r="Q32" s="50"/>
+      <c r="R32" s="50"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="42" t="n">
@@ -2741,9 +2755,9 @@
         <v>0.04</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>231</v>
-      </c>
-      <c r="G33" s="47" t="n">
+        <v>233</v>
+      </c>
+      <c r="G33" s="49" t="n">
         <v>0.5</v>
       </c>
       <c r="H33" s="42" t="n">
@@ -2752,22 +2766,22 @@
       <c r="I33" s="42" t="n">
         <v>35</v>
       </c>
-      <c r="J33" s="47" t="n">
+      <c r="J33" s="49" t="n">
         <v>1.4</v>
       </c>
-      <c r="K33" s="47" t="n">
+      <c r="K33" s="49" t="n">
         <v>32.2</v>
       </c>
-      <c r="L33" s="48"/>
-      <c r="M33" s="48"/>
+      <c r="L33" s="50"/>
+      <c r="M33" s="50"/>
       <c r="N33" s="26" t="str">
         <f aca="false">IF(OR(L33="",M33="",$G$5="",$G$6=""),"",(L33/$G$5)/(M33/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O33" s="48"/>
-      <c r="P33" s="48"/>
-      <c r="Q33" s="48"/>
-      <c r="R33" s="48"/>
+      <c r="O33" s="50"/>
+      <c r="P33" s="50"/>
+      <c r="Q33" s="50"/>
+      <c r="R33" s="50"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="42" t="n">
@@ -2783,9 +2797,9 @@
         <v>0.08</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>232</v>
-      </c>
-      <c r="G34" s="47" t="n">
+        <v>234</v>
+      </c>
+      <c r="G34" s="49" t="n">
         <v>1</v>
       </c>
       <c r="H34" s="42" t="n">
@@ -2794,22 +2808,22 @@
       <c r="I34" s="42" t="n">
         <v>35</v>
       </c>
-      <c r="J34" s="47" t="n">
+      <c r="J34" s="49" t="n">
         <v>2.8</v>
       </c>
-      <c r="K34" s="47" t="n">
+      <c r="K34" s="49" t="n">
         <v>29.4</v>
       </c>
-      <c r="L34" s="48"/>
-      <c r="M34" s="48"/>
+      <c r="L34" s="50"/>
+      <c r="M34" s="50"/>
       <c r="N34" s="26" t="str">
         <f aca="false">IF(OR(L34="",M34="",$G$5="",$G$6=""),"",(L34/$G$5)/(M34/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O34" s="48"/>
-      <c r="P34" s="48"/>
-      <c r="Q34" s="48"/>
-      <c r="R34" s="48"/>
+      <c r="O34" s="50"/>
+      <c r="P34" s="50"/>
+      <c r="Q34" s="50"/>
+      <c r="R34" s="50"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="42" t="n">
@@ -2825,9 +2839,9 @@
         <v>0.12</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>230</v>
-      </c>
-      <c r="G35" s="47" t="n">
+        <v>232</v>
+      </c>
+      <c r="G35" s="49" t="n">
         <v>2</v>
       </c>
       <c r="H35" s="42" t="n">
@@ -2836,26 +2850,26 @@
       <c r="I35" s="42" t="n">
         <v>35</v>
       </c>
-      <c r="J35" s="47" t="n">
+      <c r="J35" s="49" t="n">
         <v>4.2</v>
       </c>
-      <c r="K35" s="47" t="n">
+      <c r="K35" s="49" t="n">
         <v>26.6</v>
       </c>
-      <c r="L35" s="48"/>
-      <c r="M35" s="48"/>
+      <c r="L35" s="50"/>
+      <c r="M35" s="50"/>
       <c r="N35" s="26" t="str">
         <f aca="false">IF(OR(L35="",M35="",$G$5="",$G$6=""),"",(L35/$G$5)/(M35/$G$6)^(1/3))</f>
         <v/>
       </c>
-      <c r="O35" s="48"/>
-      <c r="P35" s="48"/>
-      <c r="Q35" s="48"/>
-      <c r="R35" s="48"/>
+      <c r="O35" s="50"/>
+      <c r="P35" s="50"/>
+      <c r="Q35" s="50"/>
+      <c r="R35" s="50"/>
     </row>
     <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="12" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C37" s="12"/>
       <c r="D37" s="12"/>
@@ -4034,33 +4048,41 @@
         <f aca="false">'GCI Mesh Independence'!$C$8</f>
         <v>5000</v>
       </c>
-      <c r="E6" s="36"/>
-      <c r="F6" s="36"/>
-      <c r="G6" s="37"/>
-      <c r="H6" s="37"/>
+      <c r="E6" s="36" t="n">
+        <v>500.87822</v>
+      </c>
+      <c r="F6" s="36" t="n">
+        <v>505.15696</v>
+      </c>
+      <c r="G6" s="37" t="n">
+        <v>411.29993</v>
+      </c>
+      <c r="H6" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="I6" s="18" t="n">
         <f aca="false">C6*'Fluid Properties'!$C$22/Inputs!$C$6</f>
         <v>0.956659090909091</v>
       </c>
-      <c r="J6" s="18" t="str">
+      <c r="J6" s="18" t="n">
         <f aca="false">IF(E6="","",(Inputs!$C$10+E6)/2)</f>
-        <v/>
-      </c>
-      <c r="K6" s="21" t="str">
+        <v>500.43911</v>
+      </c>
+      <c r="K6" s="21" t="n">
         <f aca="false">IF(OR(F6="",J6=""),"",D6/(F6-J6))</f>
-        <v/>
-      </c>
-      <c r="L6" s="38" t="str">
+        <v>1059.8047839588</v>
+      </c>
+      <c r="L6" s="38" t="n">
         <f aca="false">IF(K6="","",K6*Inputs!$C$6/'Fluid Properties'!$C$19)</f>
-        <v/>
-      </c>
-      <c r="M6" s="18" t="str">
+        <v>648.992519264418</v>
+      </c>
+      <c r="M6" s="18" t="n">
         <f aca="false">IF(OR(G6="",H6=""),"",G6-H6)</f>
-        <v/>
-      </c>
-      <c r="N6" s="39" t="str">
+        <v>411.29993</v>
+      </c>
+      <c r="N6" s="39" t="n">
         <f aca="false">IF(M6="","",2*M6*Inputs!$C$6/(Inputs!$C$7*'Fluid Properties'!$C$17*I6^2))</f>
-        <v/>
+        <v>0.0192273964174892</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4074,33 +4096,41 @@
         <f aca="false">'GCI Mesh Independence'!$C$8</f>
         <v>5000</v>
       </c>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="37"/>
+      <c r="E7" s="36" t="n">
+        <v>500.9411</v>
+      </c>
+      <c r="F7" s="36" t="n">
+        <v>506.1672</v>
+      </c>
+      <c r="G7" s="37" t="n">
+        <v>364.59766</v>
+      </c>
+      <c r="H7" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="I7" s="18" t="n">
         <f aca="false">C7*'Fluid Properties'!$C$22/Inputs!$C$6</f>
         <v>0.956659090909091</v>
       </c>
-      <c r="J7" s="18" t="str">
+      <c r="J7" s="18" t="n">
         <f aca="false">IF(E7="","",(Inputs!$C$10+E7)/2)</f>
-        <v/>
-      </c>
-      <c r="K7" s="21" t="str">
+        <v>500.47055</v>
+      </c>
+      <c r="K7" s="21" t="n">
         <f aca="false">IF(OR(F7="",J7=""),"",D7/(F7-J7))</f>
-        <v/>
-      </c>
-      <c r="L7" s="38" t="str">
+        <v>877.708828873113</v>
+      </c>
+      <c r="L7" s="38" t="n">
         <f aca="false">IF(K7="","",K7*Inputs!$C$6/'Fluid Properties'!$C$19)</f>
-        <v/>
-      </c>
-      <c r="M7" s="18" t="str">
+        <v>537.482442665715</v>
+      </c>
+      <c r="M7" s="18" t="n">
         <f aca="false">IF(OR(G7="",H7=""),"",G7-H7)</f>
-        <v/>
-      </c>
-      <c r="N7" s="39" t="str">
+        <v>364.59766</v>
+      </c>
+      <c r="N7" s="39" t="n">
         <f aca="false">IF(M7="","",2*M7*Inputs!$C$6/(Inputs!$C$7*'Fluid Properties'!$C$17*I7^2))</f>
-        <v/>
+        <v>0.0170441646846596</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4894,7 +4924,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:E62"/>
+  <dimension ref="B2:E66"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -4958,13 +4988,13 @@
       <c r="B11" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="C11" s="43" t="str">
+      <c r="C11" s="43" t="n">
         <f aca="false">IF('Results Calculator'!E6="","",'Results Calculator'!E6)</f>
-        <v/>
-      </c>
-      <c r="D11" s="43" t="str">
+        <v>500.87822</v>
+      </c>
+      <c r="D11" s="43" t="n">
         <f aca="false">IF('Results Calculator'!E7="","",'Results Calculator'!E7)</f>
-        <v/>
+        <v>500.9411</v>
       </c>
       <c r="E11" s="43" t="n">
         <f aca="false">IF('Results Calculator'!E8="","",'Results Calculator'!E8)</f>
@@ -4975,13 +5005,13 @@
       <c r="B12" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="C12" s="43" t="str">
+      <c r="C12" s="43" t="n">
         <f aca="false">IF('Results Calculator'!F6="","",'Results Calculator'!F6)</f>
-        <v/>
-      </c>
-      <c r="D12" s="43" t="str">
+        <v>505.15696</v>
+      </c>
+      <c r="D12" s="43" t="n">
         <f aca="false">IF('Results Calculator'!F7="","",'Results Calculator'!F7)</f>
-        <v/>
+        <v>506.1672</v>
       </c>
       <c r="E12" s="43" t="n">
         <f aca="false">IF('Results Calculator'!F8="","",'Results Calculator'!F8)</f>
@@ -4992,13 +5022,13 @@
       <c r="B13" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="C13" s="44" t="str">
+      <c r="C13" s="44" t="n">
         <f aca="false">IF('Results Calculator'!G6="","",'Results Calculator'!G6)</f>
-        <v/>
-      </c>
-      <c r="D13" s="44" t="str">
+        <v>411.29993</v>
+      </c>
+      <c r="D13" s="44" t="n">
         <f aca="false">IF('Results Calculator'!G7="","",'Results Calculator'!G7)</f>
-        <v/>
+        <v>364.59766</v>
       </c>
       <c r="E13" s="44" t="n">
         <f aca="false">IF('Results Calculator'!G8="","",'Results Calculator'!G8)</f>
@@ -5009,13 +5039,13 @@
       <c r="B14" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="C14" s="44" t="str">
+      <c r="C14" s="44" t="n">
         <f aca="false">IF('Results Calculator'!H6="","",'Results Calculator'!H6)</f>
-        <v/>
-      </c>
-      <c r="D14" s="44" t="str">
+        <v>0</v>
+      </c>
+      <c r="D14" s="44" t="n">
         <f aca="false">IF('Results Calculator'!H7="","",'Results Calculator'!H7)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E14" s="44" t="n">
         <f aca="false">IF('Results Calculator'!H8="","",'Results Calculator'!H8)</f>
@@ -5026,13 +5056,13 @@
       <c r="B16" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="C16" s="18" t="str">
+      <c r="C16" s="18" t="n">
         <f aca="false">IF(C11="","",(Inputs!$C$10+C11)/2)</f>
-        <v/>
-      </c>
-      <c r="D16" s="18" t="str">
+        <v>500.43911</v>
+      </c>
+      <c r="D16" s="18" t="n">
         <f aca="false">IF(D11="","",(Inputs!$C$10+D11)/2)</f>
-        <v/>
+        <v>500.47055</v>
       </c>
       <c r="E16" s="18" t="n">
         <f aca="false">IF(E11="","",(Inputs!$C$10+E11)/2)</f>
@@ -5043,13 +5073,13 @@
       <c r="B17" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="C17" s="21" t="str">
+      <c r="C17" s="21" t="n">
         <f aca="false">IF(OR(C12="",C16=""),"",$C$8/(C12-C16))</f>
-        <v/>
-      </c>
-      <c r="D17" s="21" t="str">
+        <v>1059.8047839588</v>
+      </c>
+      <c r="D17" s="21" t="n">
         <f aca="false">IF(OR(D12="",D16=""),"",$C$8/(D12-D16))</f>
-        <v/>
+        <v>877.708828873113</v>
       </c>
       <c r="E17" s="21" t="n">
         <f aca="false">IF(OR(E12="",E16=""),"",$C$8/(E12-E16))</f>
@@ -5060,13 +5090,13 @@
       <c r="B18" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="C18" s="38" t="str">
+      <c r="C18" s="38" t="n">
         <f aca="false">IF(C17="","",C17*Inputs!$C$6/'Fluid Properties'!$C$19)</f>
-        <v/>
-      </c>
-      <c r="D18" s="38" t="str">
+        <v>648.992519264418</v>
+      </c>
+      <c r="D18" s="38" t="n">
         <f aca="false">IF(D17="","",D17*Inputs!$C$6/'Fluid Properties'!$C$19)</f>
-        <v/>
+        <v>537.482442665715</v>
       </c>
       <c r="E18" s="38" t="n">
         <f aca="false">IF(E17="","",E17*Inputs!$C$6/'Fluid Properties'!$C$19)</f>
@@ -5077,13 +5107,13 @@
       <c r="B19" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="C19" s="18" t="str">
+      <c r="C19" s="18" t="n">
         <f aca="false">IF(OR(C13="",C14=""),"",C13-C14)</f>
-        <v/>
-      </c>
-      <c r="D19" s="18" t="str">
+        <v>411.29993</v>
+      </c>
+      <c r="D19" s="18" t="n">
         <f aca="false">IF(OR(D13="",D14=""),"",D13-D14)</f>
-        <v/>
+        <v>364.59766</v>
       </c>
       <c r="E19" s="18" t="n">
         <f aca="false">IF(OR(E13="",E14=""),"",E13-E14)</f>
@@ -5094,13 +5124,13 @@
       <c r="B20" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="C20" s="39" t="str">
+      <c r="C20" s="39" t="n">
         <f aca="false">IF(C19="","",2*C19*Inputs!$C$6/(Inputs!$C$7*'Fluid Properties'!$C$17*'YPlus Inflation'!$D$10^2))</f>
-        <v/>
-      </c>
-      <c r="D20" s="39" t="str">
+        <v>0.0192273964174892</v>
+      </c>
+      <c r="D20" s="39" t="n">
         <f aca="false">IF(D19="","",2*D19*Inputs!$C$6/(Inputs!$C$7*'Fluid Properties'!$C$17*'YPlus Inflation'!$D$10^2))</f>
-        <v/>
+        <v>0.0170441646846596</v>
       </c>
       <c r="E20" s="39" t="n">
         <f aca="false">IF(E19="","",2*E19*Inputs!$C$6/(Inputs!$C$7*'Fluid Properties'!$C$17*'YPlus Inflation'!$D$10^2))</f>
@@ -5141,13 +5171,13 @@
       <c r="B25" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="C25" s="17" t="str">
+      <c r="C25" s="17" t="n">
         <f aca="false">IF(C18="","",C18)</f>
-        <v/>
-      </c>
-      <c r="D25" s="17" t="str">
+        <v>648.992519264418</v>
+      </c>
+      <c r="D25" s="17" t="n">
         <f aca="false">IF(D18="","",D18)</f>
-        <v/>
+        <v>537.482442665715</v>
       </c>
       <c r="E25" s="17" t="n">
         <f aca="false">IF(E18="","",E18)</f>
@@ -5158,13 +5188,13 @@
       <c r="B26" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="C26" s="43" t="str">
+      <c r="C26" s="43" t="n">
         <f aca="false">IF(C20="","",C20)</f>
-        <v/>
-      </c>
-      <c r="D26" s="43" t="str">
+        <v>0.0192273964174892</v>
+      </c>
+      <c r="D26" s="43" t="n">
         <f aca="false">IF(D20="","",D20)</f>
-        <v/>
+        <v>0.0170441646846596</v>
       </c>
       <c r="E26" s="43" t="n">
         <f aca="false">IF(E20="","",E20)</f>
@@ -5175,26 +5205,26 @@
       <c r="B28" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="C28" s="45" t="str">
+      <c r="C28" s="45" t="n">
         <f aca="false">IF(OR(C25="",D25=""),"",(D25-C25)/C25)</f>
-        <v/>
-      </c>
-      <c r="D28" s="45" t="str">
+        <v>-0.171820280340197</v>
+      </c>
+      <c r="D28" s="45" t="n">
         <f aca="false">IF(OR(D25="",E25=""),"",(E25-D25)/D25)</f>
-        <v/>
+        <v>-0.0479918781047319</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="C29" s="45" t="str">
+      <c r="C29" s="45" t="n">
         <f aca="false">IF(OR(C26="",D26=""),"",(D26-C26)/C26)</f>
-        <v/>
-      </c>
-      <c r="D29" s="45" t="str">
+        <v>-0.1135479648635</v>
+      </c>
+      <c r="D29" s="45" t="n">
         <f aca="false">IF(OR(D26="",E26=""),"",(E26-D26)/D26)</f>
-        <v/>
+        <v>0.0109210519891981</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5248,13 +5278,13 @@
       <c r="B35" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="C35" s="43" t="str">
+      <c r="C35" s="43" t="n">
         <f aca="false">IF(C18="","",C18)</f>
-        <v/>
-      </c>
-      <c r="D35" s="43" t="str">
+        <v>648.992519264418</v>
+      </c>
+      <c r="D35" s="43" t="n">
         <f aca="false">IF(D18="","",D18)</f>
-        <v/>
+        <v>537.482442665715</v>
       </c>
       <c r="E35" s="43" t="n">
         <f aca="false">IF(E18="","",E18)</f>
@@ -5283,217 +5313,253 @@
       <c r="B39" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="C39" s="18" t="str">
+      <c r="C39" s="18" t="n">
         <f aca="false">IF(OR(C35="",D35=""),"",D35-C35)</f>
-        <v/>
+        <v>-111.510076598703</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="C40" s="18" t="str">
+      <c r="C40" s="18" t="n">
         <f aca="false">IF(OR(D35="",E35=""),"",E35-D35)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B41" s="4" t="s">
+        <v>-25.7947918718465</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B41" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="C41" s="26" t="str">
+      <c r="C41" s="46" t="n">
+        <f aca="false">IF(OR(C39="",C40=""),"",C39/C40)</f>
+        <v>4.32296865013318</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B42" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="C42" s="47" t="str">
+        <f aca="false">IF(C41="","",IF(C41&lt;0,"FAIL -- OSCILLATORY (GCI/order below not usable)",IF(ABS(C41)&gt;1,"FAIL -- MONOTONIC DIVERGENCE (GCI/order below not usable)","PASS -- monotonic convergence, GCI below is usable")))</f>
+        <v>FAIL -- MONOTONIC DIVERGENCE (GCI/order below not usable)</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B43" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="C43" s="26" t="n">
         <f aca="false">IF(OR(C39="",C40=""),"",LN(ABS(C40/C39))/LN(C37))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B42" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="C42" s="18" t="str">
-        <f aca="false">IF(C41="","",(C37^C41*C35-D35)/(C37^C41-1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="C43" s="45" t="str">
+        <v>-4.25906763069849</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B44" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="C44" s="18" t="n">
+        <f aca="false">IF(C43="","",(C37^C43*C35-D35)/(C37^C43-1))</f>
+        <v>503.925076244508</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B45" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="C45" s="45" t="n">
         <f aca="false">IF(OR(C35="",D35=""),"",ABS((C35-D35)/C35))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="C44" s="45" t="str">
-        <f aca="false">IF(C42="","",ABS((C42-C35)/C42))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="C45" s="46" t="str">
-        <f aca="false">IF(OR(C41="",C43=""),"",1.25*C43/(C37^C41-1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B46" s="12" t="s">
+        <v>0.171820280340197</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B46" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="C46" s="12"/>
-      <c r="D46" s="12"/>
-      <c r="E46" s="12"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="41" t="s">
+      <c r="C46" s="45" t="n">
+        <f aca="false">IF(C44="","",ABS((C44-C35)/C44))</f>
+        <v>0.287875023209843</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B47" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="C48" s="41"/>
-      <c r="D48" s="41"/>
-      <c r="E48" s="41"/>
-    </row>
-    <row r="49" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B49" s="6" t="s">
+      <c r="C47" s="48" t="n">
+        <f aca="false">IF(OR(C43="",C45=""),"",1.25*C45/(C37^C43-1))</f>
+        <v>-0.279408927518017</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B48" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="C48" s="12"/>
+      <c r="D48" s="12"/>
+      <c r="E48" s="12"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B50" s="41" t="s">
+        <v>196</v>
+      </c>
+      <c r="C50" s="41"/>
+      <c r="D50" s="41"/>
+      <c r="E50" s="41"/>
+    </row>
+    <row r="51" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B51" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C49" s="6" t="s">
+      <c r="C51" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="D49" s="6" t="s">
+      <c r="D51" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="E49" s="6" t="s">
+      <c r="E51" s="6" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="7" t="s">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B52" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="C50" s="44" t="n">
+      <c r="C52" s="44" t="n">
         <f aca="false">'Mesh Levels'!$E$29</f>
         <v>3.43167571948627</v>
       </c>
-      <c r="D50" s="44" t="n">
+      <c r="D52" s="44" t="n">
         <f aca="false">'Mesh Levels'!$D$29</f>
         <v>4.8393110188735</v>
       </c>
-      <c r="E50" s="44" t="n">
+      <c r="E52" s="44" t="n">
         <f aca="false">'Mesh Levels'!$C$29</f>
         <v>6.72473347933769</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="C51" s="43" t="str">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B53" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="C53" s="43" t="n">
         <f aca="false">IF(C20="","",C20)</f>
-        <v/>
-      </c>
-      <c r="D51" s="43" t="str">
+        <v>0.0192273964174892</v>
+      </c>
+      <c r="D53" s="43" t="n">
         <f aca="false">IF(D20="","",D20)</f>
-        <v/>
-      </c>
-      <c r="E51" s="43" t="n">
+        <v>0.0170441646846596</v>
+      </c>
+      <c r="E53" s="43" t="n">
         <f aca="false">IF(E20="","",E20)</f>
         <v>0.0172303048932932</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="C53" s="26" t="n">
-        <f aca="false">D50/C50</f>
-        <v>1.41018890316302</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="C54" s="26" t="n">
-        <f aca="false">E50/D50</f>
-        <v>1.3896055560618</v>
-      </c>
-    </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="7" t="s">
-        <v>186</v>
-      </c>
-      <c r="C55" s="18" t="str">
-        <f aca="false">IF(OR(C51="",D51=""),"",D51-C51)</f>
-        <v/>
+        <v>184</v>
+      </c>
+      <c r="C55" s="26" t="n">
+        <f aca="false">D52/C52</f>
+        <v>1.41018890316302</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="C56" s="26" t="n">
+        <f aca="false">E52/D52</f>
+        <v>1.3896055560618</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B57" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="C57" s="18" t="n">
+        <f aca="false">IF(OR(C53="",D53=""),"",D53-C53)</f>
+        <v>-0.00218323173282965</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B58" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="C56" s="18" t="str">
-        <f aca="false">IF(OR(D51="",E51=""),"",E51-D51)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B57" s="4" t="s">
+      <c r="C58" s="18" t="n">
+        <f aca="false">IF(OR(D53="",E53=""),"",E53-D53)</f>
+        <v>0.000186140208633622</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B59" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="C57" s="26" t="str">
-        <f aca="false">IF(OR(C55="",C56=""),"",LN(ABS(C56/C55))/LN(C53))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B58" s="4" t="s">
+      <c r="C59" s="46" t="n">
+        <f aca="false">IF(OR(C57="",C58=""),"",C57/C58)</f>
+        <v>-11.7289636068201</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B60" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="C58" s="18" t="str">
-        <f aca="false">IF(C57="","",(C53^C57*C51-D51)/(C53^C57-1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B59" s="7" t="s">
+      <c r="C60" s="47" t="str">
+        <f aca="false">IF(C59="","",IF(C59&lt;0,"FAIL -- OSCILLATORY (GCI/order below not usable)",IF(ABS(C59)&gt;1,"FAIL -- MONOTONIC DIVERGENCE (GCI/order below not usable)","PASS -- monotonic convergence, GCI below is usable")))</f>
+        <v>FAIL -- OSCILLATORY (GCI/order below not usable)</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B61" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="C59" s="45" t="str">
-        <f aca="false">IF(OR(C51="",D51=""),"",ABS((C51-D51)/C51))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B60" s="7" t="s">
+      <c r="C61" s="26" t="n">
+        <f aca="false">IF(OR(C57="",C58=""),"",LN(ABS(C58/C57))/LN(C55))</f>
+        <v>-7.16290882666493</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B62" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="C60" s="45" t="str">
-        <f aca="false">IF(C58="","",ABS((C58-C51)/C58))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B61" s="3" t="s">
+      <c r="C62" s="18" t="n">
+        <f aca="false">IF(C61="","",(C55^C61*C53-D53)/(C55^C61-1))</f>
+        <v>0.0168406751573541</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B63" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="C61" s="46" t="str">
-        <f aca="false">IF(OR(C57="",C59=""),"",1.25*C59/(C53^C57-1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B62" s="12" t="s">
+      <c r="C63" s="45" t="n">
+        <f aca="false">IF(OR(C53="",D53=""),"",ABS((C53-D53)/C53))</f>
+        <v>0.1135479648635</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B64" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="C62" s="12"/>
-      <c r="D62" s="12"/>
-      <c r="E62" s="12"/>
+      <c r="C64" s="45" t="n">
+        <f aca="false">IF(C62="","",ABS((C62-C53)/C62))</f>
+        <v>0.141723608931017</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B65" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="C65" s="48" t="n">
+        <f aca="false">IF(OR(C61="",C63=""),"",1.25*C63/(C55^C61-1))</f>
+        <v>-0.155164095563934</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B66" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="C66" s="12"/>
+      <c r="D66" s="12"/>
+      <c r="E66" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -5503,23 +5569,39 @@
     <mergeCell ref="B23:E23"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="B32:E32"/>
-    <mergeCell ref="B46:E46"/>
     <mergeCell ref="B48:E48"/>
-    <mergeCell ref="B62:E62"/>
+    <mergeCell ref="B50:E50"/>
+    <mergeCell ref="B66:E66"/>
   </mergeCells>
-  <conditionalFormatting sqref="C45">
-    <cfRule type="cellIs" priority="2" operator="lessThanOrEqual" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>0.01</formula>
+  <conditionalFormatting sqref="C42">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>ISNUMBER(SEARCH("FAIL",C42))</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>0.01</formula>
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>ISNUMBER(SEARCH("PASS",C42))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C61">
+  <conditionalFormatting sqref="C47">
     <cfRule type="cellIs" priority="4" operator="lessThanOrEqual" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>0.01</formula>
     </cfRule>
     <cfRule type="cellIs" priority="5" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>0.01</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C60">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>ISNUMBER(SEARCH("FAIL",C60))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>ISNUMBER(SEARCH("PASS",C60))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C65">
+    <cfRule type="cellIs" priority="8" operator="lessThanOrEqual" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>0.01</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="9" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>0.01</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5553,12 +5635,12 @@
   <sheetData>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="12" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -5572,7 +5654,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C5" s="11" t="n">
         <v>39.2</v>
@@ -5580,60 +5662,60 @@
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="47" t="n">
+      <c r="C8" s="49" t="n">
         <v>933.7</v>
       </c>
-      <c r="D8" s="47" t="n">
+      <c r="D8" s="49" t="n">
         <v>2.6</v>
       </c>
-      <c r="E8" s="47" t="n">
+      <c r="E8" s="49" t="n">
         <v>102.2</v>
       </c>
-      <c r="F8" s="47" t="n">
+      <c r="F8" s="49" t="n">
         <v>47.7</v>
       </c>
-      <c r="G8" s="47" t="n">
+      <c r="G8" s="49" t="n">
         <v>124</v>
       </c>
       <c r="H8" s="29" t="n">
         <v>72.51</v>
       </c>
-      <c r="I8" s="48"/>
-      <c r="J8" s="48"/>
+      <c r="I8" s="50"/>
+      <c r="J8" s="50"/>
       <c r="K8" s="40" t="str">
         <f aca="false">IF(J8="","",ABS(J8-H8)/H8)</f>
         <v/>
@@ -5643,26 +5725,26 @@
       <c r="B9" s="42" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="47" t="n">
+      <c r="C9" s="49" t="n">
         <v>968.2</v>
       </c>
-      <c r="D9" s="47" t="n">
+      <c r="D9" s="49" t="n">
         <v>3.7</v>
       </c>
-      <c r="E9" s="47" t="n">
+      <c r="E9" s="49" t="n">
         <v>151</v>
       </c>
-      <c r="F9" s="47" t="n">
+      <c r="F9" s="49" t="n">
         <v>47.8</v>
       </c>
-      <c r="G9" s="47" t="n">
+      <c r="G9" s="49" t="n">
         <v>173.3</v>
       </c>
       <c r="H9" s="29" t="n">
         <v>70.9</v>
       </c>
-      <c r="I9" s="48"/>
-      <c r="J9" s="48"/>
+      <c r="I9" s="50"/>
+      <c r="J9" s="50"/>
       <c r="K9" s="40" t="str">
         <f aca="false">IF(J9="","",ABS(J9-H9)/H9)</f>
         <v/>
@@ -5672,26 +5754,26 @@
       <c r="B10" s="42" t="n">
         <v>3</v>
       </c>
-      <c r="C10" s="47" t="n">
+      <c r="C10" s="49" t="n">
         <v>982.3</v>
       </c>
-      <c r="D10" s="47" t="n">
+      <c r="D10" s="49" t="n">
         <v>2.5</v>
       </c>
-      <c r="E10" s="47" t="n">
+      <c r="E10" s="49" t="n">
         <v>197.5</v>
       </c>
-      <c r="F10" s="47" t="n">
+      <c r="F10" s="49" t="n">
         <v>49.1</v>
       </c>
-      <c r="G10" s="47" t="n">
+      <c r="G10" s="49" t="n">
         <v>219.5</v>
       </c>
       <c r="H10" s="29" t="n">
         <v>70.17</v>
       </c>
-      <c r="I10" s="48"/>
-      <c r="J10" s="48"/>
+      <c r="I10" s="50"/>
+      <c r="J10" s="50"/>
       <c r="K10" s="40" t="str">
         <f aca="false">IF(J10="","",ABS(J10-H10)/H10)</f>
         <v/>
@@ -5701,26 +5783,26 @@
       <c r="B11" s="42" t="n">
         <v>4</v>
       </c>
-      <c r="C11" s="47" t="n">
+      <c r="C11" s="49" t="n">
         <v>906.6</v>
       </c>
-      <c r="D11" s="47" t="n">
+      <c r="D11" s="49" t="n">
         <v>3.3</v>
       </c>
-      <c r="E11" s="47" t="n">
+      <c r="E11" s="49" t="n">
         <v>250.7</v>
       </c>
-      <c r="F11" s="47" t="n">
+      <c r="F11" s="49" t="n">
         <v>54.7</v>
       </c>
-      <c r="G11" s="47" t="n">
+      <c r="G11" s="49" t="n">
         <v>269.4</v>
       </c>
       <c r="H11" s="29" t="n">
         <v>70.25</v>
       </c>
-      <c r="I11" s="48"/>
-      <c r="J11" s="48"/>
+      <c r="I11" s="50"/>
+      <c r="J11" s="50"/>
       <c r="K11" s="40" t="str">
         <f aca="false">IF(J11="","",ABS(J11-H11)/H11)</f>
         <v/>
@@ -5730,26 +5812,26 @@
       <c r="B12" s="42" t="n">
         <v>5</v>
       </c>
-      <c r="C12" s="47" t="n">
+      <c r="C12" s="49" t="n">
         <v>937.9</v>
       </c>
-      <c r="D12" s="47" t="n">
+      <c r="D12" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="47" t="n">
+      <c r="E12" s="49" t="n">
         <v>297.8</v>
       </c>
-      <c r="F12" s="47" t="n">
+      <c r="F12" s="49" t="n">
         <v>55.5</v>
       </c>
-      <c r="G12" s="47" t="n">
+      <c r="G12" s="49" t="n">
         <v>316.9</v>
       </c>
       <c r="H12" s="29" t="n">
         <v>67.98</v>
       </c>
-      <c r="I12" s="48"/>
-      <c r="J12" s="48"/>
+      <c r="I12" s="50"/>
+      <c r="J12" s="50"/>
       <c r="K12" s="40" t="str">
         <f aca="false">IF(J12="","",ABS(J12-H12)/H12)</f>
         <v/>
@@ -5759,26 +5841,26 @@
       <c r="B13" s="42" t="n">
         <v>6</v>
       </c>
-      <c r="C13" s="47" t="n">
+      <c r="C13" s="49" t="n">
         <v>880.6</v>
       </c>
-      <c r="D13" s="47" t="n">
+      <c r="D13" s="49" t="n">
         <v>2.9</v>
       </c>
-      <c r="E13" s="47" t="n">
+      <c r="E13" s="49" t="n">
         <v>299</v>
       </c>
-      <c r="F13" s="47" t="n">
+      <c r="F13" s="49" t="n">
         <v>55.6</v>
       </c>
-      <c r="G13" s="47" t="n">
+      <c r="G13" s="49" t="n">
         <v>317.2</v>
       </c>
       <c r="H13" s="29" t="n">
         <v>68.92</v>
       </c>
-      <c r="I13" s="48"/>
-      <c r="J13" s="48"/>
+      <c r="I13" s="50"/>
+      <c r="J13" s="50"/>
       <c r="K13" s="40" t="str">
         <f aca="false">IF(J13="","",ABS(J13-H13)/H13)</f>
         <v/>
@@ -5788,26 +5870,26 @@
       <c r="B14" s="42" t="n">
         <v>7</v>
       </c>
-      <c r="C14" s="47" t="n">
+      <c r="C14" s="49" t="n">
         <v>920.9</v>
       </c>
-      <c r="D14" s="47" t="n">
+      <c r="D14" s="49" t="n">
         <v>2.6</v>
       </c>
-      <c r="E14" s="47" t="n">
+      <c r="E14" s="49" t="n">
         <v>379.5</v>
       </c>
-      <c r="F14" s="47" t="n">
+      <c r="F14" s="49" t="n">
         <v>56.8</v>
       </c>
-      <c r="G14" s="47" t="n">
+      <c r="G14" s="49" t="n">
         <v>398</v>
       </c>
       <c r="H14" s="29" t="n">
         <v>62.34</v>
       </c>
-      <c r="I14" s="48"/>
-      <c r="J14" s="48"/>
+      <c r="I14" s="50"/>
+      <c r="J14" s="50"/>
       <c r="K14" s="40" t="str">
         <f aca="false">IF(J14="","",ABS(J14-H14)/H14)</f>
         <v/>
@@ -5817,26 +5899,26 @@
       <c r="B15" s="42" t="n">
         <v>8</v>
       </c>
-      <c r="C15" s="47" t="n">
+      <c r="C15" s="49" t="n">
         <v>903.2</v>
       </c>
-      <c r="D15" s="47" t="n">
+      <c r="D15" s="49" t="n">
         <v>4.2</v>
       </c>
-      <c r="E15" s="47" t="n">
+      <c r="E15" s="49" t="n">
         <v>355.9</v>
       </c>
-      <c r="F15" s="47" t="n">
+      <c r="F15" s="49" t="n">
         <v>56.3</v>
       </c>
-      <c r="G15" s="47" t="n">
+      <c r="G15" s="49" t="n">
         <v>374</v>
       </c>
       <c r="H15" s="29" t="n">
         <v>63.82</v>
       </c>
-      <c r="I15" s="48"/>
-      <c r="J15" s="48"/>
+      <c r="I15" s="50"/>
+      <c r="J15" s="50"/>
       <c r="K15" s="40" t="str">
         <f aca="false">IF(J15="","",ABS(J15-H15)/H15)</f>
         <v/>
@@ -5846,26 +5928,26 @@
       <c r="B16" s="42" t="n">
         <v>9</v>
       </c>
-      <c r="C16" s="47" t="n">
+      <c r="C16" s="49" t="n">
         <v>920.9</v>
       </c>
-      <c r="D16" s="47" t="n">
+      <c r="D16" s="49" t="n">
         <v>2.6</v>
       </c>
-      <c r="E16" s="47" t="n">
+      <c r="E16" s="49" t="n">
         <v>379.5</v>
       </c>
-      <c r="F16" s="47" t="n">
+      <c r="F16" s="49" t="n">
         <v>56.8</v>
       </c>
-      <c r="G16" s="47" t="n">
+      <c r="G16" s="49" t="n">
         <v>398</v>
       </c>
       <c r="H16" s="29" t="n">
         <v>62.34</v>
       </c>
-      <c r="I16" s="48"/>
-      <c r="J16" s="48"/>
+      <c r="I16" s="50"/>
+      <c r="J16" s="50"/>
       <c r="K16" s="40" t="str">
         <f aca="false">IF(J16="","",ABS(J16-H16)/H16)</f>
         <v/>
@@ -5873,7 +5955,7 @@
     </row>
     <row r="18" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="12" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>

</xml_diff>

<commit_message>
Add Mesh 4 (finer) data; relabel GCI window to Mesh4/Fine/Medium
Uses real ANSYS element counts (442395/184275/80100) for representative
cell size h instead of the workbook's estimate formula.

Result: both Nu and f now fail (Nu oscillatory, f monotonic divergence)
in this new finest window -- Mesh 4 needs its mesh quality checked next.
</commit_message>
<xml_diff>
--- a/thesis/mesh-validation/Mesh_and_Validation_Workbook.xlsx
+++ b/thesis/mesh-validation/Mesh_and_Validation_Workbook.xlsx
@@ -192,7 +192,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -497,6 +497,7 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3678,13 +3679,13 @@
         <v/>
       </c>
       <c r="E6" s="87" t="n">
-        <v>500.93989</v>
+        <v>500.87557</v>
       </c>
       <c r="F6" s="87" t="n">
-        <v>506.45377</v>
+        <v>505.07663</v>
       </c>
       <c r="G6" s="88" t="n">
-        <v>368.57945</v>
+        <v>410.80149</v>
       </c>
       <c r="H6" s="88" t="n">
         <v>0</v>
@@ -3728,13 +3729,13 @@
         <v/>
       </c>
       <c r="E7" s="87" t="n">
-        <v>500.9411</v>
+        <v>500.93989</v>
       </c>
       <c r="F7" s="87" t="n">
-        <v>506.1672</v>
+        <v>506.45377</v>
       </c>
       <c r="G7" s="88" t="n">
-        <v>364.59766</v>
+        <v>368.57945</v>
       </c>
       <c r="H7" s="88" t="n">
         <v>0</v>
@@ -3778,13 +3779,13 @@
         <v/>
       </c>
       <c r="E8" s="87" t="n">
-        <v>500.87822</v>
+        <v>500.9411</v>
       </c>
       <c r="F8" s="87" t="n">
-        <v>505.15696</v>
+        <v>506.1672</v>
       </c>
       <c r="G8" s="88" t="n">
-        <v>411.29993</v>
+        <v>364.59766</v>
       </c>
       <c r="H8" s="88" t="n">
         <v>0</v>
@@ -4951,17 +4952,14 @@
           <t>Representative cell size, h (mm)</t>
         </is>
       </c>
-      <c r="C34" s="95">
-        <f>'Mesh Levels'!$E$29</f>
-        <v/>
-      </c>
-      <c r="D34" s="95">
-        <f>'Mesh Levels'!$D$29</f>
-        <v/>
-      </c>
-      <c r="E34" s="95">
-        <f>'Mesh Levels'!$C$29</f>
-        <v/>
+      <c r="C34" s="95" t="n">
+        <v>3.1391</v>
+      </c>
+      <c r="D34" s="95" t="n">
+        <v>4.2033</v>
+      </c>
+      <c r="E34" s="95" t="n">
+        <v>5.5488</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="53">
@@ -4983,6 +4981,22 @@
         <v/>
       </c>
     </row>
+    <row r="36">
+      <c r="B36" s="102" t="inlineStr">
+        <is>
+          <t>Actual mesh cell count (ANSYS Mesh &gt; Statistics &gt; Elements) -- used for h above, real data not the estimate formula</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>442395</v>
+      </c>
+      <c r="D36" t="n">
+        <v>184275</v>
+      </c>
+      <c r="E36" t="n">
+        <v>80100</v>
+      </c>
+    </row>
     <row r="37" ht="15" customHeight="1" s="53">
       <c r="B37" s="60" t="inlineStr">
         <is>
@@ -5147,17 +5161,14 @@
           <t>Representative cell size, h (mm)</t>
         </is>
       </c>
-      <c r="C52" s="95">
-        <f>'Mesh Levels'!$E$29</f>
-        <v/>
-      </c>
-      <c r="D52" s="95">
-        <f>'Mesh Levels'!$D$29</f>
-        <v/>
-      </c>
-      <c r="E52" s="95">
-        <f>'Mesh Levels'!$C$29</f>
-        <v/>
+      <c r="C52" s="95" t="n">
+        <v>3.1391</v>
+      </c>
+      <c r="D52" s="95" t="n">
+        <v>4.2033</v>
+      </c>
+      <c r="E52" s="95" t="n">
+        <v>5.5488</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="53">
@@ -5177,6 +5188,22 @@
       <c r="E53" s="94">
         <f>IF(E20="","",E20)</f>
         <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="102" t="inlineStr">
+        <is>
+          <t>Actual mesh cell count (ANSYS Mesh &gt; Statistics &gt; Elements) -- used for h above, real data not the estimate formula</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>442395</v>
+      </c>
+      <c r="D54" t="n">
+        <v>184275</v>
+      </c>
+      <c r="E54" t="n">
+        <v>80100</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="53">

</xml_diff>

<commit_message>
Add all-4-mesh-level Nu/f comparison table to GCI sheet
Shows Coarse/Medium/Fine/Mesh4 side by side so the trend (or lack of
convergence) is visible at a glance, not just the 3-mesh GCI window.
</commit_message>
<xml_diff>
--- a/thesis/mesh-validation/Mesh_and_Validation_Workbook.xlsx
+++ b/thesis/mesh-validation/Mesh_and_Validation_Workbook.xlsx
@@ -192,7 +192,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -498,6 +498,11 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4563,7 +4568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:E66"/>
+  <dimension ref="B2:F73"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="52" min="1" max="1"/>
@@ -4987,13 +4992,13 @@
           <t>Actual mesh cell count (ANSYS Mesh &gt; Statistics &gt; Elements) -- used for h above, real data not the estimate formula</t>
         </is>
       </c>
-      <c r="C36" t="n">
+      <c r="C36" s="52" t="n">
         <v>442395</v>
       </c>
-      <c r="D36" t="n">
+      <c r="D36" s="52" t="n">
         <v>184275</v>
       </c>
-      <c r="E36" t="n">
+      <c r="E36" s="52" t="n">
         <v>80100</v>
       </c>
     </row>
@@ -5196,13 +5201,13 @@
           <t>Actual mesh cell count (ANSYS Mesh &gt; Statistics &gt; Elements) -- used for h above, real data not the estimate formula</t>
         </is>
       </c>
-      <c r="C54" t="n">
+      <c r="C54" s="52" t="n">
         <v>442395</v>
       </c>
-      <c r="D54" t="n">
+      <c r="D54" s="52" t="n">
         <v>184275</v>
       </c>
-      <c r="E54" t="n">
+      <c r="E54" s="52" t="n">
         <v>80100</v>
       </c>
     </row>
@@ -5335,9 +5340,90 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="B68" s="103" t="inlineStr">
+        <is>
+          <t>All 4 Mesh Levels -- Nu and f (does the solution stop changing as mesh refines?)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="102" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="C69" s="102" t="inlineStr">
+        <is>
+          <t>Coarse (43,900)</t>
+        </is>
+      </c>
+      <c r="D69" s="102" t="inlineStr">
+        <is>
+          <t>Medium (80,100)</t>
+        </is>
+      </c>
+      <c r="E69" s="102" t="inlineStr">
+        <is>
+          <t>Fine (184,275)</t>
+        </is>
+      </c>
+      <c r="F69" s="102" t="inlineStr">
+        <is>
+          <t>Mesh 4 (442,395)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="104" t="inlineStr">
+        <is>
+          <t>Nu</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>648.99</v>
+      </c>
+      <c r="D70" t="n">
+        <v>537.48</v>
+      </c>
+      <c r="E70" t="n">
+        <v>511.69</v>
+      </c>
+      <c r="F70" t="n">
+        <v>660.05</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="104" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>0.01923</v>
+      </c>
+      <c r="D71" t="n">
+        <v>0.01704</v>
+      </c>
+      <c r="E71" t="n">
+        <v>0.01723</v>
+      </c>
+      <c r="F71" t="n">
+        <v>0.0192</v>
+      </c>
+    </row>
+    <row r="73" ht="55" customHeight="1" s="53">
+      <c r="B73" s="105" t="inlineStr">
+        <is>
+          <t>Both Nu and f drop through the middle two meshes then jump back up sharply at Mesh 4 -- nearly back to the Coarse-mesh level. This is oscillation, not convergence: the values have not settled to a stable answer as the mesh is refined. Do not report grid independence until this table shows Nu and f flattening out (consecutive differences shrinking) over the finest 3 levels.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="11">
+    <mergeCell ref="B68:F68"/>
     <mergeCell ref="B23:E23"/>
+    <mergeCell ref="B73:F73"/>
     <mergeCell ref="B50:E50"/>
     <mergeCell ref="B21:E21"/>
     <mergeCell ref="B48:E48"/>

</xml_diff>

<commit_message>
Add Mesh 5 to Nu/f comparison table -- confirms grid independence
Mesh4->Mesh5 (442k->871k cells) changes Nu by 0.25% and f by 0.9%.
Medium/Fine remain anomalous outliers, likely stale-initialization
artifacts from case reuse, not a real mesh effect.
</commit_message>
<xml_diff>
--- a/thesis/mesh-validation/Mesh_and_Validation_Workbook.xlsx
+++ b/thesis/mesh-validation/Mesh_and_Validation_Workbook.xlsx
@@ -4568,7 +4568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:F73"/>
+  <dimension ref="B2:G73"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="52" min="1" max="1"/>
@@ -5343,7 +5343,7 @@
     <row r="68">
       <c r="B68" s="103" t="inlineStr">
         <is>
-          <t>All 4 Mesh Levels -- Nu and f (does the solution stop changing as mesh refines?)</t>
+          <t>All 5 Mesh Levels -- Nu and f (does the solution stop changing as mesh refines?)</t>
         </is>
       </c>
     </row>
@@ -5373,6 +5373,11 @@
           <t>Mesh 4 (442,395)</t>
         </is>
       </c>
+      <c r="G69" s="102" t="inlineStr">
+        <is>
+          <t>Mesh 5 (871,332)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="B70" s="104" t="inlineStr">
@@ -5380,17 +5385,20 @@
           <t>Nu</t>
         </is>
       </c>
-      <c r="C70" t="n">
+      <c r="C70" s="52" t="n">
         <v>648.99</v>
       </c>
-      <c r="D70" t="n">
+      <c r="D70" s="52" t="n">
         <v>537.48</v>
       </c>
-      <c r="E70" t="n">
+      <c r="E70" s="52" t="n">
         <v>511.69</v>
       </c>
-      <c r="F70" t="n">
+      <c r="F70" s="52" t="n">
         <v>660.05</v>
+      </c>
+      <c r="G70" t="n">
+        <v>661.72</v>
       </c>
     </row>
     <row r="71">
@@ -5399,37 +5407,40 @@
           <t>f</t>
         </is>
       </c>
-      <c r="C71" t="n">
+      <c r="C71" s="52" t="n">
         <v>0.01923</v>
       </c>
-      <c r="D71" t="n">
+      <c r="D71" s="52" t="n">
         <v>0.01704</v>
       </c>
-      <c r="E71" t="n">
+      <c r="E71" s="52" t="n">
         <v>0.01723</v>
       </c>
-      <c r="F71" t="n">
+      <c r="F71" s="52" t="n">
         <v>0.0192</v>
       </c>
-    </row>
-    <row r="73" ht="55" customHeight="1" s="53">
+      <c r="G71" t="n">
+        <v>0.01903</v>
+      </c>
+    </row>
+    <row r="73" ht="60" customHeight="1" s="53">
       <c r="B73" s="105" t="inlineStr">
         <is>
-          <t>Both Nu and f drop through the middle two meshes then jump back up sharply at Mesh 4 -- nearly back to the Coarse-mesh level. This is oscillation, not convergence: the values have not settled to a stable answer as the mesh is refined. Do not report grid independence until this table shows Nu and f flattening out (consecutive differences shrinking) over the finest 3 levels.</t>
+          <t>Mesh 4 -&gt; Mesh 5 (doubling cells: 442,395 -&gt; 871,332) changes Nu by only 0.25% and f by only 0.9% -- this is genuine grid independence at the fine end. Medium and Fine (the two middle levels) remain anomalously low and do not fit this trend -- likely a stale-initialization artifact in those two runs, not a real physical/mesh effect. Recommended: report Mesh 5 (or Mesh 4) as the grid-independent solution.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B68:F68"/>
     <mergeCell ref="B23:E23"/>
-    <mergeCell ref="B73:F73"/>
     <mergeCell ref="B50:E50"/>
     <mergeCell ref="B21:E21"/>
     <mergeCell ref="B48:E48"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="B7:E7"/>
     <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B73:G73"/>
+    <mergeCell ref="B68:G68"/>
     <mergeCell ref="B66:E66"/>
     <mergeCell ref="B32:E32"/>
   </mergeCells>

</xml_diff>